<commit_message>
fix(pr30): set page margins to match Tenzor reference, align sheet heights
Эталон Тензора Романова имеет page margins: top=0.55" (40pt), bottom=1.69"
(122pt), L/R=0.625" (45pt). Bottom margin 122pt — это зона под overlay-штамп
ЭДО Тензора. У нас же были стандартные 0.196" (14pt) — лист прижимался к
краям A4, метки распознавания смещались.

v7 алгоритм:
1. Обрезает мёртвые хвосты строк (как v4)
2. Сохраняет угловые метки (TL/I в row 1, BL/BR в last_marker_row)
3. Выравнивает все 4 листа на одинаковую высоту 837pt (одна deficit-row)
4. Устанавливает page margins как у эталона:
   - top = 0.55" (40pt)
   - bottom = 1.69" (122pt) — зона для overlay штампа
   - left/right = 0.625" (45pt)
5. Ширины столбцов НЕ ТРОГАЕТ — координаты filler работают как прежде

Локальный тест soffice показал что метки теперь лежат на:
  TL=(45, 51), BL=(713, 51), BR=(713, 481)
По сравнению с эталоном:
  TL=(40, 45), BL=(720, 43), BR=(720, 546)
Расхождение по вертикали ~1%, что значительно лучше предыдущих 30%.
</commit_message>
<xml_diff>
--- a/modules/usn_declaration/data/declaration_template_2024.xlsx
+++ b/modules/usn_declaration/data/declaration_template_2024.xlsx
@@ -917,6 +917,9 @@
     <xf numFmtId="49" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" indent="3"/>
     </xf>
@@ -931,9 +934,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" indent="4"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -4229,8 +4229,191 @@
         </is>
       </c>
     </row>
-    <row r="61" ht="9" customHeight="1" s="127"/>
-    <row r="62" ht="75" customHeight="1" s="127"/>
+    <row r="61" ht="0.5" customHeight="1" s="127"/>
+    <row r="62" ht="13.5" customHeight="1" s="127">
+      <c r="A62" s="128" t="n"/>
+      <c r="B62" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="C62" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="D62" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="E62" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="F62" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="G62" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="H62" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="I62" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="J62" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="K62" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="L62" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="M62" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="N62" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="O62" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="P62" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="Q62" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="R62" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="S62" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="T62" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="U62" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="V62" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="W62" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="X62" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="Y62" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="Z62" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="AA62" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="AB62" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="AC62" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="AD62" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="AE62" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="AF62" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="AG62" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="AH62" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="AI62" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="AJ62" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="AK62" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="AN62" s="128" t="n"/>
+    </row>
     <row r="63" ht="17.25" customHeight="1" s="127"/>
     <row r="64" ht="17.25" customHeight="1" s="127"/>
     <row r="65" ht="17.25" customHeight="1" s="127"/>
@@ -4291,7 +4474,7 @@
     <mergeCell ref="R1:R2"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.196527777777778" right="0.196527777777778" top="0.196527777777778" bottom="0.196527777777778" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageMargins left="0.625" right="0.625" top="0.55" bottom="1.69" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" cellComments="atEnd" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
@@ -11450,8 +11633,19 @@
       <c r="AM51" s="134" t="n"/>
       <c r="AN51" s="134" t="n"/>
     </row>
-    <row r="52" ht="9" customHeight="1" s="127"/>
-    <row r="53" ht="75" customHeight="1" s="127"/>
+    <row r="52" ht="0.5" customHeight="1" s="127"/>
+    <row r="53" ht="13.5" customHeight="1" s="127">
+      <c r="A53" s="128" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="AN53" s="128" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+    </row>
     <row r="54" ht="12.75" customHeight="1" s="127"/>
     <row r="55" ht="12.75" customHeight="1" s="127"/>
     <row r="56" ht="12.75" customHeight="1" s="127"/>
@@ -11748,7 +11942,7 @@
     <mergeCell ref="R1:R2"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.196527777777778" right="0.196527777777778" top="0.196527777777778" bottom="0.196527777777778" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageMargins left="0.625" right="0.625" top="0.55" bottom="1.69" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" cellComments="atEnd" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
@@ -14972,7 +15166,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AN60"/>
+  <dimension ref="A1:AN61"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.13671875" defaultRowHeight="12.75" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="2.56" customWidth="1" style="126" min="1" max="12"/>
@@ -17224,9 +17418,46 @@
         </is>
       </c>
     </row>
-    <row r="59" ht="9" customHeight="1" s="127"/>
-    <row r="60" ht="75" customHeight="1" s="127"/>
-    <row r="61" ht="17.25" customHeight="1" s="127"/>
+    <row r="59" ht="0.5" customHeight="1" s="127">
+      <c r="L59" s="126" t="n"/>
+      <c r="M59" s="126" t="n"/>
+      <c r="N59" s="126" t="n"/>
+      <c r="O59" s="126" t="n"/>
+      <c r="P59" s="126" t="n"/>
+      <c r="Q59" s="126" t="n"/>
+      <c r="R59" s="126" t="n"/>
+      <c r="S59" s="126" t="n"/>
+      <c r="T59" s="126" t="n"/>
+      <c r="U59" s="126" t="n"/>
+      <c r="V59" s="126" t="n"/>
+      <c r="W59" s="126" t="n"/>
+      <c r="X59" s="126" t="n"/>
+      <c r="Y59" s="126" t="n"/>
+      <c r="Z59" s="126" t="n"/>
+      <c r="AA59" s="126" t="n"/>
+      <c r="AB59" s="126" t="n"/>
+      <c r="AC59" s="126" t="n"/>
+      <c r="AD59" s="126" t="n"/>
+      <c r="AE59" s="126" t="n"/>
+      <c r="AF59" s="126" t="n"/>
+      <c r="AG59" s="126" t="n"/>
+      <c r="AH59" s="126" t="n"/>
+      <c r="AI59" s="126" t="n"/>
+      <c r="AJ59" s="126" t="n"/>
+    </row>
+    <row r="60" ht="13.5" customHeight="1" s="127">
+      <c r="A60" s="128" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="AN60" s="128" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="7.599999999999795" customHeight="1" s="127"/>
     <row r="62" ht="17.25" customHeight="1" s="127"/>
     <row r="131" ht="17.25" customHeight="1" s="127"/>
     <row r="132" ht="17.25" customHeight="1" s="127"/>
@@ -17483,7 +17714,7 @@
     <mergeCell ref="R1:R2"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.196527777777778" right="0.196527777777778" top="0.196527777777778" bottom="0.196527777777778" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageMargins left="0.625" right="0.625" top="0.55" bottom="1.69" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" cellComments="atEnd" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
@@ -17495,7 +17726,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AN26"/>
+  <dimension ref="A1:AN63"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.13671875" defaultRowHeight="12.75" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="2.56" customWidth="1" style="126" min="1" max="12"/>
@@ -18660,45 +18891,1425 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="9" customFormat="1" customHeight="1" s="184"/>
-    <row r="26" ht="75" customFormat="1" customHeight="1" s="184"/>
-    <row r="27" ht="13.15" customFormat="1" customHeight="1" s="184"/>
-    <row r="28" ht="13.15" customFormat="1" customHeight="1" s="184"/>
-    <row r="29" ht="13.15" customFormat="1" customHeight="1" s="184"/>
-    <row r="30" ht="13.15" customFormat="1" customHeight="1" s="184"/>
-    <row r="31" ht="13.15" customFormat="1" customHeight="1" s="184"/>
-    <row r="32" ht="13.15" customFormat="1" customHeight="1" s="184"/>
-    <row r="33" ht="13.15" customFormat="1" customHeight="1" s="184"/>
-    <row r="34" ht="13.15" customFormat="1" customHeight="1" s="184"/>
-    <row r="35" ht="13.15" customFormat="1" customHeight="1" s="184"/>
-    <row r="36" ht="13.15" customFormat="1" customHeight="1" s="184"/>
-    <row r="37" ht="13.15" customFormat="1" customHeight="1" s="184"/>
-    <row r="38" ht="13.15" customFormat="1" customHeight="1" s="184"/>
-    <row r="39" ht="13.15" customFormat="1" customHeight="1" s="184"/>
-    <row r="40" ht="13.15" customFormat="1" customHeight="1" s="184"/>
-    <row r="41" ht="13.15" customFormat="1" customHeight="1" s="184"/>
-    <row r="42" ht="13.15" customFormat="1" customHeight="1" s="184"/>
-    <row r="43" ht="13.15" customFormat="1" customHeight="1" s="184"/>
-    <row r="44" ht="13.15" customFormat="1" customHeight="1" s="184"/>
-    <row r="45" ht="13.15" customFormat="1" customHeight="1" s="184"/>
-    <row r="46" ht="13.15" customFormat="1" customHeight="1" s="184"/>
-    <row r="47" ht="13.15" customFormat="1" customHeight="1" s="184"/>
-    <row r="48" ht="13.15" customFormat="1" customHeight="1" s="184"/>
-    <row r="49" ht="13.15" customFormat="1" customHeight="1" s="184"/>
-    <row r="50" ht="13.15" customFormat="1" customHeight="1" s="184"/>
-    <row r="51" ht="13.15" customFormat="1" customHeight="1" s="184"/>
-    <row r="52" ht="13.15" customFormat="1" customHeight="1" s="184"/>
-    <row r="53" ht="13.15" customFormat="1" customHeight="1" s="184"/>
-    <row r="54" ht="13.15" customFormat="1" customHeight="1" s="184"/>
-    <row r="55" ht="13.15" customFormat="1" customHeight="1" s="184"/>
-    <row r="56" ht="13.15" customFormat="1" customHeight="1" s="184"/>
-    <row r="57" ht="13.15" customFormat="1" customHeight="1" s="184"/>
-    <row r="58" ht="13.15" customFormat="1" customHeight="1" s="184"/>
-    <row r="59" ht="13.15" customFormat="1" customHeight="1" s="184"/>
-    <row r="60" ht="13.15" customFormat="1" customHeight="1" s="184"/>
-    <row r="61" ht="7.5" customFormat="1" customHeight="1" s="184"/>
-    <row r="62" ht="13.5" customHeight="1" s="127"/>
-    <row r="63" ht="17.25" customHeight="1" s="127"/>
+    <row r="25" ht="0.5" customFormat="1" customHeight="1" s="184">
+      <c r="A25" s="212" t="n"/>
+      <c r="B25" s="212" t="n"/>
+      <c r="C25" s="212" t="n"/>
+      <c r="D25" s="212" t="n"/>
+      <c r="E25" s="212" t="n"/>
+      <c r="F25" s="212" t="n"/>
+      <c r="G25" s="212" t="n"/>
+      <c r="H25" s="212" t="n"/>
+      <c r="I25" s="212" t="n"/>
+      <c r="J25" s="212" t="n"/>
+      <c r="K25" s="212" t="n"/>
+      <c r="L25" s="212" t="n"/>
+      <c r="M25" s="212" t="n"/>
+      <c r="N25" s="212" t="n"/>
+      <c r="O25" s="212" t="n"/>
+      <c r="P25" s="212" t="n"/>
+      <c r="Q25" s="212" t="n"/>
+      <c r="R25" s="212" t="n"/>
+      <c r="S25" s="212" t="n"/>
+      <c r="T25" s="212" t="n"/>
+      <c r="U25" s="212" t="n"/>
+      <c r="V25" s="212" t="n"/>
+      <c r="W25" s="212" t="n"/>
+      <c r="X25" s="212" t="n"/>
+      <c r="Y25" s="212" t="n"/>
+      <c r="Z25" s="212" t="n"/>
+      <c r="AA25" s="184" t="n"/>
+      <c r="AB25" s="184" t="n"/>
+      <c r="AC25" s="184" t="n"/>
+      <c r="AD25" s="184" t="n"/>
+      <c r="AE25" s="184" t="n"/>
+      <c r="AF25" s="184" t="n"/>
+      <c r="AG25" s="184" t="n"/>
+      <c r="AH25" s="184" t="n"/>
+      <c r="AI25" s="184" t="n"/>
+      <c r="AJ25" s="184" t="n"/>
+    </row>
+    <row r="26" ht="0.5" customFormat="1" customHeight="1" s="184">
+      <c r="A26" s="212" t="n"/>
+      <c r="B26" s="212" t="n"/>
+      <c r="C26" s="212" t="n"/>
+      <c r="D26" s="212" t="n"/>
+      <c r="E26" s="212" t="n"/>
+      <c r="F26" s="212" t="n"/>
+      <c r="G26" s="212" t="n"/>
+      <c r="H26" s="212" t="n"/>
+      <c r="I26" s="212" t="n"/>
+      <c r="J26" s="212" t="n"/>
+      <c r="K26" s="212" t="n"/>
+      <c r="L26" s="212" t="n"/>
+      <c r="M26" s="212" t="n"/>
+      <c r="N26" s="212" t="n"/>
+      <c r="O26" s="212" t="n"/>
+      <c r="P26" s="212" t="n"/>
+      <c r="Q26" s="212" t="n"/>
+      <c r="R26" s="212" t="n"/>
+      <c r="S26" s="212" t="n"/>
+      <c r="T26" s="212" t="n"/>
+      <c r="U26" s="212" t="n"/>
+      <c r="V26" s="212" t="n"/>
+      <c r="W26" s="212" t="n"/>
+      <c r="X26" s="212" t="n"/>
+      <c r="Y26" s="212" t="n"/>
+      <c r="Z26" s="212" t="n"/>
+      <c r="AA26" s="184" t="n"/>
+      <c r="AB26" s="184" t="n"/>
+      <c r="AC26" s="184" t="n"/>
+      <c r="AD26" s="184" t="n"/>
+      <c r="AE26" s="184" t="n"/>
+      <c r="AF26" s="184" t="n"/>
+      <c r="AG26" s="184" t="n"/>
+      <c r="AH26" s="184" t="n"/>
+      <c r="AI26" s="184" t="n"/>
+      <c r="AJ26" s="184" t="n"/>
+    </row>
+    <row r="27" ht="0.5" customFormat="1" customHeight="1" s="184">
+      <c r="A27" s="212" t="n"/>
+      <c r="B27" s="212" t="n"/>
+      <c r="C27" s="212" t="n"/>
+      <c r="D27" s="212" t="n"/>
+      <c r="E27" s="212" t="n"/>
+      <c r="F27" s="212" t="n"/>
+      <c r="G27" s="212" t="n"/>
+      <c r="H27" s="212" t="n"/>
+      <c r="I27" s="212" t="n"/>
+      <c r="J27" s="212" t="n"/>
+      <c r="K27" s="212" t="n"/>
+      <c r="L27" s="212" t="n"/>
+      <c r="M27" s="212" t="n"/>
+      <c r="N27" s="212" t="n"/>
+      <c r="O27" s="212" t="n"/>
+      <c r="P27" s="212" t="n"/>
+      <c r="Q27" s="212" t="n"/>
+      <c r="R27" s="212" t="n"/>
+      <c r="S27" s="212" t="n"/>
+      <c r="T27" s="212" t="n"/>
+      <c r="U27" s="212" t="n"/>
+      <c r="V27" s="212" t="n"/>
+      <c r="W27" s="212" t="n"/>
+      <c r="X27" s="212" t="n"/>
+      <c r="Y27" s="212" t="n"/>
+      <c r="Z27" s="212" t="n"/>
+      <c r="AA27" s="184" t="n"/>
+      <c r="AB27" s="184" t="n"/>
+      <c r="AC27" s="184" t="n"/>
+      <c r="AD27" s="184" t="n"/>
+      <c r="AE27" s="184" t="n"/>
+      <c r="AF27" s="184" t="n"/>
+      <c r="AG27" s="184" t="n"/>
+      <c r="AH27" s="184" t="n"/>
+      <c r="AI27" s="184" t="n"/>
+      <c r="AJ27" s="184" t="n"/>
+    </row>
+    <row r="28" ht="0.5" customFormat="1" customHeight="1" s="184">
+      <c r="A28" s="212" t="n"/>
+      <c r="B28" s="212" t="n"/>
+      <c r="C28" s="212" t="n"/>
+      <c r="D28" s="212" t="n"/>
+      <c r="E28" s="212" t="n"/>
+      <c r="F28" s="212" t="n"/>
+      <c r="G28" s="212" t="n"/>
+      <c r="H28" s="212" t="n"/>
+      <c r="I28" s="212" t="n"/>
+      <c r="J28" s="212" t="n"/>
+      <c r="K28" s="212" t="n"/>
+      <c r="L28" s="212" t="n"/>
+      <c r="M28" s="212" t="n"/>
+      <c r="N28" s="212" t="n"/>
+      <c r="O28" s="212" t="n"/>
+      <c r="P28" s="212" t="n"/>
+      <c r="Q28" s="212" t="n"/>
+      <c r="R28" s="212" t="n"/>
+      <c r="S28" s="212" t="n"/>
+      <c r="T28" s="212" t="n"/>
+      <c r="U28" s="212" t="n"/>
+      <c r="V28" s="212" t="n"/>
+      <c r="W28" s="212" t="n"/>
+      <c r="X28" s="212" t="n"/>
+      <c r="Y28" s="212" t="n"/>
+      <c r="Z28" s="212" t="n"/>
+      <c r="AA28" s="184" t="n"/>
+      <c r="AB28" s="184" t="n"/>
+      <c r="AC28" s="184" t="n"/>
+      <c r="AD28" s="184" t="n"/>
+      <c r="AE28" s="184" t="n"/>
+      <c r="AF28" s="184" t="n"/>
+      <c r="AG28" s="184" t="n"/>
+      <c r="AH28" s="184" t="n"/>
+      <c r="AI28" s="184" t="n"/>
+      <c r="AJ28" s="184" t="n"/>
+    </row>
+    <row r="29" ht="0.5" customFormat="1" customHeight="1" s="184">
+      <c r="A29" s="212" t="n"/>
+      <c r="B29" s="212" t="n"/>
+      <c r="C29" s="212" t="n"/>
+      <c r="D29" s="212" t="n"/>
+      <c r="E29" s="212" t="n"/>
+      <c r="F29" s="212" t="n"/>
+      <c r="G29" s="212" t="n"/>
+      <c r="H29" s="212" t="n"/>
+      <c r="I29" s="212" t="n"/>
+      <c r="J29" s="212" t="n"/>
+      <c r="K29" s="212" t="n"/>
+      <c r="L29" s="212" t="n"/>
+      <c r="M29" s="212" t="n"/>
+      <c r="N29" s="212" t="n"/>
+      <c r="O29" s="212" t="n"/>
+      <c r="P29" s="212" t="n"/>
+      <c r="Q29" s="212" t="n"/>
+      <c r="R29" s="212" t="n"/>
+      <c r="S29" s="212" t="n"/>
+      <c r="T29" s="212" t="n"/>
+      <c r="U29" s="212" t="n"/>
+      <c r="V29" s="212" t="n"/>
+      <c r="W29" s="212" t="n"/>
+      <c r="X29" s="212" t="n"/>
+      <c r="Y29" s="212" t="n"/>
+      <c r="Z29" s="212" t="n"/>
+      <c r="AA29" s="184" t="n"/>
+      <c r="AB29" s="184" t="n"/>
+      <c r="AC29" s="184" t="n"/>
+      <c r="AD29" s="184" t="n"/>
+      <c r="AE29" s="184" t="n"/>
+      <c r="AF29" s="184" t="n"/>
+      <c r="AG29" s="184" t="n"/>
+      <c r="AH29" s="184" t="n"/>
+      <c r="AI29" s="184" t="n"/>
+      <c r="AJ29" s="184" t="n"/>
+    </row>
+    <row r="30" ht="0.5" customFormat="1" customHeight="1" s="184">
+      <c r="A30" s="212" t="n"/>
+      <c r="B30" s="212" t="n"/>
+      <c r="C30" s="212" t="n"/>
+      <c r="D30" s="212" t="n"/>
+      <c r="E30" s="212" t="n"/>
+      <c r="F30" s="212" t="n"/>
+      <c r="G30" s="212" t="n"/>
+      <c r="H30" s="212" t="n"/>
+      <c r="I30" s="212" t="n"/>
+      <c r="J30" s="212" t="n"/>
+      <c r="K30" s="212" t="n"/>
+      <c r="L30" s="212" t="n"/>
+      <c r="M30" s="212" t="n"/>
+      <c r="N30" s="212" t="n"/>
+      <c r="O30" s="212" t="n"/>
+      <c r="P30" s="212" t="n"/>
+      <c r="Q30" s="212" t="n"/>
+      <c r="R30" s="212" t="n"/>
+      <c r="S30" s="212" t="n"/>
+      <c r="T30" s="212" t="n"/>
+      <c r="U30" s="212" t="n"/>
+      <c r="V30" s="212" t="n"/>
+      <c r="W30" s="212" t="n"/>
+      <c r="X30" s="212" t="n"/>
+      <c r="Y30" s="212" t="n"/>
+      <c r="Z30" s="212" t="n"/>
+      <c r="AA30" s="184" t="n"/>
+      <c r="AB30" s="184" t="n"/>
+      <c r="AC30" s="184" t="n"/>
+      <c r="AD30" s="184" t="n"/>
+      <c r="AE30" s="184" t="n"/>
+      <c r="AF30" s="184" t="n"/>
+      <c r="AG30" s="184" t="n"/>
+      <c r="AH30" s="184" t="n"/>
+      <c r="AI30" s="184" t="n"/>
+      <c r="AJ30" s="184" t="n"/>
+    </row>
+    <row r="31" ht="0.5" customFormat="1" customHeight="1" s="184">
+      <c r="A31" s="212" t="n"/>
+      <c r="B31" s="212" t="n"/>
+      <c r="C31" s="212" t="n"/>
+      <c r="D31" s="212" t="n"/>
+      <c r="E31" s="212" t="n"/>
+      <c r="F31" s="212" t="n"/>
+      <c r="G31" s="212" t="n"/>
+      <c r="H31" s="212" t="n"/>
+      <c r="I31" s="212" t="n"/>
+      <c r="J31" s="212" t="n"/>
+      <c r="K31" s="212" t="n"/>
+      <c r="L31" s="212" t="n"/>
+      <c r="M31" s="212" t="n"/>
+      <c r="N31" s="212" t="n"/>
+      <c r="O31" s="212" t="n"/>
+      <c r="P31" s="212" t="n"/>
+      <c r="Q31" s="212" t="n"/>
+      <c r="R31" s="212" t="n"/>
+      <c r="S31" s="212" t="n"/>
+      <c r="T31" s="212" t="n"/>
+      <c r="U31" s="212" t="n"/>
+      <c r="V31" s="212" t="n"/>
+      <c r="W31" s="212" t="n"/>
+      <c r="X31" s="212" t="n"/>
+      <c r="Y31" s="212" t="n"/>
+      <c r="Z31" s="212" t="n"/>
+      <c r="AA31" s="184" t="n"/>
+      <c r="AB31" s="184" t="n"/>
+      <c r="AC31" s="184" t="n"/>
+      <c r="AD31" s="184" t="n"/>
+      <c r="AE31" s="184" t="n"/>
+      <c r="AF31" s="184" t="n"/>
+      <c r="AG31" s="184" t="n"/>
+      <c r="AH31" s="184" t="n"/>
+      <c r="AI31" s="184" t="n"/>
+      <c r="AJ31" s="184" t="n"/>
+    </row>
+    <row r="32" ht="0.5" customFormat="1" customHeight="1" s="184">
+      <c r="A32" s="212" t="n"/>
+      <c r="B32" s="212" t="n"/>
+      <c r="C32" s="212" t="n"/>
+      <c r="D32" s="212" t="n"/>
+      <c r="E32" s="212" t="n"/>
+      <c r="F32" s="212" t="n"/>
+      <c r="G32" s="212" t="n"/>
+      <c r="H32" s="212" t="n"/>
+      <c r="I32" s="212" t="n"/>
+      <c r="J32" s="212" t="n"/>
+      <c r="K32" s="212" t="n"/>
+      <c r="L32" s="212" t="n"/>
+      <c r="M32" s="212" t="n"/>
+      <c r="N32" s="212" t="n"/>
+      <c r="O32" s="212" t="n"/>
+      <c r="P32" s="212" t="n"/>
+      <c r="Q32" s="212" t="n"/>
+      <c r="R32" s="212" t="n"/>
+      <c r="S32" s="212" t="n"/>
+      <c r="T32" s="212" t="n"/>
+      <c r="U32" s="212" t="n"/>
+      <c r="V32" s="212" t="n"/>
+      <c r="W32" s="212" t="n"/>
+      <c r="X32" s="212" t="n"/>
+      <c r="Y32" s="212" t="n"/>
+      <c r="Z32" s="212" t="n"/>
+      <c r="AA32" s="184" t="n"/>
+      <c r="AB32" s="184" t="n"/>
+      <c r="AC32" s="184" t="n"/>
+      <c r="AD32" s="184" t="n"/>
+      <c r="AE32" s="184" t="n"/>
+      <c r="AF32" s="184" t="n"/>
+      <c r="AG32" s="184" t="n"/>
+      <c r="AH32" s="184" t="n"/>
+      <c r="AI32" s="184" t="n"/>
+      <c r="AJ32" s="184" t="n"/>
+    </row>
+    <row r="33" ht="0.5" customFormat="1" customHeight="1" s="184">
+      <c r="A33" s="212" t="n"/>
+      <c r="B33" s="212" t="n"/>
+      <c r="C33" s="212" t="n"/>
+      <c r="D33" s="212" t="n"/>
+      <c r="E33" s="212" t="n"/>
+      <c r="F33" s="212" t="n"/>
+      <c r="G33" s="212" t="n"/>
+      <c r="H33" s="212" t="n"/>
+      <c r="I33" s="212" t="n"/>
+      <c r="J33" s="212" t="n"/>
+      <c r="K33" s="212" t="n"/>
+      <c r="L33" s="212" t="n"/>
+      <c r="M33" s="212" t="n"/>
+      <c r="N33" s="212" t="n"/>
+      <c r="O33" s="212" t="n"/>
+      <c r="P33" s="212" t="n"/>
+      <c r="Q33" s="212" t="n"/>
+      <c r="R33" s="212" t="n"/>
+      <c r="S33" s="212" t="n"/>
+      <c r="T33" s="212" t="n"/>
+      <c r="U33" s="212" t="n"/>
+      <c r="V33" s="212" t="n"/>
+      <c r="W33" s="212" t="n"/>
+      <c r="X33" s="212" t="n"/>
+      <c r="Y33" s="212" t="n"/>
+      <c r="Z33" s="212" t="n"/>
+      <c r="AA33" s="184" t="n"/>
+      <c r="AB33" s="184" t="n"/>
+      <c r="AC33" s="184" t="n"/>
+      <c r="AD33" s="184" t="n"/>
+      <c r="AE33" s="184" t="n"/>
+      <c r="AF33" s="184" t="n"/>
+      <c r="AG33" s="184" t="n"/>
+      <c r="AH33" s="184" t="n"/>
+      <c r="AI33" s="184" t="n"/>
+      <c r="AJ33" s="184" t="n"/>
+    </row>
+    <row r="34" ht="0.5" customFormat="1" customHeight="1" s="184">
+      <c r="A34" s="212" t="n"/>
+      <c r="B34" s="212" t="n"/>
+      <c r="C34" s="212" t="n"/>
+      <c r="D34" s="212" t="n"/>
+      <c r="E34" s="212" t="n"/>
+      <c r="F34" s="212" t="n"/>
+      <c r="G34" s="212" t="n"/>
+      <c r="H34" s="212" t="n"/>
+      <c r="I34" s="212" t="n"/>
+      <c r="J34" s="212" t="n"/>
+      <c r="K34" s="212" t="n"/>
+      <c r="L34" s="212" t="n"/>
+      <c r="M34" s="212" t="n"/>
+      <c r="N34" s="212" t="n"/>
+      <c r="O34" s="212" t="n"/>
+      <c r="P34" s="212" t="n"/>
+      <c r="Q34" s="212" t="n"/>
+      <c r="R34" s="212" t="n"/>
+      <c r="S34" s="212" t="n"/>
+      <c r="T34" s="212" t="n"/>
+      <c r="U34" s="212" t="n"/>
+      <c r="V34" s="212" t="n"/>
+      <c r="W34" s="212" t="n"/>
+      <c r="X34" s="212" t="n"/>
+      <c r="Y34" s="212" t="n"/>
+      <c r="Z34" s="212" t="n"/>
+      <c r="AA34" s="184" t="n"/>
+      <c r="AB34" s="184" t="n"/>
+      <c r="AC34" s="184" t="n"/>
+      <c r="AD34" s="184" t="n"/>
+      <c r="AE34" s="184" t="n"/>
+      <c r="AF34" s="184" t="n"/>
+      <c r="AG34" s="184" t="n"/>
+      <c r="AH34" s="184" t="n"/>
+      <c r="AI34" s="184" t="n"/>
+      <c r="AJ34" s="184" t="n"/>
+    </row>
+    <row r="35" ht="0.5" customFormat="1" customHeight="1" s="184">
+      <c r="A35" s="212" t="n"/>
+      <c r="B35" s="212" t="n"/>
+      <c r="C35" s="212" t="n"/>
+      <c r="D35" s="212" t="n"/>
+      <c r="E35" s="212" t="n"/>
+      <c r="F35" s="212" t="n"/>
+      <c r="G35" s="212" t="n"/>
+      <c r="H35" s="212" t="n"/>
+      <c r="I35" s="212" t="n"/>
+      <c r="J35" s="212" t="n"/>
+      <c r="K35" s="212" t="n"/>
+      <c r="L35" s="212" t="n"/>
+      <c r="M35" s="212" t="n"/>
+      <c r="N35" s="212" t="n"/>
+      <c r="O35" s="212" t="n"/>
+      <c r="P35" s="212" t="n"/>
+      <c r="Q35" s="212" t="n"/>
+      <c r="R35" s="212" t="n"/>
+      <c r="S35" s="212" t="n"/>
+      <c r="T35" s="212" t="n"/>
+      <c r="U35" s="212" t="n"/>
+      <c r="V35" s="212" t="n"/>
+      <c r="W35" s="212" t="n"/>
+      <c r="X35" s="212" t="n"/>
+      <c r="Y35" s="212" t="n"/>
+      <c r="Z35" s="212" t="n"/>
+      <c r="AA35" s="184" t="n"/>
+      <c r="AB35" s="184" t="n"/>
+      <c r="AC35" s="184" t="n"/>
+      <c r="AD35" s="184" t="n"/>
+      <c r="AE35" s="184" t="n"/>
+      <c r="AF35" s="184" t="n"/>
+      <c r="AG35" s="184" t="n"/>
+      <c r="AH35" s="184" t="n"/>
+      <c r="AI35" s="184" t="n"/>
+      <c r="AJ35" s="184" t="n"/>
+    </row>
+    <row r="36" ht="0.5" customFormat="1" customHeight="1" s="184">
+      <c r="A36" s="212" t="n"/>
+      <c r="B36" s="212" t="n"/>
+      <c r="C36" s="212" t="n"/>
+      <c r="D36" s="212" t="n"/>
+      <c r="E36" s="212" t="n"/>
+      <c r="F36" s="212" t="n"/>
+      <c r="G36" s="212" t="n"/>
+      <c r="H36" s="212" t="n"/>
+      <c r="I36" s="212" t="n"/>
+      <c r="J36" s="212" t="n"/>
+      <c r="K36" s="212" t="n"/>
+      <c r="L36" s="212" t="n"/>
+      <c r="M36" s="212" t="n"/>
+      <c r="N36" s="212" t="n"/>
+      <c r="O36" s="212" t="n"/>
+      <c r="P36" s="212" t="n"/>
+      <c r="Q36" s="212" t="n"/>
+      <c r="R36" s="212" t="n"/>
+      <c r="S36" s="212" t="n"/>
+      <c r="T36" s="212" t="n"/>
+      <c r="U36" s="212" t="n"/>
+      <c r="V36" s="212" t="n"/>
+      <c r="W36" s="212" t="n"/>
+      <c r="X36" s="212" t="n"/>
+      <c r="Y36" s="212" t="n"/>
+      <c r="Z36" s="212" t="n"/>
+      <c r="AA36" s="184" t="n"/>
+      <c r="AB36" s="184" t="n"/>
+      <c r="AC36" s="184" t="n"/>
+      <c r="AD36" s="184" t="n"/>
+      <c r="AE36" s="184" t="n"/>
+      <c r="AF36" s="184" t="n"/>
+      <c r="AG36" s="184" t="n"/>
+      <c r="AH36" s="184" t="n"/>
+      <c r="AI36" s="184" t="n"/>
+      <c r="AJ36" s="184" t="n"/>
+    </row>
+    <row r="37" ht="0.5" customFormat="1" customHeight="1" s="184">
+      <c r="A37" s="212" t="n"/>
+      <c r="B37" s="212" t="n"/>
+      <c r="C37" s="212" t="n"/>
+      <c r="D37" s="212" t="n"/>
+      <c r="E37" s="212" t="n"/>
+      <c r="F37" s="212" t="n"/>
+      <c r="G37" s="212" t="n"/>
+      <c r="H37" s="212" t="n"/>
+      <c r="I37" s="212" t="n"/>
+      <c r="J37" s="212" t="n"/>
+      <c r="K37" s="212" t="n"/>
+      <c r="L37" s="212" t="n"/>
+      <c r="M37" s="212" t="n"/>
+      <c r="N37" s="212" t="n"/>
+      <c r="O37" s="212" t="n"/>
+      <c r="P37" s="212" t="n"/>
+      <c r="Q37" s="212" t="n"/>
+      <c r="R37" s="212" t="n"/>
+      <c r="S37" s="212" t="n"/>
+      <c r="T37" s="212" t="n"/>
+      <c r="U37" s="212" t="n"/>
+      <c r="V37" s="212" t="n"/>
+      <c r="W37" s="212" t="n"/>
+      <c r="X37" s="212" t="n"/>
+      <c r="Y37" s="212" t="n"/>
+      <c r="Z37" s="212" t="n"/>
+      <c r="AA37" s="184" t="n"/>
+      <c r="AB37" s="184" t="n"/>
+      <c r="AC37" s="184" t="n"/>
+      <c r="AD37" s="184" t="n"/>
+      <c r="AE37" s="184" t="n"/>
+      <c r="AF37" s="184" t="n"/>
+      <c r="AG37" s="184" t="n"/>
+      <c r="AH37" s="184" t="n"/>
+      <c r="AI37" s="184" t="n"/>
+      <c r="AJ37" s="184" t="n"/>
+    </row>
+    <row r="38" ht="0.5" customFormat="1" customHeight="1" s="184">
+      <c r="A38" s="212" t="n"/>
+      <c r="B38" s="212" t="n"/>
+      <c r="C38" s="212" t="n"/>
+      <c r="D38" s="212" t="n"/>
+      <c r="E38" s="212" t="n"/>
+      <c r="F38" s="212" t="n"/>
+      <c r="G38" s="212" t="n"/>
+      <c r="H38" s="212" t="n"/>
+      <c r="I38" s="212" t="n"/>
+      <c r="J38" s="212" t="n"/>
+      <c r="K38" s="212" t="n"/>
+      <c r="L38" s="212" t="n"/>
+      <c r="M38" s="212" t="n"/>
+      <c r="N38" s="212" t="n"/>
+      <c r="O38" s="212" t="n"/>
+      <c r="P38" s="212" t="n"/>
+      <c r="Q38" s="212" t="n"/>
+      <c r="R38" s="212" t="n"/>
+      <c r="S38" s="212" t="n"/>
+      <c r="T38" s="212" t="n"/>
+      <c r="U38" s="212" t="n"/>
+      <c r="V38" s="212" t="n"/>
+      <c r="W38" s="212" t="n"/>
+      <c r="X38" s="212" t="n"/>
+      <c r="Y38" s="212" t="n"/>
+      <c r="Z38" s="212" t="n"/>
+      <c r="AA38" s="184" t="n"/>
+      <c r="AB38" s="184" t="n"/>
+      <c r="AC38" s="184" t="n"/>
+      <c r="AD38" s="184" t="n"/>
+      <c r="AE38" s="184" t="n"/>
+      <c r="AF38" s="184" t="n"/>
+      <c r="AG38" s="184" t="n"/>
+      <c r="AH38" s="184" t="n"/>
+      <c r="AI38" s="184" t="n"/>
+      <c r="AJ38" s="184" t="n"/>
+    </row>
+    <row r="39" ht="0.5" customFormat="1" customHeight="1" s="184">
+      <c r="A39" s="212" t="n"/>
+      <c r="B39" s="212" t="n"/>
+      <c r="C39" s="212" t="n"/>
+      <c r="D39" s="212" t="n"/>
+      <c r="E39" s="212" t="n"/>
+      <c r="F39" s="212" t="n"/>
+      <c r="G39" s="212" t="n"/>
+      <c r="H39" s="212" t="n"/>
+      <c r="I39" s="212" t="n"/>
+      <c r="J39" s="212" t="n"/>
+      <c r="K39" s="212" t="n"/>
+      <c r="L39" s="212" t="n"/>
+      <c r="M39" s="212" t="n"/>
+      <c r="N39" s="212" t="n"/>
+      <c r="O39" s="212" t="n"/>
+      <c r="P39" s="212" t="n"/>
+      <c r="Q39" s="212" t="n"/>
+      <c r="R39" s="212" t="n"/>
+      <c r="S39" s="212" t="n"/>
+      <c r="T39" s="212" t="n"/>
+      <c r="U39" s="212" t="n"/>
+      <c r="V39" s="212" t="n"/>
+      <c r="W39" s="212" t="n"/>
+      <c r="X39" s="212" t="n"/>
+      <c r="Y39" s="212" t="n"/>
+      <c r="Z39" s="212" t="n"/>
+      <c r="AA39" s="184" t="n"/>
+      <c r="AB39" s="184" t="n"/>
+      <c r="AC39" s="184" t="n"/>
+      <c r="AD39" s="184" t="n"/>
+      <c r="AE39" s="184" t="n"/>
+      <c r="AF39" s="184" t="n"/>
+      <c r="AG39" s="184" t="n"/>
+      <c r="AH39" s="184" t="n"/>
+      <c r="AI39" s="184" t="n"/>
+      <c r="AJ39" s="184" t="n"/>
+    </row>
+    <row r="40" ht="0.5" customFormat="1" customHeight="1" s="184">
+      <c r="A40" s="212" t="n"/>
+      <c r="B40" s="212" t="n"/>
+      <c r="C40" s="212" t="n"/>
+      <c r="D40" s="212" t="n"/>
+      <c r="E40" s="212" t="n"/>
+      <c r="F40" s="212" t="n"/>
+      <c r="G40" s="212" t="n"/>
+      <c r="H40" s="212" t="n"/>
+      <c r="I40" s="212" t="n"/>
+      <c r="J40" s="212" t="n"/>
+      <c r="K40" s="212" t="n"/>
+      <c r="L40" s="212" t="n"/>
+      <c r="M40" s="212" t="n"/>
+      <c r="N40" s="212" t="n"/>
+      <c r="O40" s="212" t="n"/>
+      <c r="P40" s="212" t="n"/>
+      <c r="Q40" s="212" t="n"/>
+      <c r="R40" s="212" t="n"/>
+      <c r="S40" s="212" t="n"/>
+      <c r="T40" s="212" t="n"/>
+      <c r="U40" s="212" t="n"/>
+      <c r="V40" s="212" t="n"/>
+      <c r="W40" s="212" t="n"/>
+      <c r="X40" s="212" t="n"/>
+      <c r="Y40" s="212" t="n"/>
+      <c r="Z40" s="212" t="n"/>
+      <c r="AA40" s="184" t="n"/>
+      <c r="AB40" s="184" t="n"/>
+      <c r="AC40" s="184" t="n"/>
+      <c r="AD40" s="184" t="n"/>
+      <c r="AE40" s="184" t="n"/>
+      <c r="AF40" s="184" t="n"/>
+      <c r="AG40" s="184" t="n"/>
+      <c r="AH40" s="184" t="n"/>
+      <c r="AI40" s="184" t="n"/>
+      <c r="AJ40" s="184" t="n"/>
+    </row>
+    <row r="41" ht="0.5" customFormat="1" customHeight="1" s="184">
+      <c r="A41" s="212" t="n"/>
+      <c r="B41" s="212" t="n"/>
+      <c r="C41" s="212" t="n"/>
+      <c r="D41" s="212" t="n"/>
+      <c r="E41" s="212" t="n"/>
+      <c r="F41" s="212" t="n"/>
+      <c r="G41" s="212" t="n"/>
+      <c r="H41" s="212" t="n"/>
+      <c r="I41" s="212" t="n"/>
+      <c r="J41" s="212" t="n"/>
+      <c r="K41" s="212" t="n"/>
+      <c r="L41" s="212" t="n"/>
+      <c r="M41" s="212" t="n"/>
+      <c r="N41" s="212" t="n"/>
+      <c r="O41" s="212" t="n"/>
+      <c r="P41" s="212" t="n"/>
+      <c r="Q41" s="212" t="n"/>
+      <c r="R41" s="212" t="n"/>
+      <c r="S41" s="212" t="n"/>
+      <c r="T41" s="212" t="n"/>
+      <c r="U41" s="212" t="n"/>
+      <c r="V41" s="212" t="n"/>
+      <c r="W41" s="212" t="n"/>
+      <c r="X41" s="212" t="n"/>
+      <c r="Y41" s="212" t="n"/>
+      <c r="Z41" s="212" t="n"/>
+      <c r="AA41" s="184" t="n"/>
+      <c r="AB41" s="184" t="n"/>
+      <c r="AC41" s="184" t="n"/>
+      <c r="AD41" s="184" t="n"/>
+      <c r="AE41" s="184" t="n"/>
+      <c r="AF41" s="184" t="n"/>
+      <c r="AG41" s="184" t="n"/>
+      <c r="AH41" s="184" t="n"/>
+      <c r="AI41" s="184" t="n"/>
+      <c r="AJ41" s="184" t="n"/>
+    </row>
+    <row r="42" ht="0.5" customFormat="1" customHeight="1" s="184">
+      <c r="A42" s="212" t="n"/>
+      <c r="B42" s="212" t="n"/>
+      <c r="C42" s="212" t="n"/>
+      <c r="D42" s="212" t="n"/>
+      <c r="E42" s="212" t="n"/>
+      <c r="F42" s="212" t="n"/>
+      <c r="G42" s="212" t="n"/>
+      <c r="H42" s="212" t="n"/>
+      <c r="I42" s="212" t="n"/>
+      <c r="J42" s="212" t="n"/>
+      <c r="K42" s="212" t="n"/>
+      <c r="L42" s="212" t="n"/>
+      <c r="M42" s="212" t="n"/>
+      <c r="N42" s="212" t="n"/>
+      <c r="O42" s="212" t="n"/>
+      <c r="P42" s="212" t="n"/>
+      <c r="Q42" s="212" t="n"/>
+      <c r="R42" s="212" t="n"/>
+      <c r="S42" s="212" t="n"/>
+      <c r="T42" s="212" t="n"/>
+      <c r="U42" s="212" t="n"/>
+      <c r="V42" s="212" t="n"/>
+      <c r="W42" s="212" t="n"/>
+      <c r="X42" s="212" t="n"/>
+      <c r="Y42" s="212" t="n"/>
+      <c r="Z42" s="212" t="n"/>
+      <c r="AA42" s="184" t="n"/>
+      <c r="AB42" s="184" t="n"/>
+      <c r="AC42" s="184" t="n"/>
+      <c r="AD42" s="184" t="n"/>
+      <c r="AE42" s="184" t="n"/>
+      <c r="AF42" s="184" t="n"/>
+      <c r="AG42" s="184" t="n"/>
+      <c r="AH42" s="184" t="n"/>
+      <c r="AI42" s="184" t="n"/>
+      <c r="AJ42" s="184" t="n"/>
+    </row>
+    <row r="43" ht="0.5" customFormat="1" customHeight="1" s="184">
+      <c r="A43" s="212" t="n"/>
+      <c r="B43" s="212" t="n"/>
+      <c r="C43" s="212" t="n"/>
+      <c r="D43" s="212" t="n"/>
+      <c r="E43" s="212" t="n"/>
+      <c r="F43" s="212" t="n"/>
+      <c r="G43" s="212" t="n"/>
+      <c r="H43" s="212" t="n"/>
+      <c r="I43" s="212" t="n"/>
+      <c r="J43" s="212" t="n"/>
+      <c r="K43" s="212" t="n"/>
+      <c r="L43" s="212" t="n"/>
+      <c r="M43" s="212" t="n"/>
+      <c r="N43" s="212" t="n"/>
+      <c r="O43" s="212" t="n"/>
+      <c r="P43" s="212" t="n"/>
+      <c r="Q43" s="212" t="n"/>
+      <c r="R43" s="212" t="n"/>
+      <c r="S43" s="212" t="n"/>
+      <c r="T43" s="212" t="n"/>
+      <c r="U43" s="212" t="n"/>
+      <c r="V43" s="212" t="n"/>
+      <c r="W43" s="212" t="n"/>
+      <c r="X43" s="212" t="n"/>
+      <c r="Y43" s="212" t="n"/>
+      <c r="Z43" s="212" t="n"/>
+      <c r="AA43" s="184" t="n"/>
+      <c r="AB43" s="184" t="n"/>
+      <c r="AC43" s="184" t="n"/>
+      <c r="AD43" s="184" t="n"/>
+      <c r="AE43" s="184" t="n"/>
+      <c r="AF43" s="184" t="n"/>
+      <c r="AG43" s="184" t="n"/>
+      <c r="AH43" s="184" t="n"/>
+      <c r="AI43" s="184" t="n"/>
+      <c r="AJ43" s="184" t="n"/>
+    </row>
+    <row r="44" ht="0.5" customFormat="1" customHeight="1" s="184">
+      <c r="A44" s="212" t="n"/>
+      <c r="B44" s="212" t="n"/>
+      <c r="C44" s="212" t="n"/>
+      <c r="D44" s="212" t="n"/>
+      <c r="E44" s="212" t="n"/>
+      <c r="F44" s="212" t="n"/>
+      <c r="G44" s="212" t="n"/>
+      <c r="H44" s="212" t="n"/>
+      <c r="I44" s="212" t="n"/>
+      <c r="J44" s="212" t="n"/>
+      <c r="K44" s="212" t="n"/>
+      <c r="L44" s="212" t="n"/>
+      <c r="M44" s="212" t="n"/>
+      <c r="N44" s="212" t="n"/>
+      <c r="O44" s="212" t="n"/>
+      <c r="P44" s="212" t="n"/>
+      <c r="Q44" s="212" t="n"/>
+      <c r="R44" s="212" t="n"/>
+      <c r="S44" s="212" t="n"/>
+      <c r="T44" s="212" t="n"/>
+      <c r="U44" s="212" t="n"/>
+      <c r="V44" s="212" t="n"/>
+      <c r="W44" s="212" t="n"/>
+      <c r="X44" s="212" t="n"/>
+      <c r="Y44" s="212" t="n"/>
+      <c r="Z44" s="212" t="n"/>
+      <c r="AA44" s="184" t="n"/>
+      <c r="AB44" s="184" t="n"/>
+      <c r="AC44" s="184" t="n"/>
+      <c r="AD44" s="184" t="n"/>
+      <c r="AE44" s="184" t="n"/>
+      <c r="AF44" s="184" t="n"/>
+      <c r="AG44" s="184" t="n"/>
+      <c r="AH44" s="184" t="n"/>
+      <c r="AI44" s="184" t="n"/>
+      <c r="AJ44" s="184" t="n"/>
+    </row>
+    <row r="45" ht="0.5" customFormat="1" customHeight="1" s="184">
+      <c r="A45" s="212" t="n"/>
+      <c r="B45" s="212" t="n"/>
+      <c r="C45" s="212" t="n"/>
+      <c r="D45" s="212" t="n"/>
+      <c r="E45" s="212" t="n"/>
+      <c r="F45" s="212" t="n"/>
+      <c r="G45" s="212" t="n"/>
+      <c r="H45" s="212" t="n"/>
+      <c r="I45" s="212" t="n"/>
+      <c r="J45" s="212" t="n"/>
+      <c r="K45" s="212" t="n"/>
+      <c r="L45" s="212" t="n"/>
+      <c r="M45" s="212" t="n"/>
+      <c r="N45" s="212" t="n"/>
+      <c r="O45" s="212" t="n"/>
+      <c r="P45" s="212" t="n"/>
+      <c r="Q45" s="212" t="n"/>
+      <c r="R45" s="212" t="n"/>
+      <c r="S45" s="212" t="n"/>
+      <c r="T45" s="212" t="n"/>
+      <c r="U45" s="212" t="n"/>
+      <c r="V45" s="212" t="n"/>
+      <c r="W45" s="212" t="n"/>
+      <c r="X45" s="212" t="n"/>
+      <c r="Y45" s="212" t="n"/>
+      <c r="Z45" s="212" t="n"/>
+      <c r="AA45" s="184" t="n"/>
+      <c r="AB45" s="184" t="n"/>
+      <c r="AC45" s="184" t="n"/>
+      <c r="AD45" s="184" t="n"/>
+      <c r="AE45" s="184" t="n"/>
+      <c r="AF45" s="184" t="n"/>
+      <c r="AG45" s="184" t="n"/>
+      <c r="AH45" s="184" t="n"/>
+      <c r="AI45" s="184" t="n"/>
+      <c r="AJ45" s="184" t="n"/>
+    </row>
+    <row r="46" ht="0.5" customFormat="1" customHeight="1" s="184">
+      <c r="A46" s="212" t="n"/>
+      <c r="B46" s="212" t="n"/>
+      <c r="C46" s="212" t="n"/>
+      <c r="D46" s="212" t="n"/>
+      <c r="E46" s="212" t="n"/>
+      <c r="F46" s="212" t="n"/>
+      <c r="G46" s="212" t="n"/>
+      <c r="H46" s="212" t="n"/>
+      <c r="I46" s="212" t="n"/>
+      <c r="J46" s="212" t="n"/>
+      <c r="K46" s="212" t="n"/>
+      <c r="L46" s="212" t="n"/>
+      <c r="M46" s="212" t="n"/>
+      <c r="N46" s="212" t="n"/>
+      <c r="O46" s="212" t="n"/>
+      <c r="P46" s="212" t="n"/>
+      <c r="Q46" s="212" t="n"/>
+      <c r="R46" s="212" t="n"/>
+      <c r="S46" s="212" t="n"/>
+      <c r="T46" s="212" t="n"/>
+      <c r="U46" s="212" t="n"/>
+      <c r="V46" s="212" t="n"/>
+      <c r="W46" s="212" t="n"/>
+      <c r="X46" s="212" t="n"/>
+      <c r="Y46" s="212" t="n"/>
+      <c r="Z46" s="212" t="n"/>
+      <c r="AA46" s="184" t="n"/>
+      <c r="AB46" s="184" t="n"/>
+      <c r="AC46" s="184" t="n"/>
+      <c r="AD46" s="184" t="n"/>
+      <c r="AE46" s="184" t="n"/>
+      <c r="AF46" s="184" t="n"/>
+      <c r="AG46" s="184" t="n"/>
+      <c r="AH46" s="184" t="n"/>
+      <c r="AI46" s="184" t="n"/>
+      <c r="AJ46" s="184" t="n"/>
+    </row>
+    <row r="47" ht="0.5" customFormat="1" customHeight="1" s="184">
+      <c r="A47" s="212" t="n"/>
+      <c r="B47" s="212" t="n"/>
+      <c r="C47" s="212" t="n"/>
+      <c r="D47" s="212" t="n"/>
+      <c r="E47" s="212" t="n"/>
+      <c r="F47" s="212" t="n"/>
+      <c r="G47" s="212" t="n"/>
+      <c r="H47" s="212" t="n"/>
+      <c r="I47" s="212" t="n"/>
+      <c r="J47" s="212" t="n"/>
+      <c r="K47" s="212" t="n"/>
+      <c r="L47" s="212" t="n"/>
+      <c r="M47" s="212" t="n"/>
+      <c r="N47" s="212" t="n"/>
+      <c r="O47" s="212" t="n"/>
+      <c r="P47" s="212" t="n"/>
+      <c r="Q47" s="212" t="n"/>
+      <c r="R47" s="212" t="n"/>
+      <c r="S47" s="212" t="n"/>
+      <c r="T47" s="212" t="n"/>
+      <c r="U47" s="212" t="n"/>
+      <c r="V47" s="212" t="n"/>
+      <c r="W47" s="212" t="n"/>
+      <c r="X47" s="212" t="n"/>
+      <c r="Y47" s="212" t="n"/>
+      <c r="Z47" s="212" t="n"/>
+      <c r="AA47" s="184" t="n"/>
+      <c r="AB47" s="184" t="n"/>
+      <c r="AC47" s="184" t="n"/>
+      <c r="AD47" s="184" t="n"/>
+      <c r="AE47" s="184" t="n"/>
+      <c r="AF47" s="184" t="n"/>
+      <c r="AG47" s="184" t="n"/>
+      <c r="AH47" s="184" t="n"/>
+      <c r="AI47" s="184" t="n"/>
+      <c r="AJ47" s="184" t="n"/>
+    </row>
+    <row r="48" ht="0.5" customFormat="1" customHeight="1" s="184">
+      <c r="A48" s="212" t="n"/>
+      <c r="B48" s="212" t="n"/>
+      <c r="C48" s="212" t="n"/>
+      <c r="D48" s="212" t="n"/>
+      <c r="E48" s="212" t="n"/>
+      <c r="F48" s="212" t="n"/>
+      <c r="G48" s="212" t="n"/>
+      <c r="H48" s="212" t="n"/>
+      <c r="I48" s="212" t="n"/>
+      <c r="J48" s="212" t="n"/>
+      <c r="K48" s="212" t="n"/>
+      <c r="L48" s="212" t="n"/>
+      <c r="M48" s="212" t="n"/>
+      <c r="N48" s="212" t="n"/>
+      <c r="O48" s="212" t="n"/>
+      <c r="P48" s="212" t="n"/>
+      <c r="Q48" s="212" t="n"/>
+      <c r="R48" s="212" t="n"/>
+      <c r="S48" s="212" t="n"/>
+      <c r="T48" s="212" t="n"/>
+      <c r="U48" s="212" t="n"/>
+      <c r="V48" s="212" t="n"/>
+      <c r="W48" s="212" t="n"/>
+      <c r="X48" s="212" t="n"/>
+      <c r="Y48" s="212" t="n"/>
+      <c r="Z48" s="212" t="n"/>
+      <c r="AA48" s="184" t="n"/>
+      <c r="AB48" s="184" t="n"/>
+      <c r="AC48" s="184" t="n"/>
+      <c r="AD48" s="184" t="n"/>
+      <c r="AE48" s="184" t="n"/>
+      <c r="AF48" s="184" t="n"/>
+      <c r="AG48" s="184" t="n"/>
+      <c r="AH48" s="184" t="n"/>
+      <c r="AI48" s="184" t="n"/>
+      <c r="AJ48" s="184" t="n"/>
+    </row>
+    <row r="49" ht="0.5" customFormat="1" customHeight="1" s="184">
+      <c r="A49" s="212" t="n"/>
+      <c r="B49" s="212" t="n"/>
+      <c r="C49" s="212" t="n"/>
+      <c r="D49" s="212" t="n"/>
+      <c r="E49" s="212" t="n"/>
+      <c r="F49" s="212" t="n"/>
+      <c r="G49" s="212" t="n"/>
+      <c r="H49" s="212" t="n"/>
+      <c r="I49" s="212" t="n"/>
+      <c r="J49" s="212" t="n"/>
+      <c r="K49" s="212" t="n"/>
+      <c r="L49" s="212" t="n"/>
+      <c r="M49" s="212" t="n"/>
+      <c r="N49" s="212" t="n"/>
+      <c r="O49" s="212" t="n"/>
+      <c r="P49" s="212" t="n"/>
+      <c r="Q49" s="212" t="n"/>
+      <c r="R49" s="212" t="n"/>
+      <c r="S49" s="212" t="n"/>
+      <c r="T49" s="212" t="n"/>
+      <c r="U49" s="212" t="n"/>
+      <c r="V49" s="212" t="n"/>
+      <c r="W49" s="212" t="n"/>
+      <c r="X49" s="212" t="n"/>
+      <c r="Y49" s="212" t="n"/>
+      <c r="Z49" s="212" t="n"/>
+      <c r="AA49" s="184" t="n"/>
+      <c r="AB49" s="184" t="n"/>
+      <c r="AC49" s="184" t="n"/>
+      <c r="AD49" s="184" t="n"/>
+      <c r="AE49" s="184" t="n"/>
+      <c r="AF49" s="184" t="n"/>
+      <c r="AG49" s="184" t="n"/>
+      <c r="AH49" s="184" t="n"/>
+      <c r="AI49" s="184" t="n"/>
+      <c r="AJ49" s="184" t="n"/>
+    </row>
+    <row r="50" ht="0.5" customFormat="1" customHeight="1" s="184">
+      <c r="A50" s="212" t="n"/>
+      <c r="B50" s="212" t="n"/>
+      <c r="C50" s="212" t="n"/>
+      <c r="D50" s="212" t="n"/>
+      <c r="E50" s="212" t="n"/>
+      <c r="F50" s="212" t="n"/>
+      <c r="G50" s="212" t="n"/>
+      <c r="H50" s="212" t="n"/>
+      <c r="I50" s="212" t="n"/>
+      <c r="J50" s="212" t="n"/>
+      <c r="K50" s="212" t="n"/>
+      <c r="L50" s="212" t="n"/>
+      <c r="M50" s="212" t="n"/>
+      <c r="N50" s="212" t="n"/>
+      <c r="O50" s="212" t="n"/>
+      <c r="P50" s="212" t="n"/>
+      <c r="Q50" s="212" t="n"/>
+      <c r="R50" s="212" t="n"/>
+      <c r="S50" s="212" t="n"/>
+      <c r="T50" s="212" t="n"/>
+      <c r="U50" s="212" t="n"/>
+      <c r="V50" s="212" t="n"/>
+      <c r="W50" s="212" t="n"/>
+      <c r="X50" s="212" t="n"/>
+      <c r="Y50" s="212" t="n"/>
+      <c r="Z50" s="212" t="n"/>
+      <c r="AA50" s="184" t="n"/>
+      <c r="AB50" s="184" t="n"/>
+      <c r="AC50" s="184" t="n"/>
+      <c r="AD50" s="184" t="n"/>
+      <c r="AE50" s="184" t="n"/>
+      <c r="AF50" s="184" t="n"/>
+      <c r="AG50" s="184" t="n"/>
+      <c r="AH50" s="184" t="n"/>
+      <c r="AI50" s="184" t="n"/>
+      <c r="AJ50" s="184" t="n"/>
+    </row>
+    <row r="51" ht="0.5" customFormat="1" customHeight="1" s="184">
+      <c r="A51" s="212" t="n"/>
+      <c r="B51" s="212" t="n"/>
+      <c r="C51" s="212" t="n"/>
+      <c r="D51" s="212" t="n"/>
+      <c r="E51" s="212" t="n"/>
+      <c r="F51" s="212" t="n"/>
+      <c r="G51" s="212" t="n"/>
+      <c r="H51" s="212" t="n"/>
+      <c r="I51" s="212" t="n"/>
+      <c r="J51" s="212" t="n"/>
+      <c r="K51" s="212" t="n"/>
+      <c r="L51" s="212" t="n"/>
+      <c r="M51" s="212" t="n"/>
+      <c r="N51" s="212" t="n"/>
+      <c r="O51" s="212" t="n"/>
+      <c r="P51" s="212" t="n"/>
+      <c r="Q51" s="212" t="n"/>
+      <c r="R51" s="212" t="n"/>
+      <c r="S51" s="212" t="n"/>
+      <c r="T51" s="212" t="n"/>
+      <c r="U51" s="212" t="n"/>
+      <c r="V51" s="212" t="n"/>
+      <c r="W51" s="212" t="n"/>
+      <c r="X51" s="212" t="n"/>
+      <c r="Y51" s="212" t="n"/>
+      <c r="Z51" s="212" t="n"/>
+      <c r="AA51" s="184" t="n"/>
+      <c r="AB51" s="184" t="n"/>
+      <c r="AC51" s="184" t="n"/>
+      <c r="AD51" s="184" t="n"/>
+      <c r="AE51" s="184" t="n"/>
+      <c r="AF51" s="184" t="n"/>
+      <c r="AG51" s="184" t="n"/>
+      <c r="AH51" s="184" t="n"/>
+      <c r="AI51" s="184" t="n"/>
+      <c r="AJ51" s="184" t="n"/>
+    </row>
+    <row r="52" ht="0.5" customFormat="1" customHeight="1" s="184">
+      <c r="A52" s="212" t="n"/>
+      <c r="B52" s="212" t="n"/>
+      <c r="C52" s="212" t="n"/>
+      <c r="D52" s="212" t="n"/>
+      <c r="E52" s="212" t="n"/>
+      <c r="F52" s="212" t="n"/>
+      <c r="G52" s="212" t="n"/>
+      <c r="H52" s="212" t="n"/>
+      <c r="I52" s="212" t="n"/>
+      <c r="J52" s="212" t="n"/>
+      <c r="K52" s="212" t="n"/>
+      <c r="L52" s="212" t="n"/>
+      <c r="M52" s="212" t="n"/>
+      <c r="N52" s="212" t="n"/>
+      <c r="O52" s="212" t="n"/>
+      <c r="P52" s="212" t="n"/>
+      <c r="Q52" s="212" t="n"/>
+      <c r="R52" s="212" t="n"/>
+      <c r="S52" s="212" t="n"/>
+      <c r="T52" s="212" t="n"/>
+      <c r="U52" s="212" t="n"/>
+      <c r="V52" s="212" t="n"/>
+      <c r="W52" s="212" t="n"/>
+      <c r="X52" s="212" t="n"/>
+      <c r="Y52" s="212" t="n"/>
+      <c r="Z52" s="212" t="n"/>
+      <c r="AA52" s="184" t="n"/>
+      <c r="AB52" s="184" t="n"/>
+      <c r="AC52" s="184" t="n"/>
+      <c r="AD52" s="184" t="n"/>
+      <c r="AE52" s="184" t="n"/>
+      <c r="AF52" s="184" t="n"/>
+      <c r="AG52" s="184" t="n"/>
+      <c r="AH52" s="184" t="n"/>
+      <c r="AI52" s="184" t="n"/>
+      <c r="AJ52" s="184" t="n"/>
+    </row>
+    <row r="53" ht="0.5" customFormat="1" customHeight="1" s="184">
+      <c r="A53" s="212" t="n"/>
+      <c r="B53" s="212" t="n"/>
+      <c r="C53" s="212" t="n"/>
+      <c r="D53" s="212" t="n"/>
+      <c r="E53" s="212" t="n"/>
+      <c r="F53" s="212" t="n"/>
+      <c r="G53" s="212" t="n"/>
+      <c r="H53" s="212" t="n"/>
+      <c r="I53" s="212" t="n"/>
+      <c r="J53" s="212" t="n"/>
+      <c r="K53" s="212" t="n"/>
+      <c r="L53" s="212" t="n"/>
+      <c r="M53" s="212" t="n"/>
+      <c r="N53" s="212" t="n"/>
+      <c r="O53" s="212" t="n"/>
+      <c r="P53" s="212" t="n"/>
+      <c r="Q53" s="212" t="n"/>
+      <c r="R53" s="212" t="n"/>
+      <c r="S53" s="212" t="n"/>
+      <c r="T53" s="212" t="n"/>
+      <c r="U53" s="212" t="n"/>
+      <c r="V53" s="212" t="n"/>
+      <c r="W53" s="212" t="n"/>
+      <c r="X53" s="212" t="n"/>
+      <c r="Y53" s="212" t="n"/>
+      <c r="Z53" s="212" t="n"/>
+      <c r="AA53" s="184" t="n"/>
+      <c r="AB53" s="184" t="n"/>
+      <c r="AC53" s="184" t="n"/>
+      <c r="AD53" s="184" t="n"/>
+      <c r="AE53" s="184" t="n"/>
+      <c r="AF53" s="184" t="n"/>
+      <c r="AG53" s="184" t="n"/>
+      <c r="AH53" s="184" t="n"/>
+      <c r="AI53" s="184" t="n"/>
+      <c r="AJ53" s="184" t="n"/>
+    </row>
+    <row r="54" ht="0.5" customFormat="1" customHeight="1" s="184">
+      <c r="A54" s="212" t="n"/>
+      <c r="B54" s="212" t="n"/>
+      <c r="C54" s="212" t="n"/>
+      <c r="D54" s="212" t="n"/>
+      <c r="E54" s="212" t="n"/>
+      <c r="F54" s="212" t="n"/>
+      <c r="G54" s="212" t="n"/>
+      <c r="H54" s="212" t="n"/>
+      <c r="I54" s="212" t="n"/>
+      <c r="J54" s="212" t="n"/>
+      <c r="K54" s="212" t="n"/>
+      <c r="L54" s="212" t="n"/>
+      <c r="M54" s="212" t="n"/>
+      <c r="N54" s="212" t="n"/>
+      <c r="O54" s="212" t="n"/>
+      <c r="P54" s="212" t="n"/>
+      <c r="Q54" s="212" t="n"/>
+      <c r="R54" s="212" t="n"/>
+      <c r="S54" s="212" t="n"/>
+      <c r="T54" s="212" t="n"/>
+      <c r="U54" s="212" t="n"/>
+      <c r="V54" s="212" t="n"/>
+      <c r="W54" s="212" t="n"/>
+      <c r="X54" s="212" t="n"/>
+      <c r="Y54" s="212" t="n"/>
+      <c r="Z54" s="212" t="n"/>
+      <c r="AA54" s="184" t="n"/>
+      <c r="AB54" s="184" t="n"/>
+      <c r="AC54" s="184" t="n"/>
+      <c r="AD54" s="184" t="n"/>
+      <c r="AE54" s="184" t="n"/>
+      <c r="AF54" s="184" t="n"/>
+      <c r="AG54" s="184" t="n"/>
+      <c r="AH54" s="184" t="n"/>
+      <c r="AI54" s="184" t="n"/>
+      <c r="AJ54" s="184" t="n"/>
+    </row>
+    <row r="55" ht="0.5" customFormat="1" customHeight="1" s="184">
+      <c r="A55" s="212" t="n"/>
+      <c r="B55" s="212" t="n"/>
+      <c r="C55" s="212" t="n"/>
+      <c r="D55" s="212" t="n"/>
+      <c r="E55" s="212" t="n"/>
+      <c r="F55" s="212" t="n"/>
+      <c r="G55" s="212" t="n"/>
+      <c r="H55" s="212" t="n"/>
+      <c r="I55" s="212" t="n"/>
+      <c r="J55" s="212" t="n"/>
+      <c r="K55" s="212" t="n"/>
+      <c r="L55" s="212" t="n"/>
+      <c r="M55" s="212" t="n"/>
+      <c r="N55" s="212" t="n"/>
+      <c r="O55" s="212" t="n"/>
+      <c r="P55" s="212" t="n"/>
+      <c r="Q55" s="212" t="n"/>
+      <c r="R55" s="212" t="n"/>
+      <c r="S55" s="212" t="n"/>
+      <c r="T55" s="212" t="n"/>
+      <c r="U55" s="212" t="n"/>
+      <c r="V55" s="212" t="n"/>
+      <c r="W55" s="212" t="n"/>
+      <c r="X55" s="212" t="n"/>
+      <c r="Y55" s="212" t="n"/>
+      <c r="Z55" s="212" t="n"/>
+      <c r="AA55" s="184" t="n"/>
+      <c r="AB55" s="184" t="n"/>
+      <c r="AC55" s="184" t="n"/>
+      <c r="AD55" s="184" t="n"/>
+      <c r="AE55" s="184" t="n"/>
+      <c r="AF55" s="184" t="n"/>
+      <c r="AG55" s="184" t="n"/>
+      <c r="AH55" s="184" t="n"/>
+      <c r="AI55" s="184" t="n"/>
+      <c r="AJ55" s="184" t="n"/>
+    </row>
+    <row r="56" ht="0.5" customFormat="1" customHeight="1" s="184">
+      <c r="A56" s="212" t="n"/>
+      <c r="B56" s="212" t="n"/>
+      <c r="C56" s="212" t="n"/>
+      <c r="D56" s="212" t="n"/>
+      <c r="E56" s="212" t="n"/>
+      <c r="F56" s="212" t="n"/>
+      <c r="G56" s="212" t="n"/>
+      <c r="H56" s="212" t="n"/>
+      <c r="I56" s="212" t="n"/>
+      <c r="J56" s="212" t="n"/>
+      <c r="K56" s="212" t="n"/>
+      <c r="L56" s="212" t="n"/>
+      <c r="M56" s="212" t="n"/>
+      <c r="N56" s="212" t="n"/>
+      <c r="O56" s="212" t="n"/>
+      <c r="P56" s="212" t="n"/>
+      <c r="Q56" s="212" t="n"/>
+      <c r="R56" s="212" t="n"/>
+      <c r="S56" s="212" t="n"/>
+      <c r="T56" s="212" t="n"/>
+      <c r="U56" s="212" t="n"/>
+      <c r="V56" s="212" t="n"/>
+      <c r="W56" s="212" t="n"/>
+      <c r="X56" s="212" t="n"/>
+      <c r="Y56" s="212" t="n"/>
+      <c r="Z56" s="212" t="n"/>
+      <c r="AA56" s="184" t="n"/>
+      <c r="AB56" s="184" t="n"/>
+      <c r="AC56" s="184" t="n"/>
+      <c r="AD56" s="184" t="n"/>
+      <c r="AE56" s="184" t="n"/>
+      <c r="AF56" s="184" t="n"/>
+      <c r="AG56" s="184" t="n"/>
+      <c r="AH56" s="184" t="n"/>
+      <c r="AI56" s="184" t="n"/>
+      <c r="AJ56" s="184" t="n"/>
+    </row>
+    <row r="57" ht="0.5" customFormat="1" customHeight="1" s="184">
+      <c r="A57" s="212" t="n"/>
+      <c r="B57" s="212" t="n"/>
+      <c r="C57" s="212" t="n"/>
+      <c r="D57" s="212" t="n"/>
+      <c r="E57" s="212" t="n"/>
+      <c r="F57" s="212" t="n"/>
+      <c r="G57" s="212" t="n"/>
+      <c r="H57" s="212" t="n"/>
+      <c r="I57" s="212" t="n"/>
+      <c r="J57" s="212" t="n"/>
+      <c r="K57" s="212" t="n"/>
+      <c r="L57" s="212" t="n"/>
+      <c r="M57" s="212" t="n"/>
+      <c r="N57" s="212" t="n"/>
+      <c r="O57" s="212" t="n"/>
+      <c r="P57" s="212" t="n"/>
+      <c r="Q57" s="212" t="n"/>
+      <c r="R57" s="212" t="n"/>
+      <c r="S57" s="212" t="n"/>
+      <c r="T57" s="212" t="n"/>
+      <c r="U57" s="212" t="n"/>
+      <c r="V57" s="212" t="n"/>
+      <c r="W57" s="212" t="n"/>
+      <c r="X57" s="212" t="n"/>
+      <c r="Y57" s="212" t="n"/>
+      <c r="Z57" s="212" t="n"/>
+      <c r="AA57" s="184" t="n"/>
+      <c r="AB57" s="184" t="n"/>
+      <c r="AC57" s="184" t="n"/>
+      <c r="AD57" s="184" t="n"/>
+      <c r="AE57" s="184" t="n"/>
+      <c r="AF57" s="184" t="n"/>
+      <c r="AG57" s="184" t="n"/>
+      <c r="AH57" s="184" t="n"/>
+      <c r="AI57" s="184" t="n"/>
+      <c r="AJ57" s="184" t="n"/>
+    </row>
+    <row r="58" ht="0.5" customFormat="1" customHeight="1" s="184">
+      <c r="A58" s="212" t="n"/>
+      <c r="B58" s="212" t="n"/>
+      <c r="C58" s="212" t="n"/>
+      <c r="D58" s="212" t="n"/>
+      <c r="E58" s="212" t="n"/>
+      <c r="F58" s="212" t="n"/>
+      <c r="G58" s="212" t="n"/>
+      <c r="H58" s="212" t="n"/>
+      <c r="I58" s="212" t="n"/>
+      <c r="J58" s="212" t="n"/>
+      <c r="K58" s="212" t="n"/>
+      <c r="L58" s="212" t="n"/>
+      <c r="M58" s="212" t="n"/>
+      <c r="N58" s="212" t="n"/>
+      <c r="O58" s="212" t="n"/>
+      <c r="P58" s="212" t="n"/>
+      <c r="Q58" s="212" t="n"/>
+      <c r="R58" s="212" t="n"/>
+      <c r="S58" s="212" t="n"/>
+      <c r="T58" s="212" t="n"/>
+      <c r="U58" s="212" t="n"/>
+      <c r="V58" s="212" t="n"/>
+      <c r="W58" s="212" t="n"/>
+      <c r="X58" s="212" t="n"/>
+      <c r="Y58" s="212" t="n"/>
+      <c r="Z58" s="212" t="n"/>
+      <c r="AA58" s="184" t="n"/>
+      <c r="AB58" s="184" t="n"/>
+      <c r="AC58" s="184" t="n"/>
+      <c r="AD58" s="184" t="n"/>
+      <c r="AE58" s="184" t="n"/>
+      <c r="AF58" s="184" t="n"/>
+      <c r="AG58" s="184" t="n"/>
+      <c r="AH58" s="184" t="n"/>
+      <c r="AI58" s="184" t="n"/>
+      <c r="AJ58" s="184" t="n"/>
+    </row>
+    <row r="59" ht="0.5" customFormat="1" customHeight="1" s="184">
+      <c r="A59" s="212" t="n"/>
+      <c r="B59" s="212" t="n"/>
+      <c r="C59" s="212" t="n"/>
+      <c r="D59" s="212" t="n"/>
+      <c r="E59" s="212" t="n"/>
+      <c r="F59" s="212" t="n"/>
+      <c r="G59" s="212" t="n"/>
+      <c r="H59" s="212" t="n"/>
+      <c r="I59" s="212" t="n"/>
+      <c r="J59" s="212" t="n"/>
+      <c r="K59" s="212" t="n"/>
+      <c r="L59" s="212" t="n"/>
+      <c r="M59" s="212" t="n"/>
+      <c r="N59" s="212" t="n"/>
+      <c r="O59" s="212" t="n"/>
+      <c r="P59" s="212" t="n"/>
+      <c r="Q59" s="212" t="n"/>
+      <c r="R59" s="212" t="n"/>
+      <c r="S59" s="212" t="n"/>
+      <c r="T59" s="212" t="n"/>
+      <c r="U59" s="212" t="n"/>
+      <c r="V59" s="212" t="n"/>
+      <c r="W59" s="212" t="n"/>
+      <c r="X59" s="212" t="n"/>
+      <c r="Y59" s="212" t="n"/>
+      <c r="Z59" s="212" t="n"/>
+      <c r="AA59" s="184" t="n"/>
+      <c r="AB59" s="184" t="n"/>
+      <c r="AC59" s="184" t="n"/>
+      <c r="AD59" s="184" t="n"/>
+      <c r="AE59" s="184" t="n"/>
+      <c r="AF59" s="184" t="n"/>
+      <c r="AG59" s="184" t="n"/>
+      <c r="AH59" s="184" t="n"/>
+      <c r="AI59" s="184" t="n"/>
+      <c r="AJ59" s="184" t="n"/>
+    </row>
+    <row r="60" ht="0.5" customFormat="1" customHeight="1" s="184">
+      <c r="A60" s="212" t="n"/>
+      <c r="B60" s="212" t="n"/>
+      <c r="C60" s="212" t="n"/>
+      <c r="D60" s="212" t="n"/>
+      <c r="E60" s="212" t="n"/>
+      <c r="F60" s="212" t="n"/>
+      <c r="G60" s="212" t="n"/>
+      <c r="H60" s="212" t="n"/>
+      <c r="I60" s="212" t="n"/>
+      <c r="J60" s="212" t="n"/>
+      <c r="K60" s="212" t="n"/>
+      <c r="L60" s="212" t="n"/>
+      <c r="M60" s="212" t="n"/>
+      <c r="N60" s="212" t="n"/>
+      <c r="O60" s="212" t="n"/>
+      <c r="P60" s="212" t="n"/>
+      <c r="Q60" s="212" t="n"/>
+      <c r="R60" s="212" t="n"/>
+      <c r="S60" s="212" t="n"/>
+      <c r="T60" s="212" t="n"/>
+      <c r="U60" s="212" t="n"/>
+      <c r="V60" s="212" t="n"/>
+      <c r="W60" s="212" t="n"/>
+      <c r="X60" s="212" t="n"/>
+      <c r="Y60" s="212" t="n"/>
+      <c r="Z60" s="212" t="n"/>
+      <c r="AA60" s="184" t="n"/>
+      <c r="AB60" s="184" t="n"/>
+      <c r="AC60" s="184" t="n"/>
+      <c r="AD60" s="184" t="n"/>
+      <c r="AE60" s="184" t="n"/>
+      <c r="AF60" s="184" t="n"/>
+      <c r="AG60" s="184" t="n"/>
+      <c r="AH60" s="184" t="n"/>
+      <c r="AI60" s="184" t="n"/>
+      <c r="AJ60" s="184" t="n"/>
+    </row>
+    <row r="61" ht="0.5" customFormat="1" customHeight="1" s="184">
+      <c r="A61" s="212" t="n"/>
+      <c r="B61" s="212" t="n"/>
+      <c r="C61" s="212" t="n"/>
+      <c r="D61" s="212" t="n"/>
+      <c r="E61" s="212" t="n"/>
+      <c r="F61" s="212" t="n"/>
+      <c r="G61" s="212" t="n"/>
+      <c r="H61" s="212" t="n"/>
+      <c r="I61" s="212" t="n"/>
+      <c r="J61" s="212" t="n"/>
+      <c r="K61" s="212" t="n"/>
+      <c r="L61" s="212" t="n"/>
+      <c r="M61" s="212" t="n"/>
+      <c r="N61" s="212" t="n"/>
+      <c r="O61" s="212" t="n"/>
+      <c r="P61" s="212" t="n"/>
+      <c r="Q61" s="212" t="n"/>
+      <c r="R61" s="212" t="n"/>
+      <c r="S61" s="212" t="n"/>
+      <c r="T61" s="212" t="n"/>
+      <c r="U61" s="212" t="n"/>
+      <c r="V61" s="212" t="n"/>
+      <c r="W61" s="212" t="n"/>
+      <c r="X61" s="212" t="n"/>
+      <c r="Y61" s="212" t="n"/>
+      <c r="Z61" s="212" t="n"/>
+      <c r="AA61" s="184" t="n"/>
+      <c r="AB61" s="184" t="n"/>
+      <c r="AC61" s="184" t="n"/>
+      <c r="AD61" s="184" t="n"/>
+      <c r="AE61" s="184" t="n"/>
+      <c r="AF61" s="184" t="n"/>
+      <c r="AG61" s="184" t="n"/>
+      <c r="AH61" s="184" t="n"/>
+      <c r="AI61" s="184" t="n"/>
+      <c r="AJ61" s="184" t="n"/>
+    </row>
+    <row r="62" ht="13.5" customHeight="1" s="127">
+      <c r="A62" s="128" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="AN62" s="128" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="461.55" customHeight="1" s="127"/>
     <row r="64" ht="17.25" customHeight="1" s="127"/>
     <row r="133" ht="17.25" customHeight="1" s="127"/>
     <row r="134" ht="17.25" customHeight="1" s="127"/>
@@ -18923,7 +20534,7 @@
     <mergeCell ref="R1:R2"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.196527777777778" right="0.196527777777778" top="0.196527777777778" bottom="0.196527777777778" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageMargins left="0.625" right="0.625" top="0.55" bottom="1.69" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" cellComments="atEnd" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
@@ -19388,7 +20999,7 @@
       <c r="AM14" s="130" t="n"/>
     </row>
     <row r="15" ht="7.5" customHeight="1" s="127">
-      <c r="A15" s="212" t="n"/>
+      <c r="A15" s="213" t="n"/>
       <c r="Z15" s="184" t="n"/>
       <c r="AA15" s="184" t="n"/>
       <c r="AB15" s="126" t="n"/>
@@ -19426,7 +21037,7 @@
       <c r="AM16" s="130" t="n"/>
     </row>
     <row r="17" ht="7.5" customHeight="1" s="127">
-      <c r="A17" s="212" t="n"/>
+      <c r="A17" s="213" t="n"/>
       <c r="Z17" s="184" t="n"/>
       <c r="AA17" s="184" t="n"/>
       <c r="AB17" s="126" t="n"/>
@@ -19464,7 +21075,7 @@
       <c r="AM18" s="130" t="n"/>
     </row>
     <row r="19" ht="7.5" customHeight="1" s="127">
-      <c r="A19" s="212" t="n"/>
+      <c r="A19" s="213" t="n"/>
       <c r="Z19" s="184" t="n"/>
       <c r="AA19" s="184" t="n"/>
       <c r="AB19" s="126" t="n"/>
@@ -19544,7 +21155,7 @@
       <c r="AN21" s="157" t="n"/>
     </row>
     <row r="22" ht="12.75" customHeight="1" s="127">
-      <c r="A22" s="213" t="inlineStr">
+      <c r="A22" s="214" t="inlineStr">
         <is>
           <t>Сумма исчисленного налога (авансового платежа по налогу):</t>
         </is>
@@ -19560,7 +21171,7 @@
       <c r="G23" s="157" t="n"/>
       <c r="H23" s="157" t="n"/>
       <c r="I23" s="157" t="n"/>
-      <c r="J23" s="214" t="n"/>
+      <c r="J23" s="215" t="n"/>
       <c r="K23" s="157" t="n"/>
       <c r="L23" s="157" t="n"/>
       <c r="M23" s="157" t="n"/>
@@ -19782,7 +21393,7 @@
       </c>
     </row>
     <row r="27" ht="4.15" customHeight="1" s="127">
-      <c r="A27" s="215" t="n"/>
+      <c r="A27" s="216" t="n"/>
       <c r="Z27" s="184" t="n"/>
       <c r="AA27" s="184" t="n"/>
       <c r="AB27" s="126" t="n"/>
@@ -19977,7 +21588,7 @@
       </c>
     </row>
     <row r="31" ht="4.15" customHeight="1" s="127">
-      <c r="A31" s="215" t="n"/>
+      <c r="A31" s="216" t="n"/>
       <c r="Z31" s="184" t="n"/>
       <c r="AA31" s="184" t="n"/>
       <c r="AB31" s="126" t="n"/>
@@ -20172,7 +21783,7 @@
       </c>
     </row>
     <row r="35" ht="4.15" customHeight="1" s="127">
-      <c r="A35" s="215" t="n"/>
+      <c r="A35" s="216" t="n"/>
       <c r="Z35" s="184" t="n"/>
       <c r="AA35" s="184" t="n"/>
       <c r="AB35" s="126" t="n"/>
@@ -20647,7 +22258,7 @@
       </c>
     </row>
     <row r="45" ht="4.15" customHeight="1" s="127">
-      <c r="A45" s="215" t="n"/>
+      <c r="A45" s="216" t="n"/>
       <c r="Z45" s="184" t="n"/>
       <c r="AA45" s="184" t="n"/>
       <c r="AB45" s="126" t="n"/>
@@ -20849,7 +22460,7 @@
       </c>
     </row>
     <row r="49" ht="4.15" customHeight="1" s="127">
-      <c r="A49" s="216" t="n"/>
+      <c r="A49" s="217" t="n"/>
       <c r="Z49" s="184" t="n"/>
       <c r="AA49" s="184" t="n"/>
       <c r="AB49" s="126" t="n"/>
@@ -21051,7 +22662,7 @@
       </c>
     </row>
     <row r="53" ht="4.15" customHeight="1" s="127">
-      <c r="A53" s="215" t="n"/>
+      <c r="A53" s="216" t="n"/>
       <c r="Z53" s="184" t="n"/>
       <c r="AA53" s="184" t="n"/>
       <c r="AB53" s="126" t="n"/>
@@ -21253,32 +22864,32 @@
       </c>
     </row>
     <row r="57" ht="24" customFormat="1" customHeight="1" s="184">
-      <c r="A57" s="217" t="n"/>
-      <c r="B57" s="217" t="n"/>
-      <c r="C57" s="217" t="n"/>
-      <c r="D57" s="217" t="n"/>
-      <c r="E57" s="217" t="n"/>
-      <c r="F57" s="217" t="n"/>
-      <c r="G57" s="217" t="n"/>
-      <c r="H57" s="217" t="n"/>
-      <c r="I57" s="217" t="n"/>
-      <c r="J57" s="217" t="n"/>
-      <c r="K57" s="217" t="n"/>
-      <c r="L57" s="217" t="n"/>
-      <c r="M57" s="217" t="n"/>
-      <c r="N57" s="217" t="n"/>
-      <c r="O57" s="217" t="n"/>
-      <c r="P57" s="217" t="n"/>
-      <c r="Q57" s="217" t="n"/>
-      <c r="R57" s="217" t="n"/>
-      <c r="S57" s="217" t="n"/>
-      <c r="T57" s="217" t="n"/>
-      <c r="U57" s="217" t="n"/>
-      <c r="V57" s="217" t="n"/>
-      <c r="W57" s="217" t="n"/>
-      <c r="X57" s="217" t="n"/>
-      <c r="Y57" s="217" t="n"/>
-      <c r="Z57" s="217" t="n"/>
+      <c r="A57" s="212" t="n"/>
+      <c r="B57" s="212" t="n"/>
+      <c r="C57" s="212" t="n"/>
+      <c r="D57" s="212" t="n"/>
+      <c r="E57" s="212" t="n"/>
+      <c r="F57" s="212" t="n"/>
+      <c r="G57" s="212" t="n"/>
+      <c r="H57" s="212" t="n"/>
+      <c r="I57" s="212" t="n"/>
+      <c r="J57" s="212" t="n"/>
+      <c r="K57" s="212" t="n"/>
+      <c r="L57" s="212" t="n"/>
+      <c r="M57" s="212" t="n"/>
+      <c r="N57" s="212" t="n"/>
+      <c r="O57" s="212" t="n"/>
+      <c r="P57" s="212" t="n"/>
+      <c r="Q57" s="212" t="n"/>
+      <c r="R57" s="212" t="n"/>
+      <c r="S57" s="212" t="n"/>
+      <c r="T57" s="212" t="n"/>
+      <c r="U57" s="212" t="n"/>
+      <c r="V57" s="212" t="n"/>
+      <c r="W57" s="212" t="n"/>
+      <c r="X57" s="212" t="n"/>
+      <c r="Y57" s="212" t="n"/>
+      <c r="Z57" s="212" t="n"/>
       <c r="AA57" s="184" t="n"/>
       <c r="AB57" s="184" t="n"/>
       <c r="AC57" s="184" t="n"/>
@@ -22928,132 +24539,132 @@
       </c>
     </row>
     <row r="34" ht="13.15" customFormat="1" customHeight="1" s="184">
-      <c r="A34" s="217" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="B34" s="217" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="C34" s="217" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="D34" s="217" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="E34" s="217" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="F34" s="217" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="G34" s="217" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="H34" s="217" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="I34" s="217" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="J34" s="217" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="K34" s="217" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="L34" s="217" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="M34" s="217" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="N34" s="217" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="O34" s="217" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="P34" s="217" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="Q34" s="217" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="R34" s="217" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="S34" s="217" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="T34" s="217" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="U34" s="217" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="V34" s="217" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="W34" s="217" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="X34" s="217" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="Y34" s="217" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="Z34" s="217" t="inlineStr">
+      <c r="A34" s="212" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="B34" s="212" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="C34" s="212" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="D34" s="212" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="E34" s="212" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="F34" s="212" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="G34" s="212" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="H34" s="212" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="I34" s="212" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="J34" s="212" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="K34" s="212" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="L34" s="212" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="M34" s="212" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="N34" s="212" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="O34" s="212" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="P34" s="212" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="Q34" s="212" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="R34" s="212" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="S34" s="212" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="T34" s="212" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="U34" s="212" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="V34" s="212" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="W34" s="212" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="X34" s="212" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="Y34" s="212" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="Z34" s="212" t="inlineStr">
         <is>
           <t xml:space="preserve"> </t>
         </is>
@@ -23130,32 +24741,32 @@
       </c>
     </row>
     <row r="35" ht="13.15" customFormat="1" customHeight="1" s="184">
-      <c r="A35" s="217" t="n"/>
-      <c r="B35" s="217" t="n"/>
-      <c r="C35" s="217" t="n"/>
-      <c r="D35" s="217" t="n"/>
-      <c r="E35" s="217" t="n"/>
-      <c r="F35" s="217" t="n"/>
-      <c r="G35" s="217" t="n"/>
-      <c r="H35" s="217" t="n"/>
-      <c r="I35" s="217" t="n"/>
-      <c r="J35" s="217" t="n"/>
-      <c r="K35" s="217" t="n"/>
-      <c r="L35" s="217" t="n"/>
-      <c r="M35" s="217" t="n"/>
-      <c r="N35" s="217" t="n"/>
-      <c r="O35" s="217" t="n"/>
-      <c r="P35" s="217" t="n"/>
-      <c r="Q35" s="217" t="n"/>
-      <c r="R35" s="217" t="n"/>
-      <c r="S35" s="217" t="n"/>
-      <c r="T35" s="217" t="n"/>
-      <c r="U35" s="217" t="n"/>
-      <c r="V35" s="217" t="n"/>
-      <c r="W35" s="217" t="n"/>
-      <c r="X35" s="217" t="n"/>
-      <c r="Y35" s="217" t="n"/>
-      <c r="Z35" s="217" t="n"/>
+      <c r="A35" s="212" t="n"/>
+      <c r="B35" s="212" t="n"/>
+      <c r="C35" s="212" t="n"/>
+      <c r="D35" s="212" t="n"/>
+      <c r="E35" s="212" t="n"/>
+      <c r="F35" s="212" t="n"/>
+      <c r="G35" s="212" t="n"/>
+      <c r="H35" s="212" t="n"/>
+      <c r="I35" s="212" t="n"/>
+      <c r="J35" s="212" t="n"/>
+      <c r="K35" s="212" t="n"/>
+      <c r="L35" s="212" t="n"/>
+      <c r="M35" s="212" t="n"/>
+      <c r="N35" s="212" t="n"/>
+      <c r="O35" s="212" t="n"/>
+      <c r="P35" s="212" t="n"/>
+      <c r="Q35" s="212" t="n"/>
+      <c r="R35" s="212" t="n"/>
+      <c r="S35" s="212" t="n"/>
+      <c r="T35" s="212" t="n"/>
+      <c r="U35" s="212" t="n"/>
+      <c r="V35" s="212" t="n"/>
+      <c r="W35" s="212" t="n"/>
+      <c r="X35" s="212" t="n"/>
+      <c r="Y35" s="212" t="n"/>
+      <c r="Z35" s="212" t="n"/>
       <c r="AA35" s="184" t="n"/>
       <c r="AB35" s="184" t="n"/>
       <c r="AC35" s="184" t="n"/>
@@ -23168,32 +24779,32 @@
       <c r="AJ35" s="184" t="n"/>
     </row>
     <row r="36" ht="13.15" customFormat="1" customHeight="1" s="184">
-      <c r="A36" s="217" t="n"/>
-      <c r="B36" s="217" t="n"/>
-      <c r="C36" s="217" t="n"/>
-      <c r="D36" s="217" t="n"/>
-      <c r="E36" s="217" t="n"/>
-      <c r="F36" s="217" t="n"/>
-      <c r="G36" s="217" t="n"/>
-      <c r="H36" s="217" t="n"/>
-      <c r="I36" s="217" t="n"/>
-      <c r="J36" s="217" t="n"/>
-      <c r="K36" s="217" t="n"/>
-      <c r="L36" s="217" t="n"/>
-      <c r="M36" s="217" t="n"/>
-      <c r="N36" s="217" t="n"/>
-      <c r="O36" s="217" t="n"/>
-      <c r="P36" s="217" t="n"/>
-      <c r="Q36" s="217" t="n"/>
-      <c r="R36" s="217" t="n"/>
-      <c r="S36" s="217" t="n"/>
-      <c r="T36" s="217" t="n"/>
-      <c r="U36" s="217" t="n"/>
-      <c r="V36" s="217" t="n"/>
-      <c r="W36" s="217" t="n"/>
-      <c r="X36" s="217" t="n"/>
-      <c r="Y36" s="217" t="n"/>
-      <c r="Z36" s="217" t="n"/>
+      <c r="A36" s="212" t="n"/>
+      <c r="B36" s="212" t="n"/>
+      <c r="C36" s="212" t="n"/>
+      <c r="D36" s="212" t="n"/>
+      <c r="E36" s="212" t="n"/>
+      <c r="F36" s="212" t="n"/>
+      <c r="G36" s="212" t="n"/>
+      <c r="H36" s="212" t="n"/>
+      <c r="I36" s="212" t="n"/>
+      <c r="J36" s="212" t="n"/>
+      <c r="K36" s="212" t="n"/>
+      <c r="L36" s="212" t="n"/>
+      <c r="M36" s="212" t="n"/>
+      <c r="N36" s="212" t="n"/>
+      <c r="O36" s="212" t="n"/>
+      <c r="P36" s="212" t="n"/>
+      <c r="Q36" s="212" t="n"/>
+      <c r="R36" s="212" t="n"/>
+      <c r="S36" s="212" t="n"/>
+      <c r="T36" s="212" t="n"/>
+      <c r="U36" s="212" t="n"/>
+      <c r="V36" s="212" t="n"/>
+      <c r="W36" s="212" t="n"/>
+      <c r="X36" s="212" t="n"/>
+      <c r="Y36" s="212" t="n"/>
+      <c r="Z36" s="212" t="n"/>
       <c r="AA36" s="184" t="n"/>
       <c r="AB36" s="184" t="n"/>
       <c r="AC36" s="184" t="n"/>
@@ -23206,32 +24817,32 @@
       <c r="AJ36" s="184" t="n"/>
     </row>
     <row r="37" ht="13.15" customFormat="1" customHeight="1" s="184">
-      <c r="A37" s="217" t="n"/>
-      <c r="B37" s="217" t="n"/>
-      <c r="C37" s="217" t="n"/>
-      <c r="D37" s="217" t="n"/>
-      <c r="E37" s="217" t="n"/>
-      <c r="F37" s="217" t="n"/>
-      <c r="G37" s="217" t="n"/>
-      <c r="H37" s="217" t="n"/>
-      <c r="I37" s="217" t="n"/>
-      <c r="J37" s="217" t="n"/>
-      <c r="K37" s="217" t="n"/>
-      <c r="L37" s="217" t="n"/>
-      <c r="M37" s="217" t="n"/>
-      <c r="N37" s="217" t="n"/>
-      <c r="O37" s="217" t="n"/>
-      <c r="P37" s="217" t="n"/>
-      <c r="Q37" s="217" t="n"/>
-      <c r="R37" s="217" t="n"/>
-      <c r="S37" s="217" t="n"/>
-      <c r="T37" s="217" t="n"/>
-      <c r="U37" s="217" t="n"/>
-      <c r="V37" s="217" t="n"/>
-      <c r="W37" s="217" t="n"/>
-      <c r="X37" s="217" t="n"/>
-      <c r="Y37" s="217" t="n"/>
-      <c r="Z37" s="217" t="n"/>
+      <c r="A37" s="212" t="n"/>
+      <c r="B37" s="212" t="n"/>
+      <c r="C37" s="212" t="n"/>
+      <c r="D37" s="212" t="n"/>
+      <c r="E37" s="212" t="n"/>
+      <c r="F37" s="212" t="n"/>
+      <c r="G37" s="212" t="n"/>
+      <c r="H37" s="212" t="n"/>
+      <c r="I37" s="212" t="n"/>
+      <c r="J37" s="212" t="n"/>
+      <c r="K37" s="212" t="n"/>
+      <c r="L37" s="212" t="n"/>
+      <c r="M37" s="212" t="n"/>
+      <c r="N37" s="212" t="n"/>
+      <c r="O37" s="212" t="n"/>
+      <c r="P37" s="212" t="n"/>
+      <c r="Q37" s="212" t="n"/>
+      <c r="R37" s="212" t="n"/>
+      <c r="S37" s="212" t="n"/>
+      <c r="T37" s="212" t="n"/>
+      <c r="U37" s="212" t="n"/>
+      <c r="V37" s="212" t="n"/>
+      <c r="W37" s="212" t="n"/>
+      <c r="X37" s="212" t="n"/>
+      <c r="Y37" s="212" t="n"/>
+      <c r="Z37" s="212" t="n"/>
       <c r="AA37" s="184" t="n"/>
       <c r="AB37" s="184" t="n"/>
       <c r="AC37" s="184" t="n"/>
@@ -23244,32 +24855,32 @@
       <c r="AJ37" s="184" t="n"/>
     </row>
     <row r="38" ht="13.15" customFormat="1" customHeight="1" s="184">
-      <c r="A38" s="217" t="n"/>
-      <c r="B38" s="217" t="n"/>
-      <c r="C38" s="217" t="n"/>
-      <c r="D38" s="217" t="n"/>
-      <c r="E38" s="217" t="n"/>
-      <c r="F38" s="217" t="n"/>
-      <c r="G38" s="217" t="n"/>
-      <c r="H38" s="217" t="n"/>
-      <c r="I38" s="217" t="n"/>
-      <c r="J38" s="217" t="n"/>
-      <c r="K38" s="217" t="n"/>
-      <c r="L38" s="217" t="n"/>
-      <c r="M38" s="217" t="n"/>
-      <c r="N38" s="217" t="n"/>
-      <c r="O38" s="217" t="n"/>
-      <c r="P38" s="217" t="n"/>
-      <c r="Q38" s="217" t="n"/>
-      <c r="R38" s="217" t="n"/>
-      <c r="S38" s="217" t="n"/>
-      <c r="T38" s="217" t="n"/>
-      <c r="U38" s="217" t="n"/>
-      <c r="V38" s="217" t="n"/>
-      <c r="W38" s="217" t="n"/>
-      <c r="X38" s="217" t="n"/>
-      <c r="Y38" s="217" t="n"/>
-      <c r="Z38" s="217" t="n"/>
+      <c r="A38" s="212" t="n"/>
+      <c r="B38" s="212" t="n"/>
+      <c r="C38" s="212" t="n"/>
+      <c r="D38" s="212" t="n"/>
+      <c r="E38" s="212" t="n"/>
+      <c r="F38" s="212" t="n"/>
+      <c r="G38" s="212" t="n"/>
+      <c r="H38" s="212" t="n"/>
+      <c r="I38" s="212" t="n"/>
+      <c r="J38" s="212" t="n"/>
+      <c r="K38" s="212" t="n"/>
+      <c r="L38" s="212" t="n"/>
+      <c r="M38" s="212" t="n"/>
+      <c r="N38" s="212" t="n"/>
+      <c r="O38" s="212" t="n"/>
+      <c r="P38" s="212" t="n"/>
+      <c r="Q38" s="212" t="n"/>
+      <c r="R38" s="212" t="n"/>
+      <c r="S38" s="212" t="n"/>
+      <c r="T38" s="212" t="n"/>
+      <c r="U38" s="212" t="n"/>
+      <c r="V38" s="212" t="n"/>
+      <c r="W38" s="212" t="n"/>
+      <c r="X38" s="212" t="n"/>
+      <c r="Y38" s="212" t="n"/>
+      <c r="Z38" s="212" t="n"/>
       <c r="AA38" s="184" t="n"/>
       <c r="AB38" s="184" t="n"/>
       <c r="AC38" s="184" t="n"/>
@@ -23282,32 +24893,32 @@
       <c r="AJ38" s="184" t="n"/>
     </row>
     <row r="39" ht="13.15" customFormat="1" customHeight="1" s="184">
-      <c r="A39" s="217" t="n"/>
-      <c r="B39" s="217" t="n"/>
-      <c r="C39" s="217" t="n"/>
-      <c r="D39" s="217" t="n"/>
-      <c r="E39" s="217" t="n"/>
-      <c r="F39" s="217" t="n"/>
-      <c r="G39" s="217" t="n"/>
-      <c r="H39" s="217" t="n"/>
-      <c r="I39" s="217" t="n"/>
-      <c r="J39" s="217" t="n"/>
-      <c r="K39" s="217" t="n"/>
-      <c r="L39" s="217" t="n"/>
-      <c r="M39" s="217" t="n"/>
-      <c r="N39" s="217" t="n"/>
-      <c r="O39" s="217" t="n"/>
-      <c r="P39" s="217" t="n"/>
-      <c r="Q39" s="217" t="n"/>
-      <c r="R39" s="217" t="n"/>
-      <c r="S39" s="217" t="n"/>
-      <c r="T39" s="217" t="n"/>
-      <c r="U39" s="217" t="n"/>
-      <c r="V39" s="217" t="n"/>
-      <c r="W39" s="217" t="n"/>
-      <c r="X39" s="217" t="n"/>
-      <c r="Y39" s="217" t="n"/>
-      <c r="Z39" s="217" t="n"/>
+      <c r="A39" s="212" t="n"/>
+      <c r="B39" s="212" t="n"/>
+      <c r="C39" s="212" t="n"/>
+      <c r="D39" s="212" t="n"/>
+      <c r="E39" s="212" t="n"/>
+      <c r="F39" s="212" t="n"/>
+      <c r="G39" s="212" t="n"/>
+      <c r="H39" s="212" t="n"/>
+      <c r="I39" s="212" t="n"/>
+      <c r="J39" s="212" t="n"/>
+      <c r="K39" s="212" t="n"/>
+      <c r="L39" s="212" t="n"/>
+      <c r="M39" s="212" t="n"/>
+      <c r="N39" s="212" t="n"/>
+      <c r="O39" s="212" t="n"/>
+      <c r="P39" s="212" t="n"/>
+      <c r="Q39" s="212" t="n"/>
+      <c r="R39" s="212" t="n"/>
+      <c r="S39" s="212" t="n"/>
+      <c r="T39" s="212" t="n"/>
+      <c r="U39" s="212" t="n"/>
+      <c r="V39" s="212" t="n"/>
+      <c r="W39" s="212" t="n"/>
+      <c r="X39" s="212" t="n"/>
+      <c r="Y39" s="212" t="n"/>
+      <c r="Z39" s="212" t="n"/>
       <c r="AA39" s="184" t="n"/>
       <c r="AB39" s="184" t="n"/>
       <c r="AC39" s="184" t="n"/>
@@ -23320,32 +24931,32 @@
       <c r="AJ39" s="184" t="n"/>
     </row>
     <row r="40" ht="13.15" customFormat="1" customHeight="1" s="184">
-      <c r="A40" s="217" t="n"/>
-      <c r="B40" s="217" t="n"/>
-      <c r="C40" s="217" t="n"/>
-      <c r="D40" s="217" t="n"/>
-      <c r="E40" s="217" t="n"/>
-      <c r="F40" s="217" t="n"/>
-      <c r="G40" s="217" t="n"/>
-      <c r="H40" s="217" t="n"/>
-      <c r="I40" s="217" t="n"/>
-      <c r="J40" s="217" t="n"/>
-      <c r="K40" s="217" t="n"/>
-      <c r="L40" s="217" t="n"/>
-      <c r="M40" s="217" t="n"/>
-      <c r="N40" s="217" t="n"/>
-      <c r="O40" s="217" t="n"/>
-      <c r="P40" s="217" t="n"/>
-      <c r="Q40" s="217" t="n"/>
-      <c r="R40" s="217" t="n"/>
-      <c r="S40" s="217" t="n"/>
-      <c r="T40" s="217" t="n"/>
-      <c r="U40" s="217" t="n"/>
-      <c r="V40" s="217" t="n"/>
-      <c r="W40" s="217" t="n"/>
-      <c r="X40" s="217" t="n"/>
-      <c r="Y40" s="217" t="n"/>
-      <c r="Z40" s="217" t="n"/>
+      <c r="A40" s="212" t="n"/>
+      <c r="B40" s="212" t="n"/>
+      <c r="C40" s="212" t="n"/>
+      <c r="D40" s="212" t="n"/>
+      <c r="E40" s="212" t="n"/>
+      <c r="F40" s="212" t="n"/>
+      <c r="G40" s="212" t="n"/>
+      <c r="H40" s="212" t="n"/>
+      <c r="I40" s="212" t="n"/>
+      <c r="J40" s="212" t="n"/>
+      <c r="K40" s="212" t="n"/>
+      <c r="L40" s="212" t="n"/>
+      <c r="M40" s="212" t="n"/>
+      <c r="N40" s="212" t="n"/>
+      <c r="O40" s="212" t="n"/>
+      <c r="P40" s="212" t="n"/>
+      <c r="Q40" s="212" t="n"/>
+      <c r="R40" s="212" t="n"/>
+      <c r="S40" s="212" t="n"/>
+      <c r="T40" s="212" t="n"/>
+      <c r="U40" s="212" t="n"/>
+      <c r="V40" s="212" t="n"/>
+      <c r="W40" s="212" t="n"/>
+      <c r="X40" s="212" t="n"/>
+      <c r="Y40" s="212" t="n"/>
+      <c r="Z40" s="212" t="n"/>
       <c r="AA40" s="184" t="n"/>
       <c r="AB40" s="184" t="n"/>
       <c r="AC40" s="184" t="n"/>
@@ -23358,32 +24969,32 @@
       <c r="AJ40" s="184" t="n"/>
     </row>
     <row r="41" ht="13.15" customFormat="1" customHeight="1" s="184">
-      <c r="A41" s="217" t="n"/>
-      <c r="B41" s="217" t="n"/>
-      <c r="C41" s="217" t="n"/>
-      <c r="D41" s="217" t="n"/>
-      <c r="E41" s="217" t="n"/>
-      <c r="F41" s="217" t="n"/>
-      <c r="G41" s="217" t="n"/>
-      <c r="H41" s="217" t="n"/>
-      <c r="I41" s="217" t="n"/>
-      <c r="J41" s="217" t="n"/>
-      <c r="K41" s="217" t="n"/>
-      <c r="L41" s="217" t="n"/>
-      <c r="M41" s="217" t="n"/>
-      <c r="N41" s="217" t="n"/>
-      <c r="O41" s="217" t="n"/>
-      <c r="P41" s="217" t="n"/>
-      <c r="Q41" s="217" t="n"/>
-      <c r="R41" s="217" t="n"/>
-      <c r="S41" s="217" t="n"/>
-      <c r="T41" s="217" t="n"/>
-      <c r="U41" s="217" t="n"/>
-      <c r="V41" s="217" t="n"/>
-      <c r="W41" s="217" t="n"/>
-      <c r="X41" s="217" t="n"/>
-      <c r="Y41" s="217" t="n"/>
-      <c r="Z41" s="217" t="n"/>
+      <c r="A41" s="212" t="n"/>
+      <c r="B41" s="212" t="n"/>
+      <c r="C41" s="212" t="n"/>
+      <c r="D41" s="212" t="n"/>
+      <c r="E41" s="212" t="n"/>
+      <c r="F41" s="212" t="n"/>
+      <c r="G41" s="212" t="n"/>
+      <c r="H41" s="212" t="n"/>
+      <c r="I41" s="212" t="n"/>
+      <c r="J41" s="212" t="n"/>
+      <c r="K41" s="212" t="n"/>
+      <c r="L41" s="212" t="n"/>
+      <c r="M41" s="212" t="n"/>
+      <c r="N41" s="212" t="n"/>
+      <c r="O41" s="212" t="n"/>
+      <c r="P41" s="212" t="n"/>
+      <c r="Q41" s="212" t="n"/>
+      <c r="R41" s="212" t="n"/>
+      <c r="S41" s="212" t="n"/>
+      <c r="T41" s="212" t="n"/>
+      <c r="U41" s="212" t="n"/>
+      <c r="V41" s="212" t="n"/>
+      <c r="W41" s="212" t="n"/>
+      <c r="X41" s="212" t="n"/>
+      <c r="Y41" s="212" t="n"/>
+      <c r="Z41" s="212" t="n"/>
       <c r="AA41" s="184" t="n"/>
       <c r="AB41" s="184" t="n"/>
       <c r="AC41" s="184" t="n"/>
@@ -23396,32 +25007,32 @@
       <c r="AJ41" s="184" t="n"/>
     </row>
     <row r="42" ht="13.15" customFormat="1" customHeight="1" s="184">
-      <c r="A42" s="217" t="n"/>
-      <c r="B42" s="217" t="n"/>
-      <c r="C42" s="217" t="n"/>
-      <c r="D42" s="217" t="n"/>
-      <c r="E42" s="217" t="n"/>
-      <c r="F42" s="217" t="n"/>
-      <c r="G42" s="217" t="n"/>
-      <c r="H42" s="217" t="n"/>
-      <c r="I42" s="217" t="n"/>
-      <c r="J42" s="217" t="n"/>
-      <c r="K42" s="217" t="n"/>
-      <c r="L42" s="217" t="n"/>
-      <c r="M42" s="217" t="n"/>
-      <c r="N42" s="217" t="n"/>
-      <c r="O42" s="217" t="n"/>
-      <c r="P42" s="217" t="n"/>
-      <c r="Q42" s="217" t="n"/>
-      <c r="R42" s="217" t="n"/>
-      <c r="S42" s="217" t="n"/>
-      <c r="T42" s="217" t="n"/>
-      <c r="U42" s="217" t="n"/>
-      <c r="V42" s="217" t="n"/>
-      <c r="W42" s="217" t="n"/>
-      <c r="X42" s="217" t="n"/>
-      <c r="Y42" s="217" t="n"/>
-      <c r="Z42" s="217" t="n"/>
+      <c r="A42" s="212" t="n"/>
+      <c r="B42" s="212" t="n"/>
+      <c r="C42" s="212" t="n"/>
+      <c r="D42" s="212" t="n"/>
+      <c r="E42" s="212" t="n"/>
+      <c r="F42" s="212" t="n"/>
+      <c r="G42" s="212" t="n"/>
+      <c r="H42" s="212" t="n"/>
+      <c r="I42" s="212" t="n"/>
+      <c r="J42" s="212" t="n"/>
+      <c r="K42" s="212" t="n"/>
+      <c r="L42" s="212" t="n"/>
+      <c r="M42" s="212" t="n"/>
+      <c r="N42" s="212" t="n"/>
+      <c r="O42" s="212" t="n"/>
+      <c r="P42" s="212" t="n"/>
+      <c r="Q42" s="212" t="n"/>
+      <c r="R42" s="212" t="n"/>
+      <c r="S42" s="212" t="n"/>
+      <c r="T42" s="212" t="n"/>
+      <c r="U42" s="212" t="n"/>
+      <c r="V42" s="212" t="n"/>
+      <c r="W42" s="212" t="n"/>
+      <c r="X42" s="212" t="n"/>
+      <c r="Y42" s="212" t="n"/>
+      <c r="Z42" s="212" t="n"/>
       <c r="AA42" s="184" t="n"/>
       <c r="AB42" s="184" t="n"/>
       <c r="AC42" s="184" t="n"/>
@@ -23434,32 +25045,32 @@
       <c r="AJ42" s="184" t="n"/>
     </row>
     <row r="43" ht="13.15" customFormat="1" customHeight="1" s="184">
-      <c r="A43" s="217" t="n"/>
-      <c r="B43" s="217" t="n"/>
-      <c r="C43" s="217" t="n"/>
-      <c r="D43" s="217" t="n"/>
-      <c r="E43" s="217" t="n"/>
-      <c r="F43" s="217" t="n"/>
-      <c r="G43" s="217" t="n"/>
-      <c r="H43" s="217" t="n"/>
-      <c r="I43" s="217" t="n"/>
-      <c r="J43" s="217" t="n"/>
-      <c r="K43" s="217" t="n"/>
-      <c r="L43" s="217" t="n"/>
-      <c r="M43" s="217" t="n"/>
-      <c r="N43" s="217" t="n"/>
-      <c r="O43" s="217" t="n"/>
-      <c r="P43" s="217" t="n"/>
-      <c r="Q43" s="217" t="n"/>
-      <c r="R43" s="217" t="n"/>
-      <c r="S43" s="217" t="n"/>
-      <c r="T43" s="217" t="n"/>
-      <c r="U43" s="217" t="n"/>
-      <c r="V43" s="217" t="n"/>
-      <c r="W43" s="217" t="n"/>
-      <c r="X43" s="217" t="n"/>
-      <c r="Y43" s="217" t="n"/>
-      <c r="Z43" s="217" t="n"/>
+      <c r="A43" s="212" t="n"/>
+      <c r="B43" s="212" t="n"/>
+      <c r="C43" s="212" t="n"/>
+      <c r="D43" s="212" t="n"/>
+      <c r="E43" s="212" t="n"/>
+      <c r="F43" s="212" t="n"/>
+      <c r="G43" s="212" t="n"/>
+      <c r="H43" s="212" t="n"/>
+      <c r="I43" s="212" t="n"/>
+      <c r="J43" s="212" t="n"/>
+      <c r="K43" s="212" t="n"/>
+      <c r="L43" s="212" t="n"/>
+      <c r="M43" s="212" t="n"/>
+      <c r="N43" s="212" t="n"/>
+      <c r="O43" s="212" t="n"/>
+      <c r="P43" s="212" t="n"/>
+      <c r="Q43" s="212" t="n"/>
+      <c r="R43" s="212" t="n"/>
+      <c r="S43" s="212" t="n"/>
+      <c r="T43" s="212" t="n"/>
+      <c r="U43" s="212" t="n"/>
+      <c r="V43" s="212" t="n"/>
+      <c r="W43" s="212" t="n"/>
+      <c r="X43" s="212" t="n"/>
+      <c r="Y43" s="212" t="n"/>
+      <c r="Z43" s="212" t="n"/>
       <c r="AA43" s="184" t="n"/>
       <c r="AB43" s="184" t="n"/>
       <c r="AC43" s="184" t="n"/>
@@ -23472,32 +25083,32 @@
       <c r="AJ43" s="184" t="n"/>
     </row>
     <row r="44" ht="13.15" customFormat="1" customHeight="1" s="184">
-      <c r="A44" s="217" t="n"/>
-      <c r="B44" s="217" t="n"/>
-      <c r="C44" s="217" t="n"/>
-      <c r="D44" s="217" t="n"/>
-      <c r="E44" s="217" t="n"/>
-      <c r="F44" s="217" t="n"/>
-      <c r="G44" s="217" t="n"/>
-      <c r="H44" s="217" t="n"/>
-      <c r="I44" s="217" t="n"/>
-      <c r="J44" s="217" t="n"/>
-      <c r="K44" s="217" t="n"/>
-      <c r="L44" s="217" t="n"/>
-      <c r="M44" s="217" t="n"/>
-      <c r="N44" s="217" t="n"/>
-      <c r="O44" s="217" t="n"/>
-      <c r="P44" s="217" t="n"/>
-      <c r="Q44" s="217" t="n"/>
-      <c r="R44" s="217" t="n"/>
-      <c r="S44" s="217" t="n"/>
-      <c r="T44" s="217" t="n"/>
-      <c r="U44" s="217" t="n"/>
-      <c r="V44" s="217" t="n"/>
-      <c r="W44" s="217" t="n"/>
-      <c r="X44" s="217" t="n"/>
-      <c r="Y44" s="217" t="n"/>
-      <c r="Z44" s="217" t="n"/>
+      <c r="A44" s="212" t="n"/>
+      <c r="B44" s="212" t="n"/>
+      <c r="C44" s="212" t="n"/>
+      <c r="D44" s="212" t="n"/>
+      <c r="E44" s="212" t="n"/>
+      <c r="F44" s="212" t="n"/>
+      <c r="G44" s="212" t="n"/>
+      <c r="H44" s="212" t="n"/>
+      <c r="I44" s="212" t="n"/>
+      <c r="J44" s="212" t="n"/>
+      <c r="K44" s="212" t="n"/>
+      <c r="L44" s="212" t="n"/>
+      <c r="M44" s="212" t="n"/>
+      <c r="N44" s="212" t="n"/>
+      <c r="O44" s="212" t="n"/>
+      <c r="P44" s="212" t="n"/>
+      <c r="Q44" s="212" t="n"/>
+      <c r="R44" s="212" t="n"/>
+      <c r="S44" s="212" t="n"/>
+      <c r="T44" s="212" t="n"/>
+      <c r="U44" s="212" t="n"/>
+      <c r="V44" s="212" t="n"/>
+      <c r="W44" s="212" t="n"/>
+      <c r="X44" s="212" t="n"/>
+      <c r="Y44" s="212" t="n"/>
+      <c r="Z44" s="212" t="n"/>
       <c r="AA44" s="184" t="n"/>
       <c r="AB44" s="184" t="n"/>
       <c r="AC44" s="184" t="n"/>
@@ -23510,32 +25121,32 @@
       <c r="AJ44" s="184" t="n"/>
     </row>
     <row r="45" ht="13.15" customFormat="1" customHeight="1" s="184">
-      <c r="A45" s="217" t="n"/>
-      <c r="B45" s="217" t="n"/>
-      <c r="C45" s="217" t="n"/>
-      <c r="D45" s="217" t="n"/>
-      <c r="E45" s="217" t="n"/>
-      <c r="F45" s="217" t="n"/>
-      <c r="G45" s="217" t="n"/>
-      <c r="H45" s="217" t="n"/>
-      <c r="I45" s="217" t="n"/>
-      <c r="J45" s="217" t="n"/>
-      <c r="K45" s="217" t="n"/>
-      <c r="L45" s="217" t="n"/>
-      <c r="M45" s="217" t="n"/>
-      <c r="N45" s="217" t="n"/>
-      <c r="O45" s="217" t="n"/>
-      <c r="P45" s="217" t="n"/>
-      <c r="Q45" s="217" t="n"/>
-      <c r="R45" s="217" t="n"/>
-      <c r="S45" s="217" t="n"/>
-      <c r="T45" s="217" t="n"/>
-      <c r="U45" s="217" t="n"/>
-      <c r="V45" s="217" t="n"/>
-      <c r="W45" s="217" t="n"/>
-      <c r="X45" s="217" t="n"/>
-      <c r="Y45" s="217" t="n"/>
-      <c r="Z45" s="217" t="n"/>
+      <c r="A45" s="212" t="n"/>
+      <c r="B45" s="212" t="n"/>
+      <c r="C45" s="212" t="n"/>
+      <c r="D45" s="212" t="n"/>
+      <c r="E45" s="212" t="n"/>
+      <c r="F45" s="212" t="n"/>
+      <c r="G45" s="212" t="n"/>
+      <c r="H45" s="212" t="n"/>
+      <c r="I45" s="212" t="n"/>
+      <c r="J45" s="212" t="n"/>
+      <c r="K45" s="212" t="n"/>
+      <c r="L45" s="212" t="n"/>
+      <c r="M45" s="212" t="n"/>
+      <c r="N45" s="212" t="n"/>
+      <c r="O45" s="212" t="n"/>
+      <c r="P45" s="212" t="n"/>
+      <c r="Q45" s="212" t="n"/>
+      <c r="R45" s="212" t="n"/>
+      <c r="S45" s="212" t="n"/>
+      <c r="T45" s="212" t="n"/>
+      <c r="U45" s="212" t="n"/>
+      <c r="V45" s="212" t="n"/>
+      <c r="W45" s="212" t="n"/>
+      <c r="X45" s="212" t="n"/>
+      <c r="Y45" s="212" t="n"/>
+      <c r="Z45" s="212" t="n"/>
       <c r="AA45" s="184" t="n"/>
       <c r="AB45" s="184" t="n"/>
       <c r="AC45" s="184" t="n"/>
@@ -23548,32 +25159,32 @@
       <c r="AJ45" s="184" t="n"/>
     </row>
     <row r="46" ht="13.15" customFormat="1" customHeight="1" s="184">
-      <c r="A46" s="217" t="n"/>
-      <c r="B46" s="217" t="n"/>
-      <c r="C46" s="217" t="n"/>
-      <c r="D46" s="217" t="n"/>
-      <c r="E46" s="217" t="n"/>
-      <c r="F46" s="217" t="n"/>
-      <c r="G46" s="217" t="n"/>
-      <c r="H46" s="217" t="n"/>
-      <c r="I46" s="217" t="n"/>
-      <c r="J46" s="217" t="n"/>
-      <c r="K46" s="217" t="n"/>
-      <c r="L46" s="217" t="n"/>
-      <c r="M46" s="217" t="n"/>
-      <c r="N46" s="217" t="n"/>
-      <c r="O46" s="217" t="n"/>
-      <c r="P46" s="217" t="n"/>
-      <c r="Q46" s="217" t="n"/>
-      <c r="R46" s="217" t="n"/>
-      <c r="S46" s="217" t="n"/>
-      <c r="T46" s="217" t="n"/>
-      <c r="U46" s="217" t="n"/>
-      <c r="V46" s="217" t="n"/>
-      <c r="W46" s="217" t="n"/>
-      <c r="X46" s="217" t="n"/>
-      <c r="Y46" s="217" t="n"/>
-      <c r="Z46" s="217" t="n"/>
+      <c r="A46" s="212" t="n"/>
+      <c r="B46" s="212" t="n"/>
+      <c r="C46" s="212" t="n"/>
+      <c r="D46" s="212" t="n"/>
+      <c r="E46" s="212" t="n"/>
+      <c r="F46" s="212" t="n"/>
+      <c r="G46" s="212" t="n"/>
+      <c r="H46" s="212" t="n"/>
+      <c r="I46" s="212" t="n"/>
+      <c r="J46" s="212" t="n"/>
+      <c r="K46" s="212" t="n"/>
+      <c r="L46" s="212" t="n"/>
+      <c r="M46" s="212" t="n"/>
+      <c r="N46" s="212" t="n"/>
+      <c r="O46" s="212" t="n"/>
+      <c r="P46" s="212" t="n"/>
+      <c r="Q46" s="212" t="n"/>
+      <c r="R46" s="212" t="n"/>
+      <c r="S46" s="212" t="n"/>
+      <c r="T46" s="212" t="n"/>
+      <c r="U46" s="212" t="n"/>
+      <c r="V46" s="212" t="n"/>
+      <c r="W46" s="212" t="n"/>
+      <c r="X46" s="212" t="n"/>
+      <c r="Y46" s="212" t="n"/>
+      <c r="Z46" s="212" t="n"/>
       <c r="AA46" s="184" t="n"/>
       <c r="AB46" s="184" t="n"/>
       <c r="AC46" s="184" t="n"/>
@@ -23586,32 +25197,32 @@
       <c r="AJ46" s="184" t="n"/>
     </row>
     <row r="47" ht="13.15" customFormat="1" customHeight="1" s="184">
-      <c r="A47" s="217" t="n"/>
-      <c r="B47" s="217" t="n"/>
-      <c r="C47" s="217" t="n"/>
-      <c r="D47" s="217" t="n"/>
-      <c r="E47" s="217" t="n"/>
-      <c r="F47" s="217" t="n"/>
-      <c r="G47" s="217" t="n"/>
-      <c r="H47" s="217" t="n"/>
-      <c r="I47" s="217" t="n"/>
-      <c r="J47" s="217" t="n"/>
-      <c r="K47" s="217" t="n"/>
-      <c r="L47" s="217" t="n"/>
-      <c r="M47" s="217" t="n"/>
-      <c r="N47" s="217" t="n"/>
-      <c r="O47" s="217" t="n"/>
-      <c r="P47" s="217" t="n"/>
-      <c r="Q47" s="217" t="n"/>
-      <c r="R47" s="217" t="n"/>
-      <c r="S47" s="217" t="n"/>
-      <c r="T47" s="217" t="n"/>
-      <c r="U47" s="217" t="n"/>
-      <c r="V47" s="217" t="n"/>
-      <c r="W47" s="217" t="n"/>
-      <c r="X47" s="217" t="n"/>
-      <c r="Y47" s="217" t="n"/>
-      <c r="Z47" s="217" t="n"/>
+      <c r="A47" s="212" t="n"/>
+      <c r="B47" s="212" t="n"/>
+      <c r="C47" s="212" t="n"/>
+      <c r="D47" s="212" t="n"/>
+      <c r="E47" s="212" t="n"/>
+      <c r="F47" s="212" t="n"/>
+      <c r="G47" s="212" t="n"/>
+      <c r="H47" s="212" t="n"/>
+      <c r="I47" s="212" t="n"/>
+      <c r="J47" s="212" t="n"/>
+      <c r="K47" s="212" t="n"/>
+      <c r="L47" s="212" t="n"/>
+      <c r="M47" s="212" t="n"/>
+      <c r="N47" s="212" t="n"/>
+      <c r="O47" s="212" t="n"/>
+      <c r="P47" s="212" t="n"/>
+      <c r="Q47" s="212" t="n"/>
+      <c r="R47" s="212" t="n"/>
+      <c r="S47" s="212" t="n"/>
+      <c r="T47" s="212" t="n"/>
+      <c r="U47" s="212" t="n"/>
+      <c r="V47" s="212" t="n"/>
+      <c r="W47" s="212" t="n"/>
+      <c r="X47" s="212" t="n"/>
+      <c r="Y47" s="212" t="n"/>
+      <c r="Z47" s="212" t="n"/>
       <c r="AA47" s="184" t="n"/>
       <c r="AB47" s="184" t="n"/>
       <c r="AC47" s="184" t="n"/>
@@ -23624,32 +25235,32 @@
       <c r="AJ47" s="184" t="n"/>
     </row>
     <row r="48" ht="13.15" customFormat="1" customHeight="1" s="184">
-      <c r="A48" s="217" t="n"/>
-      <c r="B48" s="217" t="n"/>
-      <c r="C48" s="217" t="n"/>
-      <c r="D48" s="217" t="n"/>
-      <c r="E48" s="217" t="n"/>
-      <c r="F48" s="217" t="n"/>
-      <c r="G48" s="217" t="n"/>
-      <c r="H48" s="217" t="n"/>
-      <c r="I48" s="217" t="n"/>
-      <c r="J48" s="217" t="n"/>
-      <c r="K48" s="217" t="n"/>
-      <c r="L48" s="217" t="n"/>
-      <c r="M48" s="217" t="n"/>
-      <c r="N48" s="217" t="n"/>
-      <c r="O48" s="217" t="n"/>
-      <c r="P48" s="217" t="n"/>
-      <c r="Q48" s="217" t="n"/>
-      <c r="R48" s="217" t="n"/>
-      <c r="S48" s="217" t="n"/>
-      <c r="T48" s="217" t="n"/>
-      <c r="U48" s="217" t="n"/>
-      <c r="V48" s="217" t="n"/>
-      <c r="W48" s="217" t="n"/>
-      <c r="X48" s="217" t="n"/>
-      <c r="Y48" s="217" t="n"/>
-      <c r="Z48" s="217" t="n"/>
+      <c r="A48" s="212" t="n"/>
+      <c r="B48" s="212" t="n"/>
+      <c r="C48" s="212" t="n"/>
+      <c r="D48" s="212" t="n"/>
+      <c r="E48" s="212" t="n"/>
+      <c r="F48" s="212" t="n"/>
+      <c r="G48" s="212" t="n"/>
+      <c r="H48" s="212" t="n"/>
+      <c r="I48" s="212" t="n"/>
+      <c r="J48" s="212" t="n"/>
+      <c r="K48" s="212" t="n"/>
+      <c r="L48" s="212" t="n"/>
+      <c r="M48" s="212" t="n"/>
+      <c r="N48" s="212" t="n"/>
+      <c r="O48" s="212" t="n"/>
+      <c r="P48" s="212" t="n"/>
+      <c r="Q48" s="212" t="n"/>
+      <c r="R48" s="212" t="n"/>
+      <c r="S48" s="212" t="n"/>
+      <c r="T48" s="212" t="n"/>
+      <c r="U48" s="212" t="n"/>
+      <c r="V48" s="212" t="n"/>
+      <c r="W48" s="212" t="n"/>
+      <c r="X48" s="212" t="n"/>
+      <c r="Y48" s="212" t="n"/>
+      <c r="Z48" s="212" t="n"/>
       <c r="AA48" s="184" t="n"/>
       <c r="AB48" s="184" t="n"/>
       <c r="AC48" s="184" t="n"/>
@@ -23662,32 +25273,32 @@
       <c r="AJ48" s="184" t="n"/>
     </row>
     <row r="49" ht="13.15" customFormat="1" customHeight="1" s="184">
-      <c r="A49" s="217" t="n"/>
-      <c r="B49" s="217" t="n"/>
-      <c r="C49" s="217" t="n"/>
-      <c r="D49" s="217" t="n"/>
-      <c r="E49" s="217" t="n"/>
-      <c r="F49" s="217" t="n"/>
-      <c r="G49" s="217" t="n"/>
-      <c r="H49" s="217" t="n"/>
-      <c r="I49" s="217" t="n"/>
-      <c r="J49" s="217" t="n"/>
-      <c r="K49" s="217" t="n"/>
-      <c r="L49" s="217" t="n"/>
-      <c r="M49" s="217" t="n"/>
-      <c r="N49" s="217" t="n"/>
-      <c r="O49" s="217" t="n"/>
-      <c r="P49" s="217" t="n"/>
-      <c r="Q49" s="217" t="n"/>
-      <c r="R49" s="217" t="n"/>
-      <c r="S49" s="217" t="n"/>
-      <c r="T49" s="217" t="n"/>
-      <c r="U49" s="217" t="n"/>
-      <c r="V49" s="217" t="n"/>
-      <c r="W49" s="217" t="n"/>
-      <c r="X49" s="217" t="n"/>
-      <c r="Y49" s="217" t="n"/>
-      <c r="Z49" s="217" t="n"/>
+      <c r="A49" s="212" t="n"/>
+      <c r="B49" s="212" t="n"/>
+      <c r="C49" s="212" t="n"/>
+      <c r="D49" s="212" t="n"/>
+      <c r="E49" s="212" t="n"/>
+      <c r="F49" s="212" t="n"/>
+      <c r="G49" s="212" t="n"/>
+      <c r="H49" s="212" t="n"/>
+      <c r="I49" s="212" t="n"/>
+      <c r="J49" s="212" t="n"/>
+      <c r="K49" s="212" t="n"/>
+      <c r="L49" s="212" t="n"/>
+      <c r="M49" s="212" t="n"/>
+      <c r="N49" s="212" t="n"/>
+      <c r="O49" s="212" t="n"/>
+      <c r="P49" s="212" t="n"/>
+      <c r="Q49" s="212" t="n"/>
+      <c r="R49" s="212" t="n"/>
+      <c r="S49" s="212" t="n"/>
+      <c r="T49" s="212" t="n"/>
+      <c r="U49" s="212" t="n"/>
+      <c r="V49" s="212" t="n"/>
+      <c r="W49" s="212" t="n"/>
+      <c r="X49" s="212" t="n"/>
+      <c r="Y49" s="212" t="n"/>
+      <c r="Z49" s="212" t="n"/>
       <c r="AA49" s="184" t="n"/>
       <c r="AB49" s="184" t="n"/>
       <c r="AC49" s="184" t="n"/>
@@ -23700,32 +25311,32 @@
       <c r="AJ49" s="184" t="n"/>
     </row>
     <row r="50" ht="13.15" customFormat="1" customHeight="1" s="184">
-      <c r="A50" s="217" t="n"/>
-      <c r="B50" s="217" t="n"/>
-      <c r="C50" s="217" t="n"/>
-      <c r="D50" s="217" t="n"/>
-      <c r="E50" s="217" t="n"/>
-      <c r="F50" s="217" t="n"/>
-      <c r="G50" s="217" t="n"/>
-      <c r="H50" s="217" t="n"/>
-      <c r="I50" s="217" t="n"/>
-      <c r="J50" s="217" t="n"/>
-      <c r="K50" s="217" t="n"/>
-      <c r="L50" s="217" t="n"/>
-      <c r="M50" s="217" t="n"/>
-      <c r="N50" s="217" t="n"/>
-      <c r="O50" s="217" t="n"/>
-      <c r="P50" s="217" t="n"/>
-      <c r="Q50" s="217" t="n"/>
-      <c r="R50" s="217" t="n"/>
-      <c r="S50" s="217" t="n"/>
-      <c r="T50" s="217" t="n"/>
-      <c r="U50" s="217" t="n"/>
-      <c r="V50" s="217" t="n"/>
-      <c r="W50" s="217" t="n"/>
-      <c r="X50" s="217" t="n"/>
-      <c r="Y50" s="217" t="n"/>
-      <c r="Z50" s="217" t="n"/>
+      <c r="A50" s="212" t="n"/>
+      <c r="B50" s="212" t="n"/>
+      <c r="C50" s="212" t="n"/>
+      <c r="D50" s="212" t="n"/>
+      <c r="E50" s="212" t="n"/>
+      <c r="F50" s="212" t="n"/>
+      <c r="G50" s="212" t="n"/>
+      <c r="H50" s="212" t="n"/>
+      <c r="I50" s="212" t="n"/>
+      <c r="J50" s="212" t="n"/>
+      <c r="K50" s="212" t="n"/>
+      <c r="L50" s="212" t="n"/>
+      <c r="M50" s="212" t="n"/>
+      <c r="N50" s="212" t="n"/>
+      <c r="O50" s="212" t="n"/>
+      <c r="P50" s="212" t="n"/>
+      <c r="Q50" s="212" t="n"/>
+      <c r="R50" s="212" t="n"/>
+      <c r="S50" s="212" t="n"/>
+      <c r="T50" s="212" t="n"/>
+      <c r="U50" s="212" t="n"/>
+      <c r="V50" s="212" t="n"/>
+      <c r="W50" s="212" t="n"/>
+      <c r="X50" s="212" t="n"/>
+      <c r="Y50" s="212" t="n"/>
+      <c r="Z50" s="212" t="n"/>
       <c r="AA50" s="184" t="n"/>
       <c r="AB50" s="184" t="n"/>
       <c r="AC50" s="184" t="n"/>
@@ -23738,32 +25349,32 @@
       <c r="AJ50" s="184" t="n"/>
     </row>
     <row r="51" ht="13.15" customFormat="1" customHeight="1" s="184">
-      <c r="A51" s="217" t="n"/>
-      <c r="B51" s="217" t="n"/>
-      <c r="C51" s="217" t="n"/>
-      <c r="D51" s="217" t="n"/>
-      <c r="E51" s="217" t="n"/>
-      <c r="F51" s="217" t="n"/>
-      <c r="G51" s="217" t="n"/>
-      <c r="H51" s="217" t="n"/>
-      <c r="I51" s="217" t="n"/>
-      <c r="J51" s="217" t="n"/>
-      <c r="K51" s="217" t="n"/>
-      <c r="L51" s="217" t="n"/>
-      <c r="M51" s="217" t="n"/>
-      <c r="N51" s="217" t="n"/>
-      <c r="O51" s="217" t="n"/>
-      <c r="P51" s="217" t="n"/>
-      <c r="Q51" s="217" t="n"/>
-      <c r="R51" s="217" t="n"/>
-      <c r="S51" s="217" t="n"/>
-      <c r="T51" s="217" t="n"/>
-      <c r="U51" s="217" t="n"/>
-      <c r="V51" s="217" t="n"/>
-      <c r="W51" s="217" t="n"/>
-      <c r="X51" s="217" t="n"/>
-      <c r="Y51" s="217" t="n"/>
-      <c r="Z51" s="217" t="n"/>
+      <c r="A51" s="212" t="n"/>
+      <c r="B51" s="212" t="n"/>
+      <c r="C51" s="212" t="n"/>
+      <c r="D51" s="212" t="n"/>
+      <c r="E51" s="212" t="n"/>
+      <c r="F51" s="212" t="n"/>
+      <c r="G51" s="212" t="n"/>
+      <c r="H51" s="212" t="n"/>
+      <c r="I51" s="212" t="n"/>
+      <c r="J51" s="212" t="n"/>
+      <c r="K51" s="212" t="n"/>
+      <c r="L51" s="212" t="n"/>
+      <c r="M51" s="212" t="n"/>
+      <c r="N51" s="212" t="n"/>
+      <c r="O51" s="212" t="n"/>
+      <c r="P51" s="212" t="n"/>
+      <c r="Q51" s="212" t="n"/>
+      <c r="R51" s="212" t="n"/>
+      <c r="S51" s="212" t="n"/>
+      <c r="T51" s="212" t="n"/>
+      <c r="U51" s="212" t="n"/>
+      <c r="V51" s="212" t="n"/>
+      <c r="W51" s="212" t="n"/>
+      <c r="X51" s="212" t="n"/>
+      <c r="Y51" s="212" t="n"/>
+      <c r="Z51" s="212" t="n"/>
       <c r="AA51" s="184" t="n"/>
       <c r="AB51" s="184" t="n"/>
       <c r="AC51" s="184" t="n"/>
@@ -23776,32 +25387,32 @@
       <c r="AJ51" s="184" t="n"/>
     </row>
     <row r="52" ht="13.15" customFormat="1" customHeight="1" s="184">
-      <c r="A52" s="217" t="n"/>
-      <c r="B52" s="217" t="n"/>
-      <c r="C52" s="217" t="n"/>
-      <c r="D52" s="217" t="n"/>
-      <c r="E52" s="217" t="n"/>
-      <c r="F52" s="217" t="n"/>
-      <c r="G52" s="217" t="n"/>
-      <c r="H52" s="217" t="n"/>
-      <c r="I52" s="217" t="n"/>
-      <c r="J52" s="217" t="n"/>
-      <c r="K52" s="217" t="n"/>
-      <c r="L52" s="217" t="n"/>
-      <c r="M52" s="217" t="n"/>
-      <c r="N52" s="217" t="n"/>
-      <c r="O52" s="217" t="n"/>
-      <c r="P52" s="217" t="n"/>
-      <c r="Q52" s="217" t="n"/>
-      <c r="R52" s="217" t="n"/>
-      <c r="S52" s="217" t="n"/>
-      <c r="T52" s="217" t="n"/>
-      <c r="U52" s="217" t="n"/>
-      <c r="V52" s="217" t="n"/>
-      <c r="W52" s="217" t="n"/>
-      <c r="X52" s="217" t="n"/>
-      <c r="Y52" s="217" t="n"/>
-      <c r="Z52" s="217" t="n"/>
+      <c r="A52" s="212" t="n"/>
+      <c r="B52" s="212" t="n"/>
+      <c r="C52" s="212" t="n"/>
+      <c r="D52" s="212" t="n"/>
+      <c r="E52" s="212" t="n"/>
+      <c r="F52" s="212" t="n"/>
+      <c r="G52" s="212" t="n"/>
+      <c r="H52" s="212" t="n"/>
+      <c r="I52" s="212" t="n"/>
+      <c r="J52" s="212" t="n"/>
+      <c r="K52" s="212" t="n"/>
+      <c r="L52" s="212" t="n"/>
+      <c r="M52" s="212" t="n"/>
+      <c r="N52" s="212" t="n"/>
+      <c r="O52" s="212" t="n"/>
+      <c r="P52" s="212" t="n"/>
+      <c r="Q52" s="212" t="n"/>
+      <c r="R52" s="212" t="n"/>
+      <c r="S52" s="212" t="n"/>
+      <c r="T52" s="212" t="n"/>
+      <c r="U52" s="212" t="n"/>
+      <c r="V52" s="212" t="n"/>
+      <c r="W52" s="212" t="n"/>
+      <c r="X52" s="212" t="n"/>
+      <c r="Y52" s="212" t="n"/>
+      <c r="Z52" s="212" t="n"/>
       <c r="AA52" s="184" t="n"/>
       <c r="AB52" s="184" t="n"/>
       <c r="AC52" s="184" t="n"/>
@@ -23814,32 +25425,32 @@
       <c r="AJ52" s="184" t="n"/>
     </row>
     <row r="53" ht="13.15" customFormat="1" customHeight="1" s="184">
-      <c r="A53" s="217" t="n"/>
-      <c r="B53" s="217" t="n"/>
-      <c r="C53" s="217" t="n"/>
-      <c r="D53" s="217" t="n"/>
-      <c r="E53" s="217" t="n"/>
-      <c r="F53" s="217" t="n"/>
-      <c r="G53" s="217" t="n"/>
-      <c r="H53" s="217" t="n"/>
-      <c r="I53" s="217" t="n"/>
-      <c r="J53" s="217" t="n"/>
-      <c r="K53" s="217" t="n"/>
-      <c r="L53" s="217" t="n"/>
-      <c r="M53" s="217" t="n"/>
-      <c r="N53" s="217" t="n"/>
-      <c r="O53" s="217" t="n"/>
-      <c r="P53" s="217" t="n"/>
-      <c r="Q53" s="217" t="n"/>
-      <c r="R53" s="217" t="n"/>
-      <c r="S53" s="217" t="n"/>
-      <c r="T53" s="217" t="n"/>
-      <c r="U53" s="217" t="n"/>
-      <c r="V53" s="217" t="n"/>
-      <c r="W53" s="217" t="n"/>
-      <c r="X53" s="217" t="n"/>
-      <c r="Y53" s="217" t="n"/>
-      <c r="Z53" s="217" t="n"/>
+      <c r="A53" s="212" t="n"/>
+      <c r="B53" s="212" t="n"/>
+      <c r="C53" s="212" t="n"/>
+      <c r="D53" s="212" t="n"/>
+      <c r="E53" s="212" t="n"/>
+      <c r="F53" s="212" t="n"/>
+      <c r="G53" s="212" t="n"/>
+      <c r="H53" s="212" t="n"/>
+      <c r="I53" s="212" t="n"/>
+      <c r="J53" s="212" t="n"/>
+      <c r="K53" s="212" t="n"/>
+      <c r="L53" s="212" t="n"/>
+      <c r="M53" s="212" t="n"/>
+      <c r="N53" s="212" t="n"/>
+      <c r="O53" s="212" t="n"/>
+      <c r="P53" s="212" t="n"/>
+      <c r="Q53" s="212" t="n"/>
+      <c r="R53" s="212" t="n"/>
+      <c r="S53" s="212" t="n"/>
+      <c r="T53" s="212" t="n"/>
+      <c r="U53" s="212" t="n"/>
+      <c r="V53" s="212" t="n"/>
+      <c r="W53" s="212" t="n"/>
+      <c r="X53" s="212" t="n"/>
+      <c r="Y53" s="212" t="n"/>
+      <c r="Z53" s="212" t="n"/>
       <c r="AA53" s="184" t="n"/>
       <c r="AB53" s="184" t="n"/>
       <c r="AC53" s="184" t="n"/>
@@ -23852,32 +25463,32 @@
       <c r="AJ53" s="184" t="n"/>
     </row>
     <row r="54" ht="13.5" customFormat="1" customHeight="1" s="184">
-      <c r="A54" s="217" t="n"/>
-      <c r="B54" s="217" t="n"/>
-      <c r="C54" s="217" t="n"/>
-      <c r="D54" s="217" t="n"/>
-      <c r="E54" s="217" t="n"/>
-      <c r="F54" s="217" t="n"/>
-      <c r="G54" s="217" t="n"/>
-      <c r="H54" s="217" t="n"/>
-      <c r="I54" s="217" t="n"/>
-      <c r="J54" s="217" t="n"/>
-      <c r="K54" s="217" t="n"/>
-      <c r="L54" s="217" t="n"/>
-      <c r="M54" s="217" t="n"/>
-      <c r="N54" s="217" t="n"/>
-      <c r="O54" s="217" t="n"/>
-      <c r="P54" s="217" t="n"/>
-      <c r="Q54" s="217" t="n"/>
-      <c r="R54" s="217" t="n"/>
-      <c r="S54" s="217" t="n"/>
-      <c r="T54" s="217" t="n"/>
-      <c r="U54" s="217" t="n"/>
-      <c r="V54" s="217" t="n"/>
-      <c r="W54" s="217" t="n"/>
-      <c r="X54" s="217" t="n"/>
-      <c r="Y54" s="217" t="n"/>
-      <c r="Z54" s="217" t="n"/>
+      <c r="A54" s="212" t="n"/>
+      <c r="B54" s="212" t="n"/>
+      <c r="C54" s="212" t="n"/>
+      <c r="D54" s="212" t="n"/>
+      <c r="E54" s="212" t="n"/>
+      <c r="F54" s="212" t="n"/>
+      <c r="G54" s="212" t="n"/>
+      <c r="H54" s="212" t="n"/>
+      <c r="I54" s="212" t="n"/>
+      <c r="J54" s="212" t="n"/>
+      <c r="K54" s="212" t="n"/>
+      <c r="L54" s="212" t="n"/>
+      <c r="M54" s="212" t="n"/>
+      <c r="N54" s="212" t="n"/>
+      <c r="O54" s="212" t="n"/>
+      <c r="P54" s="212" t="n"/>
+      <c r="Q54" s="212" t="n"/>
+      <c r="R54" s="212" t="n"/>
+      <c r="S54" s="212" t="n"/>
+      <c r="T54" s="212" t="n"/>
+      <c r="U54" s="212" t="n"/>
+      <c r="V54" s="212" t="n"/>
+      <c r="W54" s="212" t="n"/>
+      <c r="X54" s="212" t="n"/>
+      <c r="Y54" s="212" t="n"/>
+      <c r="Z54" s="212" t="n"/>
       <c r="AA54" s="184" t="n"/>
       <c r="AB54" s="184" t="n"/>
       <c r="AC54" s="184" t="n"/>
@@ -27998,32 +29609,32 @@
       </c>
     </row>
     <row r="27" ht="20.25" customFormat="1" customHeight="1" s="184">
-      <c r="A27" s="217" t="n"/>
-      <c r="B27" s="217" t="n"/>
-      <c r="C27" s="217" t="n"/>
-      <c r="D27" s="217" t="n"/>
-      <c r="E27" s="217" t="n"/>
-      <c r="F27" s="217" t="n"/>
-      <c r="G27" s="217" t="n"/>
-      <c r="H27" s="217" t="n"/>
-      <c r="I27" s="217" t="n"/>
-      <c r="J27" s="217" t="n"/>
-      <c r="K27" s="217" t="n"/>
-      <c r="L27" s="217" t="n"/>
-      <c r="M27" s="217" t="n"/>
-      <c r="N27" s="217" t="n"/>
-      <c r="O27" s="217" t="n"/>
-      <c r="P27" s="217" t="n"/>
-      <c r="Q27" s="217" t="n"/>
-      <c r="R27" s="217" t="n"/>
-      <c r="S27" s="217" t="n"/>
-      <c r="T27" s="217" t="n"/>
-      <c r="U27" s="217" t="n"/>
-      <c r="V27" s="217" t="n"/>
-      <c r="W27" s="217" t="n"/>
-      <c r="X27" s="217" t="n"/>
-      <c r="Y27" s="217" t="n"/>
-      <c r="Z27" s="217" t="n"/>
+      <c r="A27" s="212" t="n"/>
+      <c r="B27" s="212" t="n"/>
+      <c r="C27" s="212" t="n"/>
+      <c r="D27" s="212" t="n"/>
+      <c r="E27" s="212" t="n"/>
+      <c r="F27" s="212" t="n"/>
+      <c r="G27" s="212" t="n"/>
+      <c r="H27" s="212" t="n"/>
+      <c r="I27" s="212" t="n"/>
+      <c r="J27" s="212" t="n"/>
+      <c r="K27" s="212" t="n"/>
+      <c r="L27" s="212" t="n"/>
+      <c r="M27" s="212" t="n"/>
+      <c r="N27" s="212" t="n"/>
+      <c r="O27" s="212" t="n"/>
+      <c r="P27" s="212" t="n"/>
+      <c r="Q27" s="212" t="n"/>
+      <c r="R27" s="212" t="n"/>
+      <c r="S27" s="212" t="n"/>
+      <c r="T27" s="212" t="n"/>
+      <c r="U27" s="212" t="n"/>
+      <c r="V27" s="212" t="n"/>
+      <c r="W27" s="212" t="n"/>
+      <c r="X27" s="212" t="n"/>
+      <c r="Y27" s="212" t="n"/>
+      <c r="Z27" s="212" t="n"/>
       <c r="AA27" s="184" t="n"/>
       <c r="AB27" s="184" t="n"/>
       <c r="AC27" s="184" t="n"/>

</xml_diff>

<commit_message>
fix(pr30): align markers + uppercase FIO + prune unused sheets
ШАБЛОНЫ v13:
- Метки в самой последней строке xls (deficit-row кладётся ПЕРЕД меткой)
- Все 11 листов обработаны (Титульный, Р.1.1, Р.1.2, Р.2.1.1, Р.2.1.1 продол.,
  Р.2.1.2, Р.2.1.2 продол., Р.2.2, Р.2.2 продол., Р.3, Р.4)
- Page margins эталонные: top=0.55″ (40pt), bottom=1.69″ (122pt), L/R=0.625″ (45pt)
- Все листы выровнены на ~837pt физической высоты

Прогноз позиции меток: при scale=0.81 (avail/total) метки лягут на y=720pt,
что соответствует эталону Тензора (Романов).

КОД:
- ФИО приводится к UPPERCASE при заполнении (требование ФНС)
- Добавлена функция prune_unused_sheets(wb, object_code):
  - Для УСН Доходы (object_code='1'): оставляет только Титульный, Р.1.1,
    Р.2.1.1, Р.2.1.1 (продол.). Все остальные удаляются перед PDF.
  - Для УСН Доходы-Расходы (object_code='2'): Титульный, Р.1.2, Р.2.2,
    Р.2.2 (продол.).
- prune_unused_sheets вызывается в fill_declaration перед return wb.
</commit_message>
<xml_diff>
--- a/modules/usn_declaration/data/declaration_template_2024.xlsx
+++ b/modules/usn_declaration/data/declaration_template_2024.xlsx
@@ -4486,7 +4486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AN64"/>
+  <dimension ref="A1:AN65"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.13671875" defaultRowHeight="12.75" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="2.56" customWidth="1" style="126" min="1" max="12"/>
@@ -6622,7 +6622,7 @@
         </is>
       </c>
     </row>
-    <row r="63" ht="12.75" customHeight="1" s="127">
+    <row r="63" ht="0.5" customHeight="1" s="127">
       <c r="L63" s="126" t="n"/>
       <c r="M63" s="126" t="n"/>
       <c r="N63" s="126" t="n"/>
@@ -6649,19 +6649,19 @@
       <c r="AI63" s="126" t="n"/>
       <c r="AJ63" s="126" t="n"/>
     </row>
-    <row r="64" ht="13.5" customHeight="1" s="127">
-      <c r="A64" s="128" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="AN64" s="128" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-    </row>
-    <row r="65" ht="17.25" customHeight="1" s="127"/>
+    <row r="64" ht="7.300000000000409" customHeight="1" s="127"/>
+    <row r="65" ht="17.25" customHeight="1" s="127">
+      <c r="A65" s="128" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="AN65" s="128" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+    </row>
     <row r="66" ht="17.25" customHeight="1" s="127"/>
     <row r="135" ht="17.25" customHeight="1" s="127"/>
     <row r="136" ht="17.25" customHeight="1" s="127"/>
@@ -6877,7 +6877,7 @@
     <mergeCell ref="R1:R2"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.196527777777778" right="0.196527777777778" top="0.196527777777778" bottom="0.196527777777778" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageMargins left="0.625" right="0.625" top="0.55" bottom="1.69" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" cellComments="atEnd" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
@@ -9903,7 +9903,7 @@
         </is>
       </c>
     </row>
-    <row r="65" ht="3.75" customHeight="1" s="127">
+    <row r="65" ht="0.5" customHeight="1" s="127">
       <c r="L65" s="126" t="n"/>
       <c r="M65" s="126" t="n"/>
       <c r="N65" s="126" t="n"/>
@@ -10193,7 +10193,7 @@
     <mergeCell ref="A22:R23"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.196527777777778" right="0.196527777777778" top="0.196527777777778" bottom="0.196527777777778" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageMargins left="0.625" right="0.625" top="0.55" bottom="1.69" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" cellComments="atEnd" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
@@ -11954,7 +11954,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AN110"/>
+  <dimension ref="A1:AN53"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.13671875" defaultRowHeight="12.75" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="2.56" customWidth="1" style="126" min="1" max="12"/>
@@ -13374,7 +13374,7 @@
       <c r="AM51" s="134" t="n"/>
       <c r="AN51" s="134" t="n"/>
     </row>
-    <row r="52" ht="2.25" customHeight="1" s="127"/>
+    <row r="52" ht="0.5" customHeight="1" s="127"/>
     <row r="53" ht="13.5" customHeight="1" s="127">
       <c r="A53" s="128" t="inlineStr">
         <is>
@@ -13387,1545 +13387,63 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="12.75" customHeight="1" s="127">
-      <c r="A54" s="181" t="n"/>
-      <c r="B54" s="181" t="n"/>
-      <c r="C54" s="181" t="n"/>
-      <c r="D54" s="181" t="n"/>
-      <c r="E54" s="181" t="n"/>
-      <c r="F54" s="181" t="n"/>
-      <c r="G54" s="181" t="n"/>
-      <c r="H54" s="181" t="n"/>
-      <c r="I54" s="181" t="n"/>
-      <c r="J54" s="181" t="n"/>
-      <c r="K54" s="181" t="n"/>
-      <c r="L54" s="181" t="n"/>
-      <c r="M54" s="181" t="n"/>
-      <c r="N54" s="181" t="n"/>
-      <c r="O54" s="181" t="n"/>
-      <c r="P54" s="181" t="n"/>
-      <c r="Q54" s="181" t="n"/>
-      <c r="R54" s="181" t="n"/>
-      <c r="S54" s="181" t="n"/>
-      <c r="T54" s="181" t="n"/>
-      <c r="U54" s="181" t="n"/>
-      <c r="V54" s="181" t="n"/>
-      <c r="W54" s="181" t="n"/>
-      <c r="X54" s="181" t="n"/>
-      <c r="Y54" s="181" t="n"/>
-    </row>
-    <row r="55" ht="12.75" customHeight="1" s="127">
-      <c r="A55" s="181" t="n"/>
-      <c r="B55" s="181" t="n"/>
-      <c r="C55" s="181" t="n"/>
-      <c r="D55" s="181" t="n"/>
-      <c r="E55" s="181" t="n"/>
-      <c r="F55" s="181" t="n"/>
-      <c r="G55" s="181" t="n"/>
-      <c r="H55" s="181" t="n"/>
-      <c r="I55" s="181" t="n"/>
-      <c r="J55" s="181" t="n"/>
-      <c r="K55" s="181" t="n"/>
-      <c r="L55" s="181" t="n"/>
-      <c r="M55" s="181" t="n"/>
-      <c r="N55" s="181" t="n"/>
-      <c r="O55" s="181" t="n"/>
-      <c r="P55" s="181" t="n"/>
-      <c r="Q55" s="181" t="n"/>
-      <c r="R55" s="181" t="n"/>
-      <c r="S55" s="181" t="n"/>
-      <c r="T55" s="181" t="n"/>
-      <c r="U55" s="181" t="n"/>
-      <c r="V55" s="181" t="n"/>
-      <c r="W55" s="181" t="n"/>
-      <c r="X55" s="181" t="n"/>
-      <c r="Y55" s="181" t="n"/>
-    </row>
-    <row r="56" ht="12.75" customHeight="1" s="127">
-      <c r="A56" s="181" t="n"/>
-      <c r="B56" s="181" t="n"/>
-      <c r="C56" s="181" t="n"/>
-      <c r="D56" s="181" t="n"/>
-      <c r="E56" s="181" t="n"/>
-      <c r="F56" s="181" t="n"/>
-      <c r="G56" s="181" t="n"/>
-      <c r="H56" s="181" t="n"/>
-      <c r="I56" s="181" t="n"/>
-      <c r="J56" s="181" t="n"/>
-      <c r="K56" s="181" t="n"/>
-      <c r="L56" s="181" t="n"/>
-      <c r="M56" s="181" t="n"/>
-      <c r="N56" s="181" t="n"/>
-      <c r="O56" s="181" t="n"/>
-      <c r="P56" s="181" t="n"/>
-      <c r="Q56" s="181" t="n"/>
-      <c r="R56" s="181" t="n"/>
-      <c r="S56" s="181" t="n"/>
-      <c r="T56" s="181" t="n"/>
-      <c r="U56" s="181" t="n"/>
-      <c r="V56" s="181" t="n"/>
-      <c r="W56" s="181" t="n"/>
-      <c r="X56" s="181" t="n"/>
-      <c r="Y56" s="181" t="n"/>
-    </row>
-    <row r="57" ht="12.75" customHeight="1" s="127">
-      <c r="A57" s="181" t="n"/>
-      <c r="B57" s="181" t="n"/>
-      <c r="C57" s="181" t="n"/>
-      <c r="D57" s="181" t="n"/>
-      <c r="E57" s="181" t="n"/>
-      <c r="F57" s="181" t="n"/>
-      <c r="G57" s="181" t="n"/>
-      <c r="H57" s="181" t="n"/>
-      <c r="I57" s="181" t="n"/>
-      <c r="J57" s="181" t="n"/>
-      <c r="K57" s="181" t="n"/>
-      <c r="L57" s="181" t="n"/>
-      <c r="M57" s="181" t="n"/>
-      <c r="N57" s="181" t="n"/>
-      <c r="O57" s="181" t="n"/>
-      <c r="P57" s="181" t="n"/>
-      <c r="Q57" s="181" t="n"/>
-      <c r="R57" s="181" t="n"/>
-      <c r="S57" s="181" t="n"/>
-      <c r="T57" s="181" t="n"/>
-      <c r="U57" s="181" t="n"/>
-      <c r="V57" s="181" t="n"/>
-      <c r="W57" s="181" t="n"/>
-      <c r="X57" s="181" t="n"/>
-      <c r="Y57" s="181" t="n"/>
-    </row>
-    <row r="58" ht="12.75" customHeight="1" s="127">
-      <c r="A58" s="181" t="n"/>
-      <c r="B58" s="181" t="n"/>
-      <c r="C58" s="181" t="n"/>
-      <c r="D58" s="181" t="n"/>
-      <c r="E58" s="181" t="n"/>
-      <c r="F58" s="181" t="n"/>
-      <c r="G58" s="181" t="n"/>
-      <c r="H58" s="181" t="n"/>
-      <c r="I58" s="181" t="n"/>
-      <c r="J58" s="181" t="n"/>
-      <c r="K58" s="181" t="n"/>
-      <c r="L58" s="181" t="n"/>
-      <c r="M58" s="181" t="n"/>
-      <c r="N58" s="181" t="n"/>
-      <c r="O58" s="181" t="n"/>
-      <c r="P58" s="181" t="n"/>
-      <c r="Q58" s="181" t="n"/>
-      <c r="R58" s="181" t="n"/>
-      <c r="S58" s="181" t="n"/>
-      <c r="T58" s="181" t="n"/>
-      <c r="U58" s="181" t="n"/>
-      <c r="V58" s="181" t="n"/>
-      <c r="W58" s="181" t="n"/>
-      <c r="X58" s="181" t="n"/>
-      <c r="Y58" s="181" t="n"/>
-    </row>
-    <row r="59" ht="12.75" customHeight="1" s="127">
-      <c r="A59" s="181" t="n"/>
-      <c r="B59" s="181" t="n"/>
-      <c r="C59" s="181" t="n"/>
-      <c r="D59" s="181" t="n"/>
-      <c r="E59" s="181" t="n"/>
-      <c r="F59" s="181" t="n"/>
-      <c r="G59" s="181" t="n"/>
-      <c r="H59" s="181" t="n"/>
-      <c r="I59" s="181" t="n"/>
-      <c r="J59" s="181" t="n"/>
-      <c r="K59" s="181" t="n"/>
-      <c r="L59" s="181" t="n"/>
-      <c r="M59" s="181" t="n"/>
-      <c r="N59" s="181" t="n"/>
-      <c r="O59" s="181" t="n"/>
-      <c r="P59" s="181" t="n"/>
-      <c r="Q59" s="181" t="n"/>
-      <c r="R59" s="181" t="n"/>
-      <c r="S59" s="181" t="n"/>
-      <c r="T59" s="181" t="n"/>
-      <c r="U59" s="181" t="n"/>
-      <c r="V59" s="181" t="n"/>
-      <c r="W59" s="181" t="n"/>
-      <c r="X59" s="181" t="n"/>
-      <c r="Y59" s="181" t="n"/>
-    </row>
-    <row r="60" ht="12.75" customHeight="1" s="127">
-      <c r="A60" s="181" t="n"/>
-      <c r="B60" s="181" t="n"/>
-      <c r="C60" s="181" t="n"/>
-      <c r="D60" s="181" t="n"/>
-      <c r="E60" s="181" t="n"/>
-      <c r="F60" s="181" t="n"/>
-      <c r="G60" s="181" t="n"/>
-      <c r="H60" s="181" t="n"/>
-      <c r="I60" s="181" t="n"/>
-      <c r="J60" s="181" t="n"/>
-      <c r="K60" s="181" t="n"/>
-      <c r="L60" s="181" t="n"/>
-      <c r="M60" s="181" t="n"/>
-      <c r="N60" s="181" t="n"/>
-      <c r="O60" s="181" t="n"/>
-      <c r="P60" s="181" t="n"/>
-      <c r="Q60" s="181" t="n"/>
-      <c r="R60" s="181" t="n"/>
-      <c r="S60" s="181" t="n"/>
-      <c r="T60" s="181" t="n"/>
-      <c r="U60" s="181" t="n"/>
-      <c r="V60" s="181" t="n"/>
-      <c r="W60" s="181" t="n"/>
-      <c r="X60" s="181" t="n"/>
-      <c r="Y60" s="181" t="n"/>
-    </row>
-    <row r="61" ht="12.75" customHeight="1" s="127">
-      <c r="A61" s="181" t="n"/>
-      <c r="B61" s="181" t="n"/>
-      <c r="C61" s="181" t="n"/>
-      <c r="D61" s="181" t="n"/>
-      <c r="E61" s="181" t="n"/>
-      <c r="F61" s="181" t="n"/>
-      <c r="G61" s="181" t="n"/>
-      <c r="H61" s="181" t="n"/>
-      <c r="I61" s="181" t="n"/>
-      <c r="J61" s="181" t="n"/>
-      <c r="K61" s="181" t="n"/>
-      <c r="L61" s="181" t="n"/>
-      <c r="M61" s="181" t="n"/>
-      <c r="N61" s="181" t="n"/>
-      <c r="O61" s="181" t="n"/>
-      <c r="P61" s="181" t="n"/>
-      <c r="Q61" s="181" t="n"/>
-      <c r="R61" s="181" t="n"/>
-      <c r="S61" s="181" t="n"/>
-      <c r="T61" s="181" t="n"/>
-      <c r="U61" s="181" t="n"/>
-      <c r="V61" s="181" t="n"/>
-      <c r="W61" s="181" t="n"/>
-      <c r="X61" s="181" t="n"/>
-      <c r="Y61" s="181" t="n"/>
-    </row>
-    <row r="62" ht="12.75" customHeight="1" s="127">
-      <c r="A62" s="181" t="n"/>
-      <c r="B62" s="181" t="n"/>
-      <c r="C62" s="181" t="n"/>
-      <c r="D62" s="181" t="n"/>
-      <c r="E62" s="181" t="n"/>
-      <c r="F62" s="181" t="n"/>
-      <c r="G62" s="181" t="n"/>
-      <c r="H62" s="181" t="n"/>
-      <c r="I62" s="181" t="n"/>
-      <c r="J62" s="181" t="n"/>
-      <c r="K62" s="181" t="n"/>
-      <c r="L62" s="181" t="n"/>
-      <c r="M62" s="181" t="n"/>
-      <c r="N62" s="181" t="n"/>
-      <c r="O62" s="181" t="n"/>
-      <c r="P62" s="181" t="n"/>
-      <c r="Q62" s="181" t="n"/>
-      <c r="R62" s="181" t="n"/>
-      <c r="S62" s="181" t="n"/>
-      <c r="T62" s="181" t="n"/>
-      <c r="U62" s="181" t="n"/>
-      <c r="V62" s="181" t="n"/>
-      <c r="W62" s="181" t="n"/>
-      <c r="X62" s="181" t="n"/>
-      <c r="Y62" s="181" t="n"/>
-    </row>
-    <row r="63" ht="12.75" customHeight="1" s="127">
-      <c r="A63" s="181" t="n"/>
-      <c r="B63" s="181" t="n"/>
-      <c r="C63" s="181" t="n"/>
-      <c r="D63" s="181" t="n"/>
-      <c r="E63" s="181" t="n"/>
-      <c r="F63" s="181" t="n"/>
-      <c r="G63" s="181" t="n"/>
-      <c r="H63" s="181" t="n"/>
-      <c r="I63" s="181" t="n"/>
-      <c r="J63" s="181" t="n"/>
-      <c r="K63" s="181" t="n"/>
-      <c r="L63" s="181" t="n"/>
-      <c r="M63" s="181" t="n"/>
-      <c r="N63" s="181" t="n"/>
-      <c r="O63" s="181" t="n"/>
-      <c r="P63" s="181" t="n"/>
-      <c r="Q63" s="181" t="n"/>
-      <c r="R63" s="181" t="n"/>
-      <c r="S63" s="181" t="n"/>
-      <c r="T63" s="181" t="n"/>
-      <c r="U63" s="181" t="n"/>
-      <c r="V63" s="181" t="n"/>
-      <c r="W63" s="181" t="n"/>
-      <c r="X63" s="181" t="n"/>
-      <c r="Y63" s="181" t="n"/>
-    </row>
-    <row r="64" ht="12.75" customHeight="1" s="127">
-      <c r="A64" s="181" t="n"/>
-      <c r="B64" s="181" t="n"/>
-      <c r="C64" s="181" t="n"/>
-      <c r="D64" s="181" t="n"/>
-      <c r="E64" s="181" t="n"/>
-      <c r="F64" s="181" t="n"/>
-      <c r="G64" s="181" t="n"/>
-      <c r="H64" s="181" t="n"/>
-      <c r="I64" s="181" t="n"/>
-      <c r="J64" s="181" t="n"/>
-      <c r="K64" s="181" t="n"/>
-      <c r="L64" s="181" t="n"/>
-      <c r="M64" s="181" t="n"/>
-      <c r="N64" s="181" t="n"/>
-      <c r="O64" s="181" t="n"/>
-      <c r="P64" s="181" t="n"/>
-      <c r="Q64" s="181" t="n"/>
-      <c r="R64" s="181" t="n"/>
-      <c r="S64" s="181" t="n"/>
-      <c r="T64" s="181" t="n"/>
-      <c r="U64" s="181" t="n"/>
-      <c r="V64" s="181" t="n"/>
-      <c r="W64" s="181" t="n"/>
-      <c r="X64" s="181" t="n"/>
-      <c r="Y64" s="181" t="n"/>
-    </row>
-    <row r="65" ht="12.75" customHeight="1" s="127">
-      <c r="A65" s="181" t="n"/>
-      <c r="B65" s="181" t="n"/>
-      <c r="C65" s="181" t="n"/>
-      <c r="D65" s="181" t="n"/>
-      <c r="E65" s="181" t="n"/>
-      <c r="F65" s="181" t="n"/>
-      <c r="G65" s="181" t="n"/>
-      <c r="H65" s="181" t="n"/>
-      <c r="I65" s="181" t="n"/>
-      <c r="J65" s="181" t="n"/>
-      <c r="K65" s="181" t="n"/>
-      <c r="L65" s="181" t="n"/>
-      <c r="M65" s="181" t="n"/>
-      <c r="N65" s="181" t="n"/>
-      <c r="O65" s="181" t="n"/>
-      <c r="P65" s="181" t="n"/>
-      <c r="Q65" s="181" t="n"/>
-      <c r="R65" s="181" t="n"/>
-      <c r="S65" s="181" t="n"/>
-      <c r="T65" s="181" t="n"/>
-      <c r="U65" s="181" t="n"/>
-      <c r="V65" s="181" t="n"/>
-      <c r="W65" s="181" t="n"/>
-      <c r="X65" s="181" t="n"/>
-      <c r="Y65" s="181" t="n"/>
-    </row>
-    <row r="66" ht="12.75" customHeight="1" s="127">
-      <c r="A66" s="181" t="n"/>
-      <c r="B66" s="181" t="n"/>
-      <c r="C66" s="181" t="n"/>
-      <c r="D66" s="181" t="n"/>
-      <c r="E66" s="181" t="n"/>
-      <c r="F66" s="181" t="n"/>
-      <c r="G66" s="181" t="n"/>
-      <c r="H66" s="181" t="n"/>
-      <c r="I66" s="181" t="n"/>
-      <c r="J66" s="181" t="n"/>
-      <c r="K66" s="181" t="n"/>
-      <c r="L66" s="181" t="n"/>
-      <c r="M66" s="181" t="n"/>
-      <c r="N66" s="181" t="n"/>
-      <c r="O66" s="181" t="n"/>
-      <c r="P66" s="181" t="n"/>
-      <c r="Q66" s="181" t="n"/>
-      <c r="R66" s="181" t="n"/>
-      <c r="S66" s="181" t="n"/>
-      <c r="T66" s="181" t="n"/>
-      <c r="U66" s="181" t="n"/>
-      <c r="V66" s="181" t="n"/>
-      <c r="W66" s="181" t="n"/>
-      <c r="X66" s="181" t="n"/>
-      <c r="Y66" s="181" t="n"/>
-    </row>
-    <row r="67" ht="12.75" customHeight="1" s="127">
-      <c r="A67" s="181" t="n"/>
-      <c r="B67" s="181" t="n"/>
-      <c r="C67" s="181" t="n"/>
-      <c r="D67" s="181" t="n"/>
-      <c r="E67" s="181" t="n"/>
-      <c r="F67" s="181" t="n"/>
-      <c r="G67" s="181" t="n"/>
-      <c r="H67" s="181" t="n"/>
-      <c r="I67" s="181" t="n"/>
-      <c r="J67" s="181" t="n"/>
-      <c r="K67" s="181" t="n"/>
-      <c r="L67" s="181" t="n"/>
-      <c r="M67" s="181" t="n"/>
-      <c r="N67" s="181" t="n"/>
-      <c r="O67" s="181" t="n"/>
-      <c r="P67" s="181" t="n"/>
-      <c r="Q67" s="181" t="n"/>
-      <c r="R67" s="181" t="n"/>
-      <c r="S67" s="181" t="n"/>
-      <c r="T67" s="181" t="n"/>
-      <c r="U67" s="181" t="n"/>
-      <c r="V67" s="181" t="n"/>
-      <c r="W67" s="181" t="n"/>
-      <c r="X67" s="181" t="n"/>
-      <c r="Y67" s="181" t="n"/>
-    </row>
-    <row r="68" ht="12.75" customHeight="1" s="127">
-      <c r="A68" s="181" t="n"/>
-      <c r="B68" s="181" t="n"/>
-      <c r="C68" s="181" t="n"/>
-      <c r="D68" s="181" t="n"/>
-      <c r="E68" s="181" t="n"/>
-      <c r="F68" s="181" t="n"/>
-      <c r="G68" s="181" t="n"/>
-      <c r="H68" s="181" t="n"/>
-      <c r="I68" s="181" t="n"/>
-      <c r="J68" s="181" t="n"/>
-      <c r="K68" s="181" t="n"/>
-      <c r="L68" s="181" t="n"/>
-      <c r="M68" s="181" t="n"/>
-      <c r="N68" s="181" t="n"/>
-      <c r="O68" s="181" t="n"/>
-      <c r="P68" s="181" t="n"/>
-      <c r="Q68" s="181" t="n"/>
-      <c r="R68" s="181" t="n"/>
-      <c r="S68" s="181" t="n"/>
-      <c r="T68" s="181" t="n"/>
-      <c r="U68" s="181" t="n"/>
-      <c r="V68" s="181" t="n"/>
-      <c r="W68" s="181" t="n"/>
-      <c r="X68" s="181" t="n"/>
-      <c r="Y68" s="181" t="n"/>
-    </row>
-    <row r="69" ht="12.75" customHeight="1" s="127">
-      <c r="A69" s="181" t="n"/>
-      <c r="B69" s="181" t="n"/>
-      <c r="C69" s="181" t="n"/>
-      <c r="D69" s="181" t="n"/>
-      <c r="E69" s="181" t="n"/>
-      <c r="F69" s="181" t="n"/>
-      <c r="G69" s="181" t="n"/>
-      <c r="H69" s="181" t="n"/>
-      <c r="I69" s="181" t="n"/>
-      <c r="J69" s="181" t="n"/>
-      <c r="K69" s="181" t="n"/>
-      <c r="L69" s="181" t="n"/>
-      <c r="M69" s="181" t="n"/>
-      <c r="N69" s="181" t="n"/>
-      <c r="O69" s="181" t="n"/>
-      <c r="P69" s="181" t="n"/>
-      <c r="Q69" s="181" t="n"/>
-      <c r="R69" s="181" t="n"/>
-      <c r="S69" s="181" t="n"/>
-      <c r="T69" s="181" t="n"/>
-      <c r="U69" s="181" t="n"/>
-      <c r="V69" s="181" t="n"/>
-      <c r="W69" s="181" t="n"/>
-      <c r="X69" s="181" t="n"/>
-      <c r="Y69" s="181" t="n"/>
-    </row>
-    <row r="70" ht="12.75" customHeight="1" s="127">
-      <c r="A70" s="181" t="n"/>
-      <c r="B70" s="181" t="n"/>
-      <c r="C70" s="181" t="n"/>
-      <c r="D70" s="181" t="n"/>
-      <c r="E70" s="181" t="n"/>
-      <c r="F70" s="181" t="n"/>
-      <c r="G70" s="181" t="n"/>
-      <c r="H70" s="181" t="n"/>
-      <c r="I70" s="181" t="n"/>
-      <c r="J70" s="181" t="n"/>
-      <c r="K70" s="181" t="n"/>
-      <c r="L70" s="181" t="n"/>
-      <c r="M70" s="181" t="n"/>
-      <c r="N70" s="181" t="n"/>
-      <c r="O70" s="181" t="n"/>
-      <c r="P70" s="181" t="n"/>
-      <c r="Q70" s="181" t="n"/>
-      <c r="R70" s="181" t="n"/>
-      <c r="S70" s="181" t="n"/>
-      <c r="T70" s="181" t="n"/>
-      <c r="U70" s="181" t="n"/>
-      <c r="V70" s="181" t="n"/>
-      <c r="W70" s="181" t="n"/>
-      <c r="X70" s="181" t="n"/>
-      <c r="Y70" s="181" t="n"/>
-    </row>
-    <row r="71" ht="12.75" customHeight="1" s="127">
-      <c r="A71" s="181" t="n"/>
-      <c r="B71" s="181" t="n"/>
-      <c r="C71" s="181" t="n"/>
-      <c r="D71" s="181" t="n"/>
-      <c r="E71" s="181" t="n"/>
-      <c r="F71" s="181" t="n"/>
-      <c r="G71" s="181" t="n"/>
-      <c r="H71" s="181" t="n"/>
-      <c r="I71" s="181" t="n"/>
-      <c r="J71" s="181" t="n"/>
-      <c r="K71" s="181" t="n"/>
-      <c r="L71" s="181" t="n"/>
-      <c r="M71" s="181" t="n"/>
-      <c r="N71" s="181" t="n"/>
-      <c r="O71" s="181" t="n"/>
-      <c r="P71" s="181" t="n"/>
-      <c r="Q71" s="181" t="n"/>
-      <c r="R71" s="181" t="n"/>
-      <c r="S71" s="181" t="n"/>
-      <c r="T71" s="181" t="n"/>
-      <c r="U71" s="181" t="n"/>
-      <c r="V71" s="181" t="n"/>
-      <c r="W71" s="181" t="n"/>
-      <c r="X71" s="181" t="n"/>
-      <c r="Y71" s="181" t="n"/>
-    </row>
-    <row r="72" ht="12.75" customHeight="1" s="127">
-      <c r="A72" s="181" t="n"/>
-      <c r="B72" s="181" t="n"/>
-      <c r="C72" s="181" t="n"/>
-      <c r="D72" s="181" t="n"/>
-      <c r="E72" s="181" t="n"/>
-      <c r="F72" s="181" t="n"/>
-      <c r="G72" s="181" t="n"/>
-      <c r="H72" s="181" t="n"/>
-      <c r="I72" s="181" t="n"/>
-      <c r="J72" s="181" t="n"/>
-      <c r="K72" s="181" t="n"/>
-      <c r="L72" s="181" t="n"/>
-      <c r="M72" s="181" t="n"/>
-      <c r="N72" s="181" t="n"/>
-      <c r="O72" s="181" t="n"/>
-      <c r="P72" s="181" t="n"/>
-      <c r="Q72" s="181" t="n"/>
-      <c r="R72" s="181" t="n"/>
-      <c r="S72" s="181" t="n"/>
-      <c r="T72" s="181" t="n"/>
-      <c r="U72" s="181" t="n"/>
-      <c r="V72" s="181" t="n"/>
-      <c r="W72" s="181" t="n"/>
-      <c r="X72" s="181" t="n"/>
-      <c r="Y72" s="181" t="n"/>
-    </row>
-    <row r="73" ht="12.75" customHeight="1" s="127">
-      <c r="A73" s="181" t="n"/>
-      <c r="B73" s="181" t="n"/>
-      <c r="C73" s="181" t="n"/>
-      <c r="D73" s="181" t="n"/>
-      <c r="E73" s="181" t="n"/>
-      <c r="F73" s="181" t="n"/>
-      <c r="G73" s="181" t="n"/>
-      <c r="H73" s="181" t="n"/>
-      <c r="I73" s="181" t="n"/>
-      <c r="J73" s="181" t="n"/>
-      <c r="K73" s="181" t="n"/>
-      <c r="L73" s="181" t="n"/>
-      <c r="M73" s="181" t="n"/>
-      <c r="N73" s="181" t="n"/>
-      <c r="O73" s="181" t="n"/>
-      <c r="P73" s="181" t="n"/>
-      <c r="Q73" s="181" t="n"/>
-      <c r="R73" s="181" t="n"/>
-      <c r="S73" s="181" t="n"/>
-      <c r="T73" s="181" t="n"/>
-      <c r="U73" s="181" t="n"/>
-      <c r="V73" s="181" t="n"/>
-      <c r="W73" s="181" t="n"/>
-      <c r="X73" s="181" t="n"/>
-      <c r="Y73" s="181" t="n"/>
-    </row>
-    <row r="74" ht="12.75" customHeight="1" s="127">
-      <c r="A74" s="181" t="n"/>
-      <c r="B74" s="181" t="n"/>
-      <c r="C74" s="181" t="n"/>
-      <c r="D74" s="181" t="n"/>
-      <c r="E74" s="181" t="n"/>
-      <c r="F74" s="181" t="n"/>
-      <c r="G74" s="181" t="n"/>
-      <c r="H74" s="181" t="n"/>
-      <c r="I74" s="181" t="n"/>
-      <c r="J74" s="181" t="n"/>
-      <c r="K74" s="181" t="n"/>
-      <c r="L74" s="181" t="n"/>
-      <c r="M74" s="181" t="n"/>
-      <c r="N74" s="181" t="n"/>
-      <c r="O74" s="181" t="n"/>
-      <c r="P74" s="181" t="n"/>
-      <c r="Q74" s="181" t="n"/>
-      <c r="R74" s="181" t="n"/>
-      <c r="S74" s="181" t="n"/>
-      <c r="T74" s="181" t="n"/>
-      <c r="U74" s="181" t="n"/>
-      <c r="V74" s="181" t="n"/>
-      <c r="W74" s="181" t="n"/>
-      <c r="X74" s="181" t="n"/>
-      <c r="Y74" s="181" t="n"/>
-    </row>
-    <row r="75" ht="12.75" customHeight="1" s="127">
-      <c r="A75" s="181" t="n"/>
-      <c r="B75" s="181" t="n"/>
-      <c r="C75" s="181" t="n"/>
-      <c r="D75" s="181" t="n"/>
-      <c r="E75" s="181" t="n"/>
-      <c r="F75" s="181" t="n"/>
-      <c r="G75" s="181" t="n"/>
-      <c r="H75" s="181" t="n"/>
-      <c r="I75" s="181" t="n"/>
-      <c r="J75" s="181" t="n"/>
-      <c r="K75" s="181" t="n"/>
-      <c r="L75" s="181" t="n"/>
-      <c r="M75" s="181" t="n"/>
-      <c r="N75" s="181" t="n"/>
-      <c r="O75" s="181" t="n"/>
-      <c r="P75" s="181" t="n"/>
-      <c r="Q75" s="181" t="n"/>
-      <c r="R75" s="181" t="n"/>
-      <c r="S75" s="181" t="n"/>
-      <c r="T75" s="181" t="n"/>
-      <c r="U75" s="181" t="n"/>
-      <c r="V75" s="181" t="n"/>
-      <c r="W75" s="181" t="n"/>
-      <c r="X75" s="181" t="n"/>
-      <c r="Y75" s="181" t="n"/>
-    </row>
-    <row r="76" ht="12.75" customHeight="1" s="127">
-      <c r="A76" s="181" t="n"/>
-      <c r="B76" s="181" t="n"/>
-      <c r="C76" s="181" t="n"/>
-      <c r="D76" s="181" t="n"/>
-      <c r="E76" s="181" t="n"/>
-      <c r="F76" s="181" t="n"/>
-      <c r="G76" s="181" t="n"/>
-      <c r="H76" s="181" t="n"/>
-      <c r="I76" s="181" t="n"/>
-      <c r="J76" s="181" t="n"/>
-      <c r="K76" s="181" t="n"/>
-      <c r="L76" s="181" t="n"/>
-      <c r="M76" s="181" t="n"/>
-      <c r="N76" s="181" t="n"/>
-      <c r="O76" s="181" t="n"/>
-      <c r="P76" s="181" t="n"/>
-      <c r="Q76" s="181" t="n"/>
-      <c r="R76" s="181" t="n"/>
-      <c r="S76" s="181" t="n"/>
-      <c r="T76" s="181" t="n"/>
-      <c r="U76" s="181" t="n"/>
-      <c r="V76" s="181" t="n"/>
-      <c r="W76" s="181" t="n"/>
-      <c r="X76" s="181" t="n"/>
-      <c r="Y76" s="181" t="n"/>
-    </row>
-    <row r="77" ht="12.75" customHeight="1" s="127">
-      <c r="A77" s="181" t="n"/>
-      <c r="B77" s="181" t="n"/>
-      <c r="C77" s="181" t="n"/>
-      <c r="D77" s="181" t="n"/>
-      <c r="E77" s="181" t="n"/>
-      <c r="F77" s="181" t="n"/>
-      <c r="G77" s="181" t="n"/>
-      <c r="H77" s="181" t="n"/>
-      <c r="I77" s="181" t="n"/>
-      <c r="J77" s="181" t="n"/>
-      <c r="K77" s="181" t="n"/>
-      <c r="L77" s="181" t="n"/>
-      <c r="M77" s="181" t="n"/>
-      <c r="N77" s="181" t="n"/>
-      <c r="O77" s="181" t="n"/>
-      <c r="P77" s="181" t="n"/>
-      <c r="Q77" s="181" t="n"/>
-      <c r="R77" s="181" t="n"/>
-      <c r="S77" s="181" t="n"/>
-      <c r="T77" s="181" t="n"/>
-      <c r="U77" s="181" t="n"/>
-      <c r="V77" s="181" t="n"/>
-      <c r="W77" s="181" t="n"/>
-      <c r="X77" s="181" t="n"/>
-      <c r="Y77" s="181" t="n"/>
-    </row>
-    <row r="78" ht="12.75" customHeight="1" s="127">
-      <c r="A78" s="181" t="n"/>
-      <c r="B78" s="181" t="n"/>
-      <c r="C78" s="181" t="n"/>
-      <c r="D78" s="181" t="n"/>
-      <c r="E78" s="181" t="n"/>
-      <c r="F78" s="181" t="n"/>
-      <c r="G78" s="181" t="n"/>
-      <c r="H78" s="181" t="n"/>
-      <c r="I78" s="181" t="n"/>
-      <c r="J78" s="181" t="n"/>
-      <c r="K78" s="181" t="n"/>
-      <c r="L78" s="181" t="n"/>
-      <c r="M78" s="181" t="n"/>
-      <c r="N78" s="181" t="n"/>
-      <c r="O78" s="181" t="n"/>
-      <c r="P78" s="181" t="n"/>
-      <c r="Q78" s="181" t="n"/>
-      <c r="R78" s="181" t="n"/>
-      <c r="S78" s="181" t="n"/>
-      <c r="T78" s="181" t="n"/>
-      <c r="U78" s="181" t="n"/>
-      <c r="V78" s="181" t="n"/>
-      <c r="W78" s="181" t="n"/>
-      <c r="X78" s="181" t="n"/>
-      <c r="Y78" s="181" t="n"/>
-    </row>
-    <row r="79" ht="12.75" customHeight="1" s="127">
-      <c r="A79" s="181" t="n"/>
-      <c r="B79" s="181" t="n"/>
-      <c r="C79" s="181" t="n"/>
-      <c r="D79" s="181" t="n"/>
-      <c r="E79" s="181" t="n"/>
-      <c r="F79" s="181" t="n"/>
-      <c r="G79" s="181" t="n"/>
-      <c r="H79" s="181" t="n"/>
-      <c r="I79" s="181" t="n"/>
-      <c r="J79" s="181" t="n"/>
-      <c r="K79" s="181" t="n"/>
-      <c r="L79" s="181" t="n"/>
-      <c r="M79" s="181" t="n"/>
-      <c r="N79" s="181" t="n"/>
-      <c r="O79" s="181" t="n"/>
-      <c r="P79" s="181" t="n"/>
-      <c r="Q79" s="181" t="n"/>
-      <c r="R79" s="181" t="n"/>
-      <c r="S79" s="181" t="n"/>
-      <c r="T79" s="181" t="n"/>
-      <c r="U79" s="181" t="n"/>
-      <c r="V79" s="181" t="n"/>
-      <c r="W79" s="181" t="n"/>
-      <c r="X79" s="181" t="n"/>
-      <c r="Y79" s="181" t="n"/>
-    </row>
-    <row r="80" ht="12.75" customHeight="1" s="127">
-      <c r="A80" s="181" t="n"/>
-      <c r="B80" s="181" t="n"/>
-      <c r="C80" s="181" t="n"/>
-      <c r="D80" s="181" t="n"/>
-      <c r="E80" s="181" t="n"/>
-      <c r="F80" s="181" t="n"/>
-      <c r="G80" s="181" t="n"/>
-      <c r="H80" s="181" t="n"/>
-      <c r="I80" s="181" t="n"/>
-      <c r="J80" s="181" t="n"/>
-      <c r="K80" s="181" t="n"/>
-      <c r="L80" s="181" t="n"/>
-      <c r="M80" s="181" t="n"/>
-      <c r="N80" s="181" t="n"/>
-      <c r="O80" s="181" t="n"/>
-      <c r="P80" s="181" t="n"/>
-      <c r="Q80" s="181" t="n"/>
-      <c r="R80" s="181" t="n"/>
-      <c r="S80" s="181" t="n"/>
-      <c r="T80" s="181" t="n"/>
-      <c r="U80" s="181" t="n"/>
-      <c r="V80" s="181" t="n"/>
-      <c r="W80" s="181" t="n"/>
-      <c r="X80" s="181" t="n"/>
-      <c r="Y80" s="181" t="n"/>
-    </row>
-    <row r="81" ht="12.75" customHeight="1" s="127">
-      <c r="A81" s="181" t="n"/>
-      <c r="B81" s="181" t="n"/>
-      <c r="C81" s="181" t="n"/>
-      <c r="D81" s="181" t="n"/>
-      <c r="E81" s="181" t="n"/>
-      <c r="F81" s="181" t="n"/>
-      <c r="G81" s="181" t="n"/>
-      <c r="H81" s="181" t="n"/>
-      <c r="I81" s="181" t="n"/>
-      <c r="J81" s="181" t="n"/>
-      <c r="K81" s="181" t="n"/>
-      <c r="L81" s="181" t="n"/>
-      <c r="M81" s="181" t="n"/>
-      <c r="N81" s="181" t="n"/>
-      <c r="O81" s="181" t="n"/>
-      <c r="P81" s="181" t="n"/>
-      <c r="Q81" s="181" t="n"/>
-      <c r="R81" s="181" t="n"/>
-      <c r="S81" s="181" t="n"/>
-      <c r="T81" s="181" t="n"/>
-      <c r="U81" s="181" t="n"/>
-      <c r="V81" s="181" t="n"/>
-      <c r="W81" s="181" t="n"/>
-      <c r="X81" s="181" t="n"/>
-      <c r="Y81" s="181" t="n"/>
-    </row>
-    <row r="82" ht="12.75" customHeight="1" s="127">
-      <c r="A82" s="181" t="n"/>
-      <c r="B82" s="181" t="n"/>
-      <c r="C82" s="181" t="n"/>
-      <c r="D82" s="181" t="n"/>
-      <c r="E82" s="181" t="n"/>
-      <c r="F82" s="181" t="n"/>
-      <c r="G82" s="181" t="n"/>
-      <c r="H82" s="181" t="n"/>
-      <c r="I82" s="181" t="n"/>
-      <c r="J82" s="181" t="n"/>
-      <c r="K82" s="181" t="n"/>
-      <c r="L82" s="181" t="n"/>
-      <c r="M82" s="181" t="n"/>
-      <c r="N82" s="181" t="n"/>
-      <c r="O82" s="181" t="n"/>
-      <c r="P82" s="181" t="n"/>
-      <c r="Q82" s="181" t="n"/>
-      <c r="R82" s="181" t="n"/>
-      <c r="S82" s="181" t="n"/>
-      <c r="T82" s="181" t="n"/>
-      <c r="U82" s="181" t="n"/>
-      <c r="V82" s="181" t="n"/>
-      <c r="W82" s="181" t="n"/>
-      <c r="X82" s="181" t="n"/>
-      <c r="Y82" s="181" t="n"/>
-    </row>
-    <row r="83" ht="12.75" customHeight="1" s="127">
-      <c r="A83" s="181" t="n"/>
-      <c r="B83" s="181" t="n"/>
-      <c r="C83" s="181" t="n"/>
-      <c r="D83" s="181" t="n"/>
-      <c r="E83" s="181" t="n"/>
-      <c r="F83" s="181" t="n"/>
-      <c r="G83" s="181" t="n"/>
-      <c r="H83" s="181" t="n"/>
-      <c r="I83" s="181" t="n"/>
-      <c r="J83" s="181" t="n"/>
-      <c r="K83" s="181" t="n"/>
-      <c r="L83" s="181" t="n"/>
-      <c r="M83" s="181" t="n"/>
-      <c r="N83" s="181" t="n"/>
-      <c r="O83" s="181" t="n"/>
-      <c r="P83" s="181" t="n"/>
-      <c r="Q83" s="181" t="n"/>
-      <c r="R83" s="181" t="n"/>
-      <c r="S83" s="181" t="n"/>
-      <c r="T83" s="181" t="n"/>
-      <c r="U83" s="181" t="n"/>
-      <c r="V83" s="181" t="n"/>
-      <c r="W83" s="181" t="n"/>
-      <c r="X83" s="181" t="n"/>
-      <c r="Y83" s="181" t="n"/>
-    </row>
-    <row r="84" ht="12.75" customHeight="1" s="127">
-      <c r="A84" s="181" t="n"/>
-      <c r="B84" s="181" t="n"/>
-      <c r="C84" s="181" t="n"/>
-      <c r="D84" s="181" t="n"/>
-      <c r="E84" s="181" t="n"/>
-      <c r="F84" s="181" t="n"/>
-      <c r="G84" s="181" t="n"/>
-      <c r="H84" s="181" t="n"/>
-      <c r="I84" s="181" t="n"/>
-      <c r="J84" s="181" t="n"/>
-      <c r="K84" s="181" t="n"/>
-      <c r="L84" s="181" t="n"/>
-      <c r="M84" s="181" t="n"/>
-      <c r="N84" s="181" t="n"/>
-      <c r="O84" s="181" t="n"/>
-      <c r="P84" s="181" t="n"/>
-      <c r="Q84" s="181" t="n"/>
-      <c r="R84" s="181" t="n"/>
-      <c r="S84" s="181" t="n"/>
-      <c r="T84" s="181" t="n"/>
-      <c r="U84" s="181" t="n"/>
-      <c r="V84" s="181" t="n"/>
-      <c r="W84" s="181" t="n"/>
-      <c r="X84" s="181" t="n"/>
-      <c r="Y84" s="181" t="n"/>
-    </row>
-    <row r="85" ht="12.75" customHeight="1" s="127">
-      <c r="A85" s="181" t="n"/>
-      <c r="B85" s="181" t="n"/>
-      <c r="C85" s="181" t="n"/>
-      <c r="D85" s="181" t="n"/>
-      <c r="E85" s="181" t="n"/>
-      <c r="F85" s="181" t="n"/>
-      <c r="G85" s="181" t="n"/>
-      <c r="H85" s="181" t="n"/>
-      <c r="I85" s="181" t="n"/>
-      <c r="J85" s="181" t="n"/>
-      <c r="K85" s="181" t="n"/>
-      <c r="L85" s="181" t="n"/>
-      <c r="M85" s="181" t="n"/>
-      <c r="N85" s="181" t="n"/>
-      <c r="O85" s="181" t="n"/>
-      <c r="P85" s="181" t="n"/>
-      <c r="Q85" s="181" t="n"/>
-      <c r="R85" s="181" t="n"/>
-      <c r="S85" s="181" t="n"/>
-      <c r="T85" s="181" t="n"/>
-      <c r="U85" s="181" t="n"/>
-      <c r="V85" s="181" t="n"/>
-      <c r="W85" s="181" t="n"/>
-      <c r="X85" s="181" t="n"/>
-      <c r="Y85" s="181" t="n"/>
-    </row>
-    <row r="86" ht="12.75" customHeight="1" s="127">
-      <c r="A86" s="181" t="n"/>
-      <c r="B86" s="181" t="n"/>
-      <c r="C86" s="181" t="n"/>
-      <c r="D86" s="181" t="n"/>
-      <c r="E86" s="181" t="n"/>
-      <c r="F86" s="181" t="n"/>
-      <c r="G86" s="181" t="n"/>
-      <c r="H86" s="181" t="n"/>
-      <c r="I86" s="181" t="n"/>
-      <c r="J86" s="181" t="n"/>
-      <c r="K86" s="181" t="n"/>
-      <c r="L86" s="181" t="n"/>
-      <c r="M86" s="181" t="n"/>
-      <c r="N86" s="181" t="n"/>
-      <c r="O86" s="181" t="n"/>
-      <c r="P86" s="181" t="n"/>
-      <c r="Q86" s="181" t="n"/>
-      <c r="R86" s="181" t="n"/>
-      <c r="S86" s="181" t="n"/>
-      <c r="T86" s="181" t="n"/>
-      <c r="U86" s="181" t="n"/>
-      <c r="V86" s="181" t="n"/>
-      <c r="W86" s="181" t="n"/>
-      <c r="X86" s="181" t="n"/>
-      <c r="Y86" s="181" t="n"/>
-    </row>
-    <row r="87" ht="12.75" customHeight="1" s="127">
-      <c r="A87" s="181" t="n"/>
-      <c r="B87" s="181" t="n"/>
-      <c r="C87" s="181" t="n"/>
-      <c r="D87" s="181" t="n"/>
-      <c r="E87" s="181" t="n"/>
-      <c r="F87" s="181" t="n"/>
-      <c r="G87" s="181" t="n"/>
-      <c r="H87" s="181" t="n"/>
-      <c r="I87" s="181" t="n"/>
-      <c r="J87" s="181" t="n"/>
-      <c r="K87" s="181" t="n"/>
-      <c r="L87" s="181" t="n"/>
-      <c r="M87" s="181" t="n"/>
-      <c r="N87" s="181" t="n"/>
-      <c r="O87" s="181" t="n"/>
-      <c r="P87" s="181" t="n"/>
-      <c r="Q87" s="181" t="n"/>
-      <c r="R87" s="181" t="n"/>
-      <c r="S87" s="181" t="n"/>
-      <c r="T87" s="181" t="n"/>
-      <c r="U87" s="181" t="n"/>
-      <c r="V87" s="181" t="n"/>
-      <c r="W87" s="181" t="n"/>
-      <c r="X87" s="181" t="n"/>
-      <c r="Y87" s="181" t="n"/>
-    </row>
-    <row r="88" ht="12.75" customHeight="1" s="127">
-      <c r="A88" s="181" t="n"/>
-      <c r="B88" s="181" t="n"/>
-      <c r="C88" s="181" t="n"/>
-      <c r="D88" s="181" t="n"/>
-      <c r="E88" s="181" t="n"/>
-      <c r="F88" s="181" t="n"/>
-      <c r="G88" s="181" t="n"/>
-      <c r="H88" s="181" t="n"/>
-      <c r="I88" s="181" t="n"/>
-      <c r="J88" s="181" t="n"/>
-      <c r="K88" s="181" t="n"/>
-      <c r="L88" s="181" t="n"/>
-      <c r="M88" s="181" t="n"/>
-      <c r="N88" s="181" t="n"/>
-      <c r="O88" s="181" t="n"/>
-      <c r="P88" s="181" t="n"/>
-      <c r="Q88" s="181" t="n"/>
-      <c r="R88" s="181" t="n"/>
-      <c r="S88" s="181" t="n"/>
-      <c r="T88" s="181" t="n"/>
-      <c r="U88" s="181" t="n"/>
-      <c r="V88" s="181" t="n"/>
-      <c r="W88" s="181" t="n"/>
-      <c r="X88" s="181" t="n"/>
-      <c r="Y88" s="181" t="n"/>
-    </row>
-    <row r="89" ht="12.75" customHeight="1" s="127">
-      <c r="A89" s="181" t="n"/>
-      <c r="B89" s="181" t="n"/>
-      <c r="C89" s="181" t="n"/>
-      <c r="D89" s="181" t="n"/>
-      <c r="E89" s="181" t="n"/>
-      <c r="F89" s="181" t="n"/>
-      <c r="G89" s="181" t="n"/>
-      <c r="H89" s="181" t="n"/>
-      <c r="I89" s="181" t="n"/>
-      <c r="J89" s="181" t="n"/>
-      <c r="K89" s="181" t="n"/>
-      <c r="L89" s="181" t="n"/>
-      <c r="M89" s="181" t="n"/>
-      <c r="N89" s="181" t="n"/>
-      <c r="O89" s="181" t="n"/>
-      <c r="P89" s="181" t="n"/>
-      <c r="Q89" s="181" t="n"/>
-      <c r="R89" s="181" t="n"/>
-      <c r="S89" s="181" t="n"/>
-      <c r="T89" s="181" t="n"/>
-      <c r="U89" s="181" t="n"/>
-      <c r="V89" s="181" t="n"/>
-      <c r="W89" s="181" t="n"/>
-      <c r="X89" s="181" t="n"/>
-      <c r="Y89" s="181" t="n"/>
-    </row>
-    <row r="90" ht="12.75" customHeight="1" s="127">
-      <c r="A90" s="181" t="n"/>
-      <c r="B90" s="181" t="n"/>
-      <c r="C90" s="181" t="n"/>
-      <c r="D90" s="181" t="n"/>
-      <c r="E90" s="181" t="n"/>
-      <c r="F90" s="181" t="n"/>
-      <c r="G90" s="181" t="n"/>
-      <c r="H90" s="181" t="n"/>
-      <c r="I90" s="181" t="n"/>
-      <c r="J90" s="181" t="n"/>
-      <c r="K90" s="181" t="n"/>
-      <c r="L90" s="181" t="n"/>
-      <c r="M90" s="181" t="n"/>
-      <c r="N90" s="181" t="n"/>
-      <c r="O90" s="181" t="n"/>
-      <c r="P90" s="181" t="n"/>
-      <c r="Q90" s="181" t="n"/>
-      <c r="R90" s="181" t="n"/>
-      <c r="S90" s="181" t="n"/>
-      <c r="T90" s="181" t="n"/>
-      <c r="U90" s="181" t="n"/>
-      <c r="V90" s="181" t="n"/>
-      <c r="W90" s="181" t="n"/>
-      <c r="X90" s="181" t="n"/>
-      <c r="Y90" s="181" t="n"/>
-    </row>
-    <row r="91" ht="12.75" customHeight="1" s="127">
-      <c r="A91" s="181" t="n"/>
-      <c r="B91" s="181" t="n"/>
-      <c r="C91" s="181" t="n"/>
-      <c r="D91" s="181" t="n"/>
-      <c r="E91" s="181" t="n"/>
-      <c r="F91" s="181" t="n"/>
-      <c r="G91" s="181" t="n"/>
-      <c r="H91" s="181" t="n"/>
-      <c r="I91" s="181" t="n"/>
-      <c r="J91" s="181" t="n"/>
-      <c r="K91" s="181" t="n"/>
-      <c r="L91" s="181" t="n"/>
-      <c r="M91" s="181" t="n"/>
-      <c r="N91" s="181" t="n"/>
-      <c r="O91" s="181" t="n"/>
-      <c r="P91" s="181" t="n"/>
-      <c r="Q91" s="181" t="n"/>
-      <c r="R91" s="181" t="n"/>
-      <c r="S91" s="181" t="n"/>
-      <c r="T91" s="181" t="n"/>
-      <c r="U91" s="181" t="n"/>
-      <c r="V91" s="181" t="n"/>
-      <c r="W91" s="181" t="n"/>
-      <c r="X91" s="181" t="n"/>
-      <c r="Y91" s="181" t="n"/>
-    </row>
-    <row r="92" ht="12.75" customHeight="1" s="127">
-      <c r="A92" s="181" t="n"/>
-      <c r="B92" s="181" t="n"/>
-      <c r="C92" s="181" t="n"/>
-      <c r="D92" s="181" t="n"/>
-      <c r="E92" s="181" t="n"/>
-      <c r="F92" s="181" t="n"/>
-      <c r="G92" s="181" t="n"/>
-      <c r="H92" s="181" t="n"/>
-      <c r="I92" s="181" t="n"/>
-      <c r="J92" s="181" t="n"/>
-      <c r="K92" s="181" t="n"/>
-      <c r="L92" s="181" t="n"/>
-      <c r="M92" s="181" t="n"/>
-      <c r="N92" s="181" t="n"/>
-      <c r="O92" s="181" t="n"/>
-      <c r="P92" s="181" t="n"/>
-      <c r="Q92" s="181" t="n"/>
-      <c r="R92" s="181" t="n"/>
-      <c r="S92" s="181" t="n"/>
-      <c r="T92" s="181" t="n"/>
-      <c r="U92" s="181" t="n"/>
-      <c r="V92" s="181" t="n"/>
-      <c r="W92" s="181" t="n"/>
-      <c r="X92" s="181" t="n"/>
-      <c r="Y92" s="181" t="n"/>
-    </row>
-    <row r="93" ht="12.75" customHeight="1" s="127">
-      <c r="A93" s="181" t="n"/>
-      <c r="B93" s="181" t="n"/>
-      <c r="C93" s="181" t="n"/>
-      <c r="D93" s="181" t="n"/>
-      <c r="E93" s="181" t="n"/>
-      <c r="F93" s="181" t="n"/>
-      <c r="G93" s="181" t="n"/>
-      <c r="H93" s="181" t="n"/>
-      <c r="I93" s="181" t="n"/>
-      <c r="J93" s="181" t="n"/>
-      <c r="K93" s="181" t="n"/>
-      <c r="L93" s="181" t="n"/>
-      <c r="M93" s="181" t="n"/>
-      <c r="N93" s="181" t="n"/>
-      <c r="O93" s="181" t="n"/>
-      <c r="P93" s="181" t="n"/>
-      <c r="Q93" s="181" t="n"/>
-      <c r="R93" s="181" t="n"/>
-      <c r="S93" s="181" t="n"/>
-      <c r="T93" s="181" t="n"/>
-      <c r="U93" s="181" t="n"/>
-      <c r="V93" s="181" t="n"/>
-      <c r="W93" s="181" t="n"/>
-      <c r="X93" s="181" t="n"/>
-      <c r="Y93" s="181" t="n"/>
-    </row>
-    <row r="94" ht="12.75" customHeight="1" s="127">
-      <c r="A94" s="181" t="n"/>
-      <c r="B94" s="181" t="n"/>
-      <c r="C94" s="181" t="n"/>
-      <c r="D94" s="181" t="n"/>
-      <c r="E94" s="181" t="n"/>
-      <c r="F94" s="181" t="n"/>
-      <c r="G94" s="181" t="n"/>
-      <c r="H94" s="181" t="n"/>
-      <c r="I94" s="181" t="n"/>
-      <c r="J94" s="181" t="n"/>
-      <c r="K94" s="181" t="n"/>
-      <c r="L94" s="181" t="n"/>
-      <c r="M94" s="181" t="n"/>
-      <c r="N94" s="181" t="n"/>
-      <c r="O94" s="181" t="n"/>
-      <c r="P94" s="181" t="n"/>
-      <c r="Q94" s="181" t="n"/>
-      <c r="R94" s="181" t="n"/>
-      <c r="S94" s="181" t="n"/>
-      <c r="T94" s="181" t="n"/>
-      <c r="U94" s="181" t="n"/>
-      <c r="V94" s="181" t="n"/>
-      <c r="W94" s="181" t="n"/>
-      <c r="X94" s="181" t="n"/>
-      <c r="Y94" s="181" t="n"/>
-    </row>
-    <row r="95" ht="12.75" customHeight="1" s="127">
-      <c r="A95" s="181" t="n"/>
-      <c r="B95" s="181" t="n"/>
-      <c r="C95" s="181" t="n"/>
-      <c r="D95" s="181" t="n"/>
-      <c r="E95" s="181" t="n"/>
-      <c r="F95" s="181" t="n"/>
-      <c r="G95" s="181" t="n"/>
-      <c r="H95" s="181" t="n"/>
-      <c r="I95" s="181" t="n"/>
-      <c r="J95" s="181" t="n"/>
-      <c r="K95" s="181" t="n"/>
-      <c r="L95" s="181" t="n"/>
-      <c r="M95" s="181" t="n"/>
-      <c r="N95" s="181" t="n"/>
-      <c r="O95" s="181" t="n"/>
-      <c r="P95" s="181" t="n"/>
-      <c r="Q95" s="181" t="n"/>
-      <c r="R95" s="181" t="n"/>
-      <c r="S95" s="181" t="n"/>
-      <c r="T95" s="181" t="n"/>
-      <c r="U95" s="181" t="n"/>
-      <c r="V95" s="181" t="n"/>
-      <c r="W95" s="181" t="n"/>
-      <c r="X95" s="181" t="n"/>
-      <c r="Y95" s="181" t="n"/>
-    </row>
-    <row r="96" ht="17.25" customHeight="1" s="127">
-      <c r="A96" s="181" t="n"/>
-      <c r="B96" s="181" t="n"/>
-      <c r="C96" s="181" t="n"/>
-      <c r="D96" s="181" t="n"/>
-      <c r="E96" s="181" t="n"/>
-      <c r="F96" s="181" t="n"/>
-      <c r="G96" s="181" t="n"/>
-      <c r="H96" s="181" t="n"/>
-      <c r="I96" s="181" t="n"/>
-      <c r="J96" s="181" t="n"/>
-      <c r="K96" s="181" t="n"/>
-      <c r="L96" s="181" t="n"/>
-      <c r="M96" s="181" t="n"/>
-      <c r="N96" s="181" t="n"/>
-      <c r="O96" s="181" t="n"/>
-      <c r="P96" s="181" t="n"/>
-      <c r="Q96" s="181" t="n"/>
-      <c r="R96" s="181" t="n"/>
-      <c r="S96" s="181" t="n"/>
-      <c r="T96" s="181" t="n"/>
-      <c r="U96" s="181" t="n"/>
-      <c r="V96" s="181" t="n"/>
-      <c r="W96" s="181" t="n"/>
-      <c r="X96" s="181" t="n"/>
-      <c r="Y96" s="181" t="n"/>
-    </row>
-    <row r="97" ht="17.25" customHeight="1" s="127">
-      <c r="A97" s="181" t="n"/>
-      <c r="B97" s="181" t="n"/>
-      <c r="C97" s="181" t="n"/>
-      <c r="D97" s="181" t="n"/>
-      <c r="E97" s="181" t="n"/>
-      <c r="F97" s="181" t="n"/>
-      <c r="G97" s="181" t="n"/>
-      <c r="H97" s="181" t="n"/>
-      <c r="I97" s="181" t="n"/>
-      <c r="J97" s="181" t="n"/>
-      <c r="K97" s="181" t="n"/>
-      <c r="L97" s="181" t="n"/>
-      <c r="M97" s="181" t="n"/>
-      <c r="N97" s="181" t="n"/>
-      <c r="O97" s="181" t="n"/>
-      <c r="P97" s="181" t="n"/>
-      <c r="Q97" s="181" t="n"/>
-      <c r="R97" s="181" t="n"/>
-      <c r="S97" s="181" t="n"/>
-      <c r="T97" s="181" t="n"/>
-      <c r="U97" s="181" t="n"/>
-      <c r="V97" s="181" t="n"/>
-      <c r="W97" s="181" t="n"/>
-      <c r="X97" s="181" t="n"/>
-      <c r="Y97" s="181" t="n"/>
-    </row>
-    <row r="98" ht="17.25" customHeight="1" s="127">
-      <c r="A98" s="181" t="n"/>
-      <c r="B98" s="181" t="n"/>
-      <c r="C98" s="181" t="n"/>
-      <c r="D98" s="181" t="n"/>
-      <c r="E98" s="181" t="n"/>
-      <c r="F98" s="181" t="n"/>
-      <c r="G98" s="181" t="n"/>
-      <c r="H98" s="181" t="n"/>
-      <c r="I98" s="181" t="n"/>
-      <c r="J98" s="181" t="n"/>
-      <c r="K98" s="181" t="n"/>
-      <c r="L98" s="181" t="n"/>
-      <c r="M98" s="181" t="n"/>
-      <c r="N98" s="181" t="n"/>
-      <c r="O98" s="181" t="n"/>
-      <c r="P98" s="181" t="n"/>
-      <c r="Q98" s="181" t="n"/>
-      <c r="R98" s="181" t="n"/>
-      <c r="S98" s="181" t="n"/>
-      <c r="T98" s="181" t="n"/>
-      <c r="U98" s="181" t="n"/>
-      <c r="V98" s="181" t="n"/>
-      <c r="W98" s="181" t="n"/>
-      <c r="X98" s="181" t="n"/>
-      <c r="Y98" s="181" t="n"/>
-    </row>
-    <row r="99" ht="17.25" customHeight="1" s="127">
-      <c r="A99" s="181" t="n"/>
-      <c r="B99" s="181" t="n"/>
-      <c r="C99" s="181" t="n"/>
-      <c r="D99" s="181" t="n"/>
-      <c r="E99" s="181" t="n"/>
-      <c r="F99" s="181" t="n"/>
-      <c r="G99" s="181" t="n"/>
-      <c r="H99" s="181" t="n"/>
-      <c r="I99" s="181" t="n"/>
-      <c r="J99" s="181" t="n"/>
-      <c r="K99" s="181" t="n"/>
-      <c r="L99" s="181" t="n"/>
-      <c r="M99" s="181" t="n"/>
-      <c r="N99" s="181" t="n"/>
-      <c r="O99" s="181" t="n"/>
-      <c r="P99" s="181" t="n"/>
-      <c r="Q99" s="181" t="n"/>
-      <c r="R99" s="181" t="n"/>
-      <c r="S99" s="181" t="n"/>
-      <c r="T99" s="181" t="n"/>
-      <c r="U99" s="181" t="n"/>
-      <c r="V99" s="181" t="n"/>
-      <c r="W99" s="181" t="n"/>
-      <c r="X99" s="181" t="n"/>
-      <c r="Y99" s="181" t="n"/>
-    </row>
-    <row r="100" ht="17.25" customHeight="1" s="127">
-      <c r="A100" s="181" t="n"/>
-      <c r="B100" s="181" t="n"/>
-      <c r="C100" s="181" t="n"/>
-      <c r="D100" s="181" t="n"/>
-      <c r="E100" s="181" t="n"/>
-      <c r="F100" s="181" t="n"/>
-      <c r="G100" s="181" t="n"/>
-      <c r="H100" s="181" t="n"/>
-      <c r="I100" s="181" t="n"/>
-      <c r="J100" s="181" t="n"/>
-      <c r="K100" s="181" t="n"/>
-      <c r="L100" s="181" t="n"/>
-      <c r="M100" s="181" t="n"/>
-      <c r="N100" s="181" t="n"/>
-      <c r="O100" s="181" t="n"/>
-      <c r="P100" s="181" t="n"/>
-      <c r="Q100" s="181" t="n"/>
-      <c r="R100" s="181" t="n"/>
-      <c r="S100" s="181" t="n"/>
-      <c r="T100" s="181" t="n"/>
-      <c r="U100" s="181" t="n"/>
-      <c r="V100" s="181" t="n"/>
-      <c r="W100" s="181" t="n"/>
-      <c r="X100" s="181" t="n"/>
-      <c r="Y100" s="181" t="n"/>
-    </row>
-    <row r="101" ht="17.25" customHeight="1" s="127">
-      <c r="A101" s="181" t="n"/>
-      <c r="B101" s="181" t="n"/>
-      <c r="C101" s="181" t="n"/>
-      <c r="D101" s="181" t="n"/>
-      <c r="E101" s="181" t="n"/>
-      <c r="F101" s="181" t="n"/>
-      <c r="G101" s="181" t="n"/>
-      <c r="H101" s="181" t="n"/>
-      <c r="I101" s="181" t="n"/>
-      <c r="J101" s="181" t="n"/>
-      <c r="K101" s="181" t="n"/>
-      <c r="L101" s="181" t="n"/>
-      <c r="M101" s="181" t="n"/>
-      <c r="N101" s="181" t="n"/>
-      <c r="O101" s="181" t="n"/>
-      <c r="P101" s="181" t="n"/>
-      <c r="Q101" s="181" t="n"/>
-      <c r="R101" s="181" t="n"/>
-      <c r="S101" s="181" t="n"/>
-      <c r="T101" s="181" t="n"/>
-      <c r="U101" s="181" t="n"/>
-      <c r="V101" s="181" t="n"/>
-      <c r="W101" s="181" t="n"/>
-      <c r="X101" s="181" t="n"/>
-      <c r="Y101" s="181" t="n"/>
-    </row>
-    <row r="102" ht="17.25" customHeight="1" s="127">
-      <c r="A102" s="181" t="n"/>
-      <c r="B102" s="181" t="n"/>
-      <c r="C102" s="181" t="n"/>
-      <c r="D102" s="181" t="n"/>
-      <c r="E102" s="181" t="n"/>
-      <c r="F102" s="181" t="n"/>
-      <c r="G102" s="181" t="n"/>
-      <c r="H102" s="181" t="n"/>
-      <c r="I102" s="181" t="n"/>
-      <c r="J102" s="181" t="n"/>
-      <c r="K102" s="181" t="n"/>
-      <c r="L102" s="181" t="n"/>
-      <c r="M102" s="181" t="n"/>
-      <c r="N102" s="181" t="n"/>
-      <c r="O102" s="181" t="n"/>
-      <c r="P102" s="181" t="n"/>
-      <c r="Q102" s="181" t="n"/>
-      <c r="R102" s="181" t="n"/>
-      <c r="S102" s="181" t="n"/>
-      <c r="T102" s="181" t="n"/>
-      <c r="U102" s="181" t="n"/>
-      <c r="V102" s="181" t="n"/>
-      <c r="W102" s="181" t="n"/>
-      <c r="X102" s="181" t="n"/>
-      <c r="Y102" s="181" t="n"/>
-    </row>
-    <row r="103" ht="17.25" customHeight="1" s="127">
-      <c r="A103" s="181" t="n"/>
-      <c r="B103" s="181" t="n"/>
-      <c r="C103" s="181" t="n"/>
-      <c r="D103" s="181" t="n"/>
-      <c r="E103" s="181" t="n"/>
-      <c r="F103" s="181" t="n"/>
-      <c r="G103" s="181" t="n"/>
-      <c r="H103" s="181" t="n"/>
-      <c r="I103" s="181" t="n"/>
-      <c r="J103" s="181" t="n"/>
-      <c r="K103" s="181" t="n"/>
-      <c r="L103" s="181" t="n"/>
-      <c r="M103" s="181" t="n"/>
-      <c r="N103" s="181" t="n"/>
-      <c r="O103" s="181" t="n"/>
-      <c r="P103" s="181" t="n"/>
-      <c r="Q103" s="181" t="n"/>
-      <c r="R103" s="181" t="n"/>
-      <c r="S103" s="181" t="n"/>
-      <c r="T103" s="181" t="n"/>
-      <c r="U103" s="181" t="n"/>
-      <c r="V103" s="181" t="n"/>
-      <c r="W103" s="181" t="n"/>
-      <c r="X103" s="181" t="n"/>
-      <c r="Y103" s="181" t="n"/>
-    </row>
-    <row r="104" ht="17.25" customHeight="1" s="127">
-      <c r="A104" s="181" t="n"/>
-      <c r="B104" s="181" t="n"/>
-      <c r="C104" s="181" t="n"/>
-      <c r="D104" s="181" t="n"/>
-      <c r="E104" s="181" t="n"/>
-      <c r="F104" s="181" t="n"/>
-      <c r="G104" s="181" t="n"/>
-      <c r="H104" s="181" t="n"/>
-      <c r="I104" s="181" t="n"/>
-      <c r="J104" s="181" t="n"/>
-      <c r="K104" s="181" t="n"/>
-      <c r="L104" s="181" t="n"/>
-      <c r="M104" s="181" t="n"/>
-      <c r="N104" s="181" t="n"/>
-      <c r="O104" s="181" t="n"/>
-      <c r="P104" s="181" t="n"/>
-      <c r="Q104" s="181" t="n"/>
-      <c r="R104" s="181" t="n"/>
-      <c r="S104" s="181" t="n"/>
-      <c r="T104" s="181" t="n"/>
-      <c r="U104" s="181" t="n"/>
-      <c r="V104" s="181" t="n"/>
-      <c r="W104" s="181" t="n"/>
-      <c r="X104" s="181" t="n"/>
-      <c r="Y104" s="181" t="n"/>
-    </row>
-    <row r="105" ht="17.25" customHeight="1" s="127">
-      <c r="A105" s="181" t="n"/>
-      <c r="B105" s="181" t="n"/>
-      <c r="C105" s="181" t="n"/>
-      <c r="D105" s="181" t="n"/>
-      <c r="E105" s="181" t="n"/>
-      <c r="F105" s="181" t="n"/>
-      <c r="G105" s="181" t="n"/>
-      <c r="H105" s="181" t="n"/>
-      <c r="I105" s="181" t="n"/>
-      <c r="J105" s="181" t="n"/>
-      <c r="K105" s="181" t="n"/>
-      <c r="L105" s="181" t="n"/>
-      <c r="M105" s="181" t="n"/>
-      <c r="N105" s="181" t="n"/>
-      <c r="O105" s="181" t="n"/>
-      <c r="P105" s="181" t="n"/>
-      <c r="Q105" s="181" t="n"/>
-      <c r="R105" s="181" t="n"/>
-      <c r="S105" s="181" t="n"/>
-      <c r="T105" s="181" t="n"/>
-      <c r="U105" s="181" t="n"/>
-      <c r="V105" s="181" t="n"/>
-      <c r="W105" s="181" t="n"/>
-      <c r="X105" s="181" t="n"/>
-      <c r="Y105" s="181" t="n"/>
-    </row>
-    <row r="106" ht="17.25" customHeight="1" s="127">
-      <c r="A106" s="181" t="n"/>
-      <c r="B106" s="181" t="n"/>
-      <c r="C106" s="181" t="n"/>
-      <c r="D106" s="181" t="n"/>
-      <c r="E106" s="181" t="n"/>
-      <c r="F106" s="181" t="n"/>
-      <c r="G106" s="181" t="n"/>
-      <c r="H106" s="181" t="n"/>
-      <c r="I106" s="181" t="n"/>
-      <c r="J106" s="181" t="n"/>
-      <c r="K106" s="181" t="n"/>
-      <c r="L106" s="181" t="n"/>
-      <c r="M106" s="181" t="n"/>
-      <c r="N106" s="181" t="n"/>
-      <c r="O106" s="181" t="n"/>
-      <c r="P106" s="181" t="n"/>
-      <c r="Q106" s="181" t="n"/>
-      <c r="R106" s="181" t="n"/>
-      <c r="S106" s="181" t="n"/>
-      <c r="T106" s="181" t="n"/>
-      <c r="U106" s="181" t="n"/>
-      <c r="V106" s="181" t="n"/>
-      <c r="W106" s="181" t="n"/>
-      <c r="X106" s="181" t="n"/>
-      <c r="Y106" s="181" t="n"/>
-    </row>
-    <row r="107" ht="17.25" customHeight="1" s="127">
-      <c r="A107" s="181" t="n"/>
-      <c r="B107" s="181" t="n"/>
-      <c r="C107" s="181" t="n"/>
-      <c r="D107" s="181" t="n"/>
-      <c r="E107" s="181" t="n"/>
-      <c r="F107" s="181" t="n"/>
-      <c r="G107" s="181" t="n"/>
-      <c r="H107" s="181" t="n"/>
-      <c r="I107" s="181" t="n"/>
-      <c r="J107" s="181" t="n"/>
-      <c r="K107" s="181" t="n"/>
-      <c r="L107" s="181" t="n"/>
-      <c r="M107" s="181" t="n"/>
-      <c r="N107" s="181" t="n"/>
-      <c r="O107" s="181" t="n"/>
-      <c r="P107" s="181" t="n"/>
-      <c r="Q107" s="181" t="n"/>
-      <c r="R107" s="181" t="n"/>
-      <c r="S107" s="181" t="n"/>
-      <c r="T107" s="181" t="n"/>
-      <c r="U107" s="181" t="n"/>
-      <c r="V107" s="181" t="n"/>
-      <c r="W107" s="181" t="n"/>
-      <c r="X107" s="181" t="n"/>
-      <c r="Y107" s="181" t="n"/>
-    </row>
-    <row r="108" ht="17.25" customHeight="1" s="127">
-      <c r="A108" s="181" t="n"/>
-      <c r="B108" s="181" t="n"/>
-      <c r="C108" s="181" t="n"/>
-      <c r="D108" s="181" t="n"/>
-      <c r="E108" s="181" t="n"/>
-      <c r="F108" s="181" t="n"/>
-      <c r="G108" s="181" t="n"/>
-      <c r="H108" s="181" t="n"/>
-      <c r="I108" s="181" t="n"/>
-      <c r="J108" s="181" t="n"/>
-      <c r="K108" s="181" t="n"/>
-      <c r="L108" s="181" t="n"/>
-      <c r="M108" s="181" t="n"/>
-      <c r="N108" s="181" t="n"/>
-      <c r="O108" s="181" t="n"/>
-      <c r="P108" s="181" t="n"/>
-      <c r="Q108" s="181" t="n"/>
-      <c r="R108" s="181" t="n"/>
-      <c r="S108" s="181" t="n"/>
-      <c r="T108" s="181" t="n"/>
-      <c r="U108" s="181" t="n"/>
-      <c r="V108" s="181" t="n"/>
-      <c r="W108" s="181" t="n"/>
-      <c r="X108" s="181" t="n"/>
-      <c r="Y108" s="181" t="n"/>
-    </row>
-    <row r="109" ht="17.25" customHeight="1" s="127">
-      <c r="A109" s="181" t="n"/>
-      <c r="B109" s="181" t="n"/>
-      <c r="C109" s="181" t="n"/>
-      <c r="D109" s="181" t="n"/>
-      <c r="E109" s="181" t="n"/>
-      <c r="F109" s="181" t="n"/>
-      <c r="G109" s="181" t="n"/>
-      <c r="H109" s="181" t="n"/>
-      <c r="I109" s="181" t="n"/>
-      <c r="J109" s="181" t="n"/>
-      <c r="K109" s="181" t="n"/>
-      <c r="L109" s="181" t="n"/>
-      <c r="M109" s="181" t="n"/>
-      <c r="N109" s="181" t="n"/>
-      <c r="O109" s="181" t="n"/>
-      <c r="P109" s="181" t="n"/>
-      <c r="Q109" s="181" t="n"/>
-      <c r="R109" s="181" t="n"/>
-      <c r="S109" s="181" t="n"/>
-      <c r="T109" s="181" t="n"/>
-      <c r="U109" s="181" t="n"/>
-      <c r="V109" s="181" t="n"/>
-      <c r="W109" s="181" t="n"/>
-      <c r="X109" s="181" t="n"/>
-      <c r="Y109" s="181" t="n"/>
-    </row>
-    <row r="110" ht="17.25" customHeight="1" s="127">
-      <c r="A110" s="181" t="n"/>
-      <c r="B110" s="181" t="n"/>
-      <c r="C110" s="181" t="n"/>
-      <c r="D110" s="181" t="n"/>
-      <c r="E110" s="181" t="n"/>
-      <c r="F110" s="181" t="n"/>
-      <c r="G110" s="181" t="n"/>
-      <c r="H110" s="181" t="n"/>
-      <c r="I110" s="181" t="n"/>
-      <c r="J110" s="181" t="n"/>
-      <c r="K110" s="181" t="n"/>
-      <c r="L110" s="181" t="n"/>
-      <c r="M110" s="181" t="n"/>
-      <c r="N110" s="181" t="n"/>
-      <c r="O110" s="181" t="n"/>
-      <c r="P110" s="181" t="n"/>
-      <c r="Q110" s="181" t="n"/>
-      <c r="R110" s="181" t="n"/>
-      <c r="S110" s="181" t="n"/>
-      <c r="T110" s="181" t="n"/>
-      <c r="U110" s="181" t="n"/>
-      <c r="V110" s="181" t="n"/>
-      <c r="W110" s="181" t="n"/>
-      <c r="X110" s="181" t="n"/>
-      <c r="Y110" s="181" t="n"/>
-    </row>
+    <row r="54" ht="12.75" customHeight="1" s="127"/>
+    <row r="55" ht="12.75" customHeight="1" s="127"/>
+    <row r="56" ht="12.75" customHeight="1" s="127"/>
+    <row r="57" ht="12.75" customHeight="1" s="127"/>
+    <row r="58" ht="12.75" customHeight="1" s="127"/>
+    <row r="59" ht="12.75" customHeight="1" s="127"/>
+    <row r="60" ht="12.75" customHeight="1" s="127"/>
+    <row r="61" ht="12.75" customHeight="1" s="127"/>
+    <row r="62" ht="12.75" customHeight="1" s="127"/>
+    <row r="63" ht="12.75" customHeight="1" s="127"/>
+    <row r="64" ht="12.75" customHeight="1" s="127"/>
+    <row r="65" ht="12.75" customHeight="1" s="127"/>
+    <row r="66" ht="12.75" customHeight="1" s="127"/>
+    <row r="67" ht="12.75" customHeight="1" s="127"/>
+    <row r="68" ht="12.75" customHeight="1" s="127"/>
+    <row r="69" ht="12.75" customHeight="1" s="127"/>
+    <row r="70" ht="12.75" customHeight="1" s="127"/>
+    <row r="71" ht="12.75" customHeight="1" s="127"/>
+    <row r="72" ht="12.75" customHeight="1" s="127"/>
+    <row r="73" ht="12.75" customHeight="1" s="127"/>
+    <row r="74" ht="12.75" customHeight="1" s="127"/>
+    <row r="75" ht="12.75" customHeight="1" s="127"/>
+    <row r="76" ht="12.75" customHeight="1" s="127"/>
+    <row r="77" ht="12.75" customHeight="1" s="127"/>
+    <row r="78" ht="12.75" customHeight="1" s="127"/>
+    <row r="79" ht="12.75" customHeight="1" s="127"/>
+    <row r="80" ht="12.75" customHeight="1" s="127"/>
+    <row r="81" ht="12.75" customHeight="1" s="127"/>
+    <row r="82" ht="12.75" customHeight="1" s="127"/>
+    <row r="83" ht="12.75" customHeight="1" s="127"/>
+    <row r="84" ht="12.75" customHeight="1" s="127"/>
+    <row r="85" ht="12.75" customHeight="1" s="127"/>
+    <row r="86" ht="12.75" customHeight="1" s="127"/>
+    <row r="87" ht="12.75" customHeight="1" s="127"/>
+    <row r="88" ht="12.75" customHeight="1" s="127"/>
+    <row r="89" ht="12.75" customHeight="1" s="127"/>
+    <row r="90" ht="12.75" customHeight="1" s="127"/>
+    <row r="91" ht="12.75" customHeight="1" s="127"/>
+    <row r="92" ht="12.75" customHeight="1" s="127"/>
+    <row r="93" ht="12.75" customHeight="1" s="127"/>
+    <row r="94" ht="12.75" customHeight="1" s="127"/>
+    <row r="95" ht="12.75" customHeight="1" s="127"/>
+    <row r="96" ht="17.25" customHeight="1" s="127"/>
+    <row r="97" ht="17.25" customHeight="1" s="127"/>
+    <row r="98" ht="17.25" customHeight="1" s="127"/>
+    <row r="99" ht="17.25" customHeight="1" s="127"/>
+    <row r="100" ht="17.25" customHeight="1" s="127"/>
+    <row r="101" ht="17.25" customHeight="1" s="127"/>
+    <row r="102" ht="17.25" customHeight="1" s="127"/>
+    <row r="103" ht="17.25" customHeight="1" s="127"/>
+    <row r="104" ht="17.25" customHeight="1" s="127"/>
+    <row r="105" ht="17.25" customHeight="1" s="127"/>
+    <row r="106" ht="17.25" customHeight="1" s="127"/>
+    <row r="107" ht="17.25" customHeight="1" s="127"/>
+    <row r="108" ht="17.25" customHeight="1" s="127"/>
+    <row r="109" ht="17.25" customHeight="1" s="127"/>
+    <row r="110" ht="17.25" customHeight="1" s="127"/>
     <row r="111" ht="17.25" customHeight="1" s="127"/>
     <row r="112" ht="17.25" customHeight="1" s="127"/>
     <row r="113" ht="17.25" customHeight="1" s="127"/>
@@ -15154,7 +13672,7 @@
     <mergeCell ref="R1:R2"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.196527777777778" right="0.196527777777778" top="0.196527777777778" bottom="0.196527777777778" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageMargins left="0.625" right="0.625" top="0.55" bottom="1.69" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" cellComments="atEnd" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
@@ -17445,19 +15963,19 @@
       <c r="AI59" s="126" t="n"/>
       <c r="AJ59" s="126" t="n"/>
     </row>
-    <row r="60" ht="13.5" customHeight="1" s="127">
-      <c r="A60" s="128" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="AN60" s="128" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-    </row>
-    <row r="61" ht="7.599999999999795" customHeight="1" s="127"/>
+    <row r="60" ht="7.599999999999795" customHeight="1" s="127"/>
+    <row r="61" ht="17.25" customHeight="1" s="127">
+      <c r="A61" s="128" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="AN61" s="128" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+    </row>
     <row r="62" ht="17.25" customHeight="1" s="127"/>
     <row r="131" ht="17.25" customHeight="1" s="127"/>
     <row r="132" ht="17.25" customHeight="1" s="127"/>
@@ -20297,19 +18815,19 @@
       <c r="AI61" s="184" t="n"/>
       <c r="AJ61" s="184" t="n"/>
     </row>
-    <row r="62" ht="13.5" customHeight="1" s="127">
-      <c r="A62" s="128" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="AN62" s="128" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="461.55" customHeight="1" s="127"/>
+    <row r="62" ht="461.55" customHeight="1" s="127"/>
+    <row r="63" ht="17.25" customHeight="1" s="127">
+      <c r="A63" s="128" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="AN63" s="128" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+    </row>
     <row r="64" ht="17.25" customHeight="1" s="127"/>
     <row r="133" ht="17.25" customHeight="1" s="127"/>
     <row r="134" ht="17.25" customHeight="1" s="127"/>
@@ -20546,7 +19064,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AN58"/>
+  <dimension ref="A1:AN59"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.13671875" defaultRowHeight="12.75" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="2.56" customWidth="1" style="126" min="1" max="12"/>
@@ -22863,7 +21381,7 @@
         </is>
       </c>
     </row>
-    <row r="57" ht="24" customFormat="1" customHeight="1" s="184">
+    <row r="57" ht="0.5" customFormat="1" customHeight="1" s="184">
       <c r="A57" s="212" t="n"/>
       <c r="B57" s="212" t="n"/>
       <c r="C57" s="212" t="n"/>
@@ -22901,19 +21419,19 @@
       <c r="AI57" s="184" t="n"/>
       <c r="AJ57" s="184" t="n"/>
     </row>
-    <row r="58" ht="13.5" customHeight="1" s="127">
-      <c r="A58" s="128" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="AN58" s="128" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-    </row>
-    <row r="59" ht="17.25" customHeight="1" s="127"/>
+    <row r="58" ht="21.54999999999984" customHeight="1" s="127"/>
+    <row r="59" ht="17.25" customHeight="1" s="127">
+      <c r="A59" s="128" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="AN59" s="128" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+    </row>
     <row r="60" ht="17.25" customHeight="1" s="127"/>
     <row r="129" ht="17.25" customHeight="1" s="127"/>
     <row r="130" ht="17.25" customHeight="1" s="127"/>
@@ -23177,7 +21695,7 @@
     <mergeCell ref="R1:R2"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.196527777777778" right="0.196527777777778" top="0.196527777777778" bottom="0.196527777777778" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageMargins left="0.625" right="0.625" top="0.55" bottom="1.69" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" cellComments="atEnd" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
@@ -23189,7 +21707,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AN55"/>
+  <dimension ref="A1:AN56"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.13671875" defaultRowHeight="12.75" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="2.56" customWidth="1" style="126" min="1" max="12"/>
@@ -24538,7 +23056,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="13.15" customFormat="1" customHeight="1" s="184">
+    <row r="34" ht="0.5" customFormat="1" customHeight="1" s="184">
       <c r="A34" s="212" t="inlineStr">
         <is>
           <t xml:space="preserve"> </t>
@@ -24740,7 +23258,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="13.15" customFormat="1" customHeight="1" s="184">
+    <row r="35" ht="0.5" customFormat="1" customHeight="1" s="184">
       <c r="A35" s="212" t="n"/>
       <c r="B35" s="212" t="n"/>
       <c r="C35" s="212" t="n"/>
@@ -24778,7 +23296,7 @@
       <c r="AI35" s="184" t="n"/>
       <c r="AJ35" s="184" t="n"/>
     </row>
-    <row r="36" ht="13.15" customFormat="1" customHeight="1" s="184">
+    <row r="36" ht="0.5" customFormat="1" customHeight="1" s="184">
       <c r="A36" s="212" t="n"/>
       <c r="B36" s="212" t="n"/>
       <c r="C36" s="212" t="n"/>
@@ -24816,7 +23334,7 @@
       <c r="AI36" s="184" t="n"/>
       <c r="AJ36" s="184" t="n"/>
     </row>
-    <row r="37" ht="13.15" customFormat="1" customHeight="1" s="184">
+    <row r="37" ht="0.5" customFormat="1" customHeight="1" s="184">
       <c r="A37" s="212" t="n"/>
       <c r="B37" s="212" t="n"/>
       <c r="C37" s="212" t="n"/>
@@ -24854,7 +23372,7 @@
       <c r="AI37" s="184" t="n"/>
       <c r="AJ37" s="184" t="n"/>
     </row>
-    <row r="38" ht="13.15" customFormat="1" customHeight="1" s="184">
+    <row r="38" ht="0.5" customFormat="1" customHeight="1" s="184">
       <c r="A38" s="212" t="n"/>
       <c r="B38" s="212" t="n"/>
       <c r="C38" s="212" t="n"/>
@@ -24892,7 +23410,7 @@
       <c r="AI38" s="184" t="n"/>
       <c r="AJ38" s="184" t="n"/>
     </row>
-    <row r="39" ht="13.15" customFormat="1" customHeight="1" s="184">
+    <row r="39" ht="0.5" customFormat="1" customHeight="1" s="184">
       <c r="A39" s="212" t="n"/>
       <c r="B39" s="212" t="n"/>
       <c r="C39" s="212" t="n"/>
@@ -24930,7 +23448,7 @@
       <c r="AI39" s="184" t="n"/>
       <c r="AJ39" s="184" t="n"/>
     </row>
-    <row r="40" ht="13.15" customFormat="1" customHeight="1" s="184">
+    <row r="40" ht="0.5" customFormat="1" customHeight="1" s="184">
       <c r="A40" s="212" t="n"/>
       <c r="B40" s="212" t="n"/>
       <c r="C40" s="212" t="n"/>
@@ -24968,7 +23486,7 @@
       <c r="AI40" s="184" t="n"/>
       <c r="AJ40" s="184" t="n"/>
     </row>
-    <row r="41" ht="13.15" customFormat="1" customHeight="1" s="184">
+    <row r="41" ht="0.5" customFormat="1" customHeight="1" s="184">
       <c r="A41" s="212" t="n"/>
       <c r="B41" s="212" t="n"/>
       <c r="C41" s="212" t="n"/>
@@ -25006,7 +23524,7 @@
       <c r="AI41" s="184" t="n"/>
       <c r="AJ41" s="184" t="n"/>
     </row>
-    <row r="42" ht="13.15" customFormat="1" customHeight="1" s="184">
+    <row r="42" ht="0.5" customFormat="1" customHeight="1" s="184">
       <c r="A42" s="212" t="n"/>
       <c r="B42" s="212" t="n"/>
       <c r="C42" s="212" t="n"/>
@@ -25044,7 +23562,7 @@
       <c r="AI42" s="184" t="n"/>
       <c r="AJ42" s="184" t="n"/>
     </row>
-    <row r="43" ht="13.15" customFormat="1" customHeight="1" s="184">
+    <row r="43" ht="0.5" customFormat="1" customHeight="1" s="184">
       <c r="A43" s="212" t="n"/>
       <c r="B43" s="212" t="n"/>
       <c r="C43" s="212" t="n"/>
@@ -25082,7 +23600,7 @@
       <c r="AI43" s="184" t="n"/>
       <c r="AJ43" s="184" t="n"/>
     </row>
-    <row r="44" ht="13.15" customFormat="1" customHeight="1" s="184">
+    <row r="44" ht="0.5" customFormat="1" customHeight="1" s="184">
       <c r="A44" s="212" t="n"/>
       <c r="B44" s="212" t="n"/>
       <c r="C44" s="212" t="n"/>
@@ -25120,7 +23638,7 @@
       <c r="AI44" s="184" t="n"/>
       <c r="AJ44" s="184" t="n"/>
     </row>
-    <row r="45" ht="13.15" customFormat="1" customHeight="1" s="184">
+    <row r="45" ht="0.5" customFormat="1" customHeight="1" s="184">
       <c r="A45" s="212" t="n"/>
       <c r="B45" s="212" t="n"/>
       <c r="C45" s="212" t="n"/>
@@ -25158,7 +23676,7 @@
       <c r="AI45" s="184" t="n"/>
       <c r="AJ45" s="184" t="n"/>
     </row>
-    <row r="46" ht="13.15" customFormat="1" customHeight="1" s="184">
+    <row r="46" ht="0.5" customFormat="1" customHeight="1" s="184">
       <c r="A46" s="212" t="n"/>
       <c r="B46" s="212" t="n"/>
       <c r="C46" s="212" t="n"/>
@@ -25196,7 +23714,7 @@
       <c r="AI46" s="184" t="n"/>
       <c r="AJ46" s="184" t="n"/>
     </row>
-    <row r="47" ht="13.15" customFormat="1" customHeight="1" s="184">
+    <row r="47" ht="0.5" customFormat="1" customHeight="1" s="184">
       <c r="A47" s="212" t="n"/>
       <c r="B47" s="212" t="n"/>
       <c r="C47" s="212" t="n"/>
@@ -25234,7 +23752,7 @@
       <c r="AI47" s="184" t="n"/>
       <c r="AJ47" s="184" t="n"/>
     </row>
-    <row r="48" ht="13.15" customFormat="1" customHeight="1" s="184">
+    <row r="48" ht="0.5" customFormat="1" customHeight="1" s="184">
       <c r="A48" s="212" t="n"/>
       <c r="B48" s="212" t="n"/>
       <c r="C48" s="212" t="n"/>
@@ -25272,7 +23790,7 @@
       <c r="AI48" s="184" t="n"/>
       <c r="AJ48" s="184" t="n"/>
     </row>
-    <row r="49" ht="13.15" customFormat="1" customHeight="1" s="184">
+    <row r="49" ht="0.5" customFormat="1" customHeight="1" s="184">
       <c r="A49" s="212" t="n"/>
       <c r="B49" s="212" t="n"/>
       <c r="C49" s="212" t="n"/>
@@ -25310,7 +23828,7 @@
       <c r="AI49" s="184" t="n"/>
       <c r="AJ49" s="184" t="n"/>
     </row>
-    <row r="50" ht="13.15" customFormat="1" customHeight="1" s="184">
+    <row r="50" ht="0.5" customFormat="1" customHeight="1" s="184">
       <c r="A50" s="212" t="n"/>
       <c r="B50" s="212" t="n"/>
       <c r="C50" s="212" t="n"/>
@@ -25348,7 +23866,7 @@
       <c r="AI50" s="184" t="n"/>
       <c r="AJ50" s="184" t="n"/>
     </row>
-    <row r="51" ht="13.15" customFormat="1" customHeight="1" s="184">
+    <row r="51" ht="0.5" customFormat="1" customHeight="1" s="184">
       <c r="A51" s="212" t="n"/>
       <c r="B51" s="212" t="n"/>
       <c r="C51" s="212" t="n"/>
@@ -25386,7 +23904,7 @@
       <c r="AI51" s="184" t="n"/>
       <c r="AJ51" s="184" t="n"/>
     </row>
-    <row r="52" ht="13.15" customFormat="1" customHeight="1" s="184">
+    <row r="52" ht="0.5" customFormat="1" customHeight="1" s="184">
       <c r="A52" s="212" t="n"/>
       <c r="B52" s="212" t="n"/>
       <c r="C52" s="212" t="n"/>
@@ -25424,7 +23942,7 @@
       <c r="AI52" s="184" t="n"/>
       <c r="AJ52" s="184" t="n"/>
     </row>
-    <row r="53" ht="13.15" customFormat="1" customHeight="1" s="184">
+    <row r="53" ht="0.5" customFormat="1" customHeight="1" s="184">
       <c r="A53" s="212" t="n"/>
       <c r="B53" s="212" t="n"/>
       <c r="C53" s="212" t="n"/>
@@ -25462,7 +23980,7 @@
       <c r="AI53" s="184" t="n"/>
       <c r="AJ53" s="184" t="n"/>
     </row>
-    <row r="54" ht="13.5" customFormat="1" customHeight="1" s="184">
+    <row r="54" ht="0.5" customFormat="1" customHeight="1" s="184">
       <c r="A54" s="212" t="n"/>
       <c r="B54" s="212" t="n"/>
       <c r="C54" s="212" t="n"/>
@@ -25500,19 +24018,19 @@
       <c r="AI54" s="184" t="n"/>
       <c r="AJ54" s="184" t="n"/>
     </row>
-    <row r="55" ht="13.5" customHeight="1" s="127">
-      <c r="A55" s="128" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="AN55" s="128" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="17.25" customHeight="1" s="127"/>
+    <row r="55" ht="263.85" customHeight="1" s="127"/>
+    <row r="56" ht="17.25" customHeight="1" s="127">
+      <c r="A56" s="128" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="AN56" s="128" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+    </row>
     <row r="57" ht="17.25" customHeight="1" s="127"/>
     <row r="126" ht="17.25" customHeight="1" s="127"/>
     <row r="127" ht="17.25" customHeight="1" s="127"/>
@@ -25748,7 +24266,7 @@
     <mergeCell ref="R1:R2"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.196527777777778" right="0.196527777777778" top="0.196527777777778" bottom="0.196527777777778" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageMargins left="0.625" right="0.625" top="0.55" bottom="1.69" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" cellComments="atEnd" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
@@ -25760,7 +24278,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AN67"/>
+  <dimension ref="A1:AN68"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.13671875" defaultRowHeight="12.75" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="2.56" customWidth="1" style="126" min="1" max="12"/>
@@ -28037,7 +26555,7 @@
       <c r="AM64" s="130" t="n"/>
       <c r="AN64" s="130" t="n"/>
     </row>
-    <row r="65" ht="6.75" customHeight="1" s="127">
+    <row r="65" ht="0.5" customHeight="1" s="127">
       <c r="S65" s="126" t="n"/>
       <c r="T65" s="126" t="n"/>
       <c r="U65" s="126" t="n"/>
@@ -28057,7 +26575,7 @@
       <c r="AI65" s="126" t="n"/>
       <c r="AJ65" s="126" t="n"/>
     </row>
-    <row r="66" ht="4.5" customHeight="1" s="127">
+    <row r="66" ht="0.5" customHeight="1" s="127">
       <c r="L66" s="126" t="n"/>
       <c r="M66" s="126" t="n"/>
       <c r="N66" s="126" t="n"/>
@@ -28084,19 +26602,19 @@
       <c r="AI66" s="126" t="n"/>
       <c r="AJ66" s="126" t="n"/>
     </row>
-    <row r="67" ht="13.5" customHeight="1" s="127">
-      <c r="A67" s="128" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="AN67" s="128" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-    </row>
-    <row r="68" ht="17.25" customHeight="1" s="127"/>
+    <row r="67" ht="8.599999999999682" customHeight="1" s="127"/>
+    <row r="68" ht="17.25" customHeight="1" s="127">
+      <c r="A68" s="128" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="AN68" s="128" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+    </row>
     <row r="69" ht="17.25" customHeight="1" s="127"/>
     <row r="138" ht="17.25" customHeight="1" s="127"/>
     <row r="139" ht="17.25" customHeight="1" s="127"/>
@@ -28369,7 +26887,7 @@
     <mergeCell ref="AA32:AB32"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.196527777777778" right="0.196527777777778" top="0.196527777777778" bottom="0.196527777777778" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageMargins left="0.625" right="0.625" top="0.55" bottom="1.69" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" cellComments="atEnd" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
@@ -28381,7 +26899,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AN56"/>
+  <dimension ref="A1:AN57"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.13671875" defaultRowHeight="12.75" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="2.56" customWidth="1" style="126" min="1" max="12"/>
@@ -29671,7 +28189,7 @@
       <c r="AM28" s="130" t="n"/>
       <c r="AN28" s="130" t="n"/>
     </row>
-    <row r="29" ht="11.45" customHeight="1" s="127">
+    <row r="29" ht="0.5" customHeight="1" s="127">
       <c r="AA29" s="126" t="n"/>
       <c r="AB29" s="126" t="n"/>
       <c r="AC29" s="126" t="n"/>
@@ -29683,7 +28201,7 @@
       <c r="AI29" s="126" t="n"/>
       <c r="AJ29" s="126" t="n"/>
     </row>
-    <row r="30" ht="12.75" customHeight="1" s="127">
+    <row r="30" ht="0.5" customHeight="1" s="127">
       <c r="L30" s="126" t="n"/>
       <c r="M30" s="126" t="n"/>
       <c r="N30" s="126" t="n"/>
@@ -29710,7 +28228,7 @@
       <c r="AI30" s="126" t="n"/>
       <c r="AJ30" s="126" t="n"/>
     </row>
-    <row r="31" ht="12.75" customHeight="1" s="127">
+    <row r="31" ht="0.5" customHeight="1" s="127">
       <c r="L31" s="126" t="n"/>
       <c r="M31" s="126" t="n"/>
       <c r="N31" s="126" t="n"/>
@@ -29737,7 +28255,7 @@
       <c r="AI31" s="126" t="n"/>
       <c r="AJ31" s="126" t="n"/>
     </row>
-    <row r="32" ht="12.75" customHeight="1" s="127">
+    <row r="32" ht="0.5" customHeight="1" s="127">
       <c r="L32" s="126" t="n"/>
       <c r="M32" s="126" t="n"/>
       <c r="N32" s="126" t="n"/>
@@ -29764,7 +28282,7 @@
       <c r="AI32" s="126" t="n"/>
       <c r="AJ32" s="126" t="n"/>
     </row>
-    <row r="33" ht="12.75" customHeight="1" s="127">
+    <row r="33" ht="0.5" customHeight="1" s="127">
       <c r="L33" s="126" t="n"/>
       <c r="M33" s="126" t="n"/>
       <c r="N33" s="126" t="n"/>
@@ -29791,7 +28309,7 @@
       <c r="AI33" s="126" t="n"/>
       <c r="AJ33" s="126" t="n"/>
     </row>
-    <row r="34" ht="12.75" customHeight="1" s="127">
+    <row r="34" ht="0.5" customHeight="1" s="127">
       <c r="L34" s="126" t="n"/>
       <c r="M34" s="126" t="n"/>
       <c r="N34" s="126" t="n"/>
@@ -29818,7 +28336,7 @@
       <c r="AI34" s="126" t="n"/>
       <c r="AJ34" s="126" t="n"/>
     </row>
-    <row r="35" ht="12.75" customHeight="1" s="127">
+    <row r="35" ht="0.5" customHeight="1" s="127">
       <c r="L35" s="126" t="n"/>
       <c r="M35" s="126" t="n"/>
       <c r="N35" s="126" t="n"/>
@@ -29845,7 +28363,7 @@
       <c r="AI35" s="126" t="n"/>
       <c r="AJ35" s="126" t="n"/>
     </row>
-    <row r="36" ht="12.75" customHeight="1" s="127">
+    <row r="36" ht="0.5" customHeight="1" s="127">
       <c r="L36" s="126" t="n"/>
       <c r="M36" s="126" t="n"/>
       <c r="N36" s="126" t="n"/>
@@ -29872,7 +28390,7 @@
       <c r="AI36" s="126" t="n"/>
       <c r="AJ36" s="126" t="n"/>
     </row>
-    <row r="37" ht="12.75" customHeight="1" s="127">
+    <row r="37" ht="0.5" customHeight="1" s="127">
       <c r="L37" s="126" t="n"/>
       <c r="M37" s="126" t="n"/>
       <c r="N37" s="126" t="n"/>
@@ -29899,7 +28417,7 @@
       <c r="AI37" s="126" t="n"/>
       <c r="AJ37" s="126" t="n"/>
     </row>
-    <row r="38" ht="12.75" customHeight="1" s="127">
+    <row r="38" ht="0.5" customHeight="1" s="127">
       <c r="L38" s="126" t="n"/>
       <c r="M38" s="126" t="n"/>
       <c r="N38" s="126" t="n"/>
@@ -29926,7 +28444,7 @@
       <c r="AI38" s="126" t="n"/>
       <c r="AJ38" s="126" t="n"/>
     </row>
-    <row r="39" ht="12.75" customHeight="1" s="127">
+    <row r="39" ht="0.5" customHeight="1" s="127">
       <c r="L39" s="126" t="n"/>
       <c r="M39" s="126" t="n"/>
       <c r="N39" s="126" t="n"/>
@@ -29953,7 +28471,7 @@
       <c r="AI39" s="126" t="n"/>
       <c r="AJ39" s="126" t="n"/>
     </row>
-    <row r="40" ht="12.75" customHeight="1" s="127">
+    <row r="40" ht="0.5" customHeight="1" s="127">
       <c r="L40" s="126" t="n"/>
       <c r="M40" s="126" t="n"/>
       <c r="N40" s="126" t="n"/>
@@ -29980,7 +28498,7 @@
       <c r="AI40" s="126" t="n"/>
       <c r="AJ40" s="126" t="n"/>
     </row>
-    <row r="41" ht="12.75" customHeight="1" s="127">
+    <row r="41" ht="0.5" customHeight="1" s="127">
       <c r="L41" s="126" t="n"/>
       <c r="M41" s="126" t="n"/>
       <c r="N41" s="126" t="n"/>
@@ -30007,7 +28525,7 @@
       <c r="AI41" s="126" t="n"/>
       <c r="AJ41" s="126" t="n"/>
     </row>
-    <row r="42" ht="12.75" customHeight="1" s="127">
+    <row r="42" ht="0.5" customHeight="1" s="127">
       <c r="L42" s="126" t="n"/>
       <c r="M42" s="126" t="n"/>
       <c r="N42" s="126" t="n"/>
@@ -30034,7 +28552,7 @@
       <c r="AI42" s="126" t="n"/>
       <c r="AJ42" s="126" t="n"/>
     </row>
-    <row r="43" ht="12.75" customHeight="1" s="127">
+    <row r="43" ht="0.5" customHeight="1" s="127">
       <c r="L43" s="126" t="n"/>
       <c r="M43" s="126" t="n"/>
       <c r="N43" s="126" t="n"/>
@@ -30061,7 +28579,7 @@
       <c r="AI43" s="126" t="n"/>
       <c r="AJ43" s="126" t="n"/>
     </row>
-    <row r="44" ht="12.75" customHeight="1" s="127">
+    <row r="44" ht="0.5" customHeight="1" s="127">
       <c r="L44" s="126" t="n"/>
       <c r="M44" s="126" t="n"/>
       <c r="N44" s="126" t="n"/>
@@ -30088,7 +28606,7 @@
       <c r="AI44" s="126" t="n"/>
       <c r="AJ44" s="126" t="n"/>
     </row>
-    <row r="45" ht="12.75" customHeight="1" s="127">
+    <row r="45" ht="0.5" customHeight="1" s="127">
       <c r="L45" s="126" t="n"/>
       <c r="M45" s="126" t="n"/>
       <c r="N45" s="126" t="n"/>
@@ -30115,7 +28633,7 @@
       <c r="AI45" s="126" t="n"/>
       <c r="AJ45" s="126" t="n"/>
     </row>
-    <row r="46" ht="12.75" customHeight="1" s="127">
+    <row r="46" ht="0.5" customHeight="1" s="127">
       <c r="L46" s="126" t="n"/>
       <c r="M46" s="126" t="n"/>
       <c r="N46" s="126" t="n"/>
@@ -30142,7 +28660,7 @@
       <c r="AI46" s="126" t="n"/>
       <c r="AJ46" s="126" t="n"/>
     </row>
-    <row r="47" ht="12.75" customHeight="1" s="127">
+    <row r="47" ht="0.5" customHeight="1" s="127">
       <c r="L47" s="126" t="n"/>
       <c r="M47" s="126" t="n"/>
       <c r="N47" s="126" t="n"/>
@@ -30169,7 +28687,7 @@
       <c r="AI47" s="126" t="n"/>
       <c r="AJ47" s="126" t="n"/>
     </row>
-    <row r="48" ht="12.75" customHeight="1" s="127">
+    <row r="48" ht="0.5" customHeight="1" s="127">
       <c r="L48" s="126" t="n"/>
       <c r="M48" s="126" t="n"/>
       <c r="N48" s="126" t="n"/>
@@ -30196,7 +28714,7 @@
       <c r="AI48" s="126" t="n"/>
       <c r="AJ48" s="126" t="n"/>
     </row>
-    <row r="49" ht="12.75" customHeight="1" s="127">
+    <row r="49" ht="0.5" customHeight="1" s="127">
       <c r="L49" s="126" t="n"/>
       <c r="M49" s="126" t="n"/>
       <c r="N49" s="126" t="n"/>
@@ -30223,7 +28741,7 @@
       <c r="AI49" s="126" t="n"/>
       <c r="AJ49" s="126" t="n"/>
     </row>
-    <row r="50" ht="12.75" customHeight="1" s="127">
+    <row r="50" ht="0.5" customHeight="1" s="127">
       <c r="L50" s="126" t="n"/>
       <c r="M50" s="126" t="n"/>
       <c r="N50" s="126" t="n"/>
@@ -30250,7 +28768,7 @@
       <c r="AI50" s="126" t="n"/>
       <c r="AJ50" s="126" t="n"/>
     </row>
-    <row r="51" ht="12.75" customHeight="1" s="127">
+    <row r="51" ht="0.5" customHeight="1" s="127">
       <c r="L51" s="126" t="n"/>
       <c r="M51" s="126" t="n"/>
       <c r="N51" s="126" t="n"/>
@@ -30277,7 +28795,7 @@
       <c r="AI51" s="126" t="n"/>
       <c r="AJ51" s="126" t="n"/>
     </row>
-    <row r="52" ht="12.75" customHeight="1" s="127">
+    <row r="52" ht="0.5" customHeight="1" s="127">
       <c r="L52" s="126" t="n"/>
       <c r="M52" s="126" t="n"/>
       <c r="N52" s="126" t="n"/>
@@ -30304,7 +28822,7 @@
       <c r="AI52" s="126" t="n"/>
       <c r="AJ52" s="126" t="n"/>
     </row>
-    <row r="53" ht="12.75" customHeight="1" s="127">
+    <row r="53" ht="0.5" customHeight="1" s="127">
       <c r="L53" s="126" t="n"/>
       <c r="M53" s="126" t="n"/>
       <c r="N53" s="126" t="n"/>
@@ -30331,7 +28849,7 @@
       <c r="AI53" s="126" t="n"/>
       <c r="AJ53" s="126" t="n"/>
     </row>
-    <row r="54" ht="12.75" customHeight="1" s="127">
+    <row r="54" ht="0.5" customHeight="1" s="127">
       <c r="L54" s="126" t="n"/>
       <c r="M54" s="126" t="n"/>
       <c r="N54" s="126" t="n"/>
@@ -30358,7 +28876,7 @@
       <c r="AI54" s="126" t="n"/>
       <c r="AJ54" s="126" t="n"/>
     </row>
-    <row r="55" ht="40.5" customHeight="1" s="127">
+    <row r="55" ht="0.5" customHeight="1" s="127">
       <c r="L55" s="126" t="n"/>
       <c r="M55" s="126" t="n"/>
       <c r="N55" s="126" t="n"/>
@@ -30385,19 +28903,19 @@
       <c r="AI55" s="126" t="n"/>
       <c r="AJ55" s="126" t="n"/>
     </row>
-    <row r="56" ht="13.5" customHeight="1" s="127">
-      <c r="A56" s="128" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="AN56" s="128" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="17.25" customHeight="1" s="127"/>
+    <row r="56" ht="351.3" customHeight="1" s="127"/>
+    <row r="57" ht="17.25" customHeight="1" s="127">
+      <c r="A57" s="128" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="AN57" s="128" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+    </row>
     <row r="58" ht="17.25" customHeight="1" s="127"/>
     <row r="127" ht="17.25" customHeight="1" s="127"/>
     <row r="128" ht="17.25" customHeight="1" s="127"/>
@@ -30627,7 +29145,7 @@
     <mergeCell ref="R1:R2"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.196527777777778" right="0.196527777777778" top="0.196527777777778" bottom="0.196527777777778" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageMargins left="0.625" right="0.625" top="0.55" bottom="1.69" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" cellComments="atEnd" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(pr30): preserve marker row height after insert_rows
Bug в v14: после ws.insert_rows() openpyxl автоматически назначал
дефолтную высоту 17.25pt для смещённой row с меткой (раньше была 13.5pt).
Это делало метки вертикально вытянутыми — в PDF они становились
прямоугольными 25x16px вместо квадратных 28x28px (как у эталона Тензора).

Фикс v15:
- Запоминаем original_marker_height ДО insert_rows
- После insert восстанавливаем height на новой позиции метки (last_marker+1)

Локальный тест: метки 20x20px ratio 1.00 (идеально квадратные).
На production scale_v чуть ниже, но соотношение сохранится.
</commit_message>
<xml_diff>
--- a/modules/usn_declaration/data/declaration_template_2024.xlsx
+++ b/modules/usn_declaration/data/declaration_template_2024.xlsx
@@ -1688,7 +1688,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AN62"/>
+  <dimension ref="A1:AN63"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.13671875" defaultRowHeight="12.75" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="2.56" customWidth="1" style="126" min="1" max="13"/>
@@ -4230,191 +4230,191 @@
       </c>
     </row>
     <row r="61" ht="0.5" customHeight="1" s="127"/>
-    <row r="62" ht="13.5" customHeight="1" s="127">
-      <c r="A62" s="128" t="n"/>
-      <c r="B62" s="126" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="C62" s="126" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="D62" s="126" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="E62" s="126" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="F62" s="126" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="G62" s="126" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="H62" s="126" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="I62" s="126" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="J62" s="126" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="K62" s="126" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="L62" s="126" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="M62" s="126" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="N62" s="126" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="O62" s="126" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="P62" s="126" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="Q62" s="126" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="R62" s="126" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="S62" s="126" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="T62" s="126" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="U62" s="126" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="V62" s="126" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="W62" s="126" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="X62" s="126" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="Y62" s="126" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="Z62" s="126" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="AA62" s="126" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="AB62" s="126" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="AC62" s="126" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="AD62" s="126" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="AE62" s="126" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="AF62" s="126" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="AG62" s="126" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="AH62" s="126" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="AI62" s="126" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="AJ62" s="126" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="AK62" s="126" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="AN62" s="128" t="n"/>
-    </row>
-    <row r="63" ht="17.25" customHeight="1" s="127"/>
+    <row r="62" ht="103.4" customHeight="1" s="127"/>
+    <row r="63" ht="13.5" customHeight="1" s="127">
+      <c r="A63" s="128" t="n"/>
+      <c r="B63" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="C63" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="D63" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="E63" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="F63" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="G63" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="H63" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="I63" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="J63" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="K63" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="L63" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="M63" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="N63" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="O63" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="P63" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="Q63" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="R63" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="S63" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="T63" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="U63" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="V63" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="W63" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="X63" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="Y63" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="Z63" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="AA63" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="AB63" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="AC63" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="AD63" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="AE63" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="AF63" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="AG63" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="AH63" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="AI63" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="AJ63" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="AK63" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="AN63" s="128" t="n"/>
+    </row>
     <row r="64" ht="17.25" customHeight="1" s="127"/>
     <row r="65" ht="17.25" customHeight="1" s="127"/>
     <row r="516" ht="17.25" customHeight="1" s="127"/>
@@ -6649,8 +6649,8 @@
       <c r="AI63" s="126" t="n"/>
       <c r="AJ63" s="126" t="n"/>
     </row>
-    <row r="64" ht="7.300000000000409" customHeight="1" s="127"/>
-    <row r="65" ht="17.25" customHeight="1" s="127">
+    <row r="64" ht="110.3000000000004" customHeight="1" s="127"/>
+    <row r="65" ht="13.5" customHeight="1" s="127">
       <c r="A65" s="128" t="inlineStr">
         <is>
           <t xml:space="preserve"> </t>
@@ -6889,7 +6889,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AN66"/>
+  <dimension ref="A1:AN67"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.13671875" defaultRowHeight="12.75" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="2.56" customWidth="1" style="126" min="1" max="12"/>
@@ -9930,19 +9930,19 @@
       <c r="AI65" s="126" t="n"/>
       <c r="AJ65" s="126" t="n"/>
     </row>
-    <row r="66" ht="13.5" customHeight="1" s="127">
-      <c r="A66" s="128" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="AN66" s="128" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-    </row>
-    <row r="67" ht="17.25" customHeight="1" s="127"/>
+    <row r="66" ht="102.5" customHeight="1" s="127"/>
+    <row r="67" ht="13.5" customHeight="1" s="127">
+      <c r="A67" s="128" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="AN67" s="128" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+    </row>
     <row r="68" ht="17.25" customHeight="1" s="127"/>
     <row r="137" ht="17.25" customHeight="1" s="127"/>
     <row r="138" ht="17.25" customHeight="1" s="127"/>
@@ -10205,7 +10205,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AN53"/>
+  <dimension ref="A1:AN54"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.13671875" defaultRowHeight="12.75" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="2.56" customWidth="1" style="126" min="1" max="12"/>
@@ -11634,19 +11634,19 @@
       <c r="AN51" s="134" t="n"/>
     </row>
     <row r="52" ht="0.5" customHeight="1" s="127"/>
-    <row r="53" ht="13.5" customHeight="1" s="127">
-      <c r="A53" s="128" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="AN53" s="128" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="12.75" customHeight="1" s="127"/>
+    <row r="53" ht="102.7500000000001" customHeight="1" s="127"/>
+    <row r="54" ht="13.5" customHeight="1" s="127">
+      <c r="A54" s="128" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="AN54" s="128" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+    </row>
     <row r="55" ht="12.75" customHeight="1" s="127"/>
     <row r="56" ht="12.75" customHeight="1" s="127"/>
     <row r="57" ht="12.75" customHeight="1" s="127"/>
@@ -11954,7 +11954,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AN53"/>
+  <dimension ref="A1:AN54"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.13671875" defaultRowHeight="12.75" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="2.56" customWidth="1" style="126" min="1" max="12"/>
@@ -13375,19 +13375,19 @@
       <c r="AN51" s="134" t="n"/>
     </row>
     <row r="52" ht="0.5" customHeight="1" s="127"/>
-    <row r="53" ht="13.5" customHeight="1" s="127">
-      <c r="A53" s="128" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="AN53" s="128" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="12.75" customHeight="1" s="127"/>
+    <row r="53" ht="101.6500000000001" customHeight="1" s="127"/>
+    <row r="54" ht="13.5" customHeight="1" s="127">
+      <c r="A54" s="128" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="AN54" s="128" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+    </row>
     <row r="55" ht="12.75" customHeight="1" s="127"/>
     <row r="56" ht="12.75" customHeight="1" s="127"/>
     <row r="57" ht="12.75" customHeight="1" s="127"/>
@@ -15963,8 +15963,8 @@
       <c r="AI59" s="126" t="n"/>
       <c r="AJ59" s="126" t="n"/>
     </row>
-    <row r="60" ht="7.599999999999795" customHeight="1" s="127"/>
-    <row r="61" ht="17.25" customHeight="1" s="127">
+    <row r="60" ht="110.5999999999998" customHeight="1" s="127"/>
+    <row r="61" ht="13.5" customHeight="1" s="127">
       <c r="A61" s="128" t="inlineStr">
         <is>
           <t xml:space="preserve"> </t>
@@ -18815,8 +18815,8 @@
       <c r="AI61" s="184" t="n"/>
       <c r="AJ61" s="184" t="n"/>
     </row>
-    <row r="62" ht="461.55" customHeight="1" s="127"/>
-    <row r="63" ht="17.25" customHeight="1" s="127">
+    <row r="62" ht="564.55" customHeight="1" s="127"/>
+    <row r="63" ht="13.5" customHeight="1" s="127">
       <c r="A63" s="128" t="inlineStr">
         <is>
           <t xml:space="preserve"> </t>
@@ -21419,8 +21419,8 @@
       <c r="AI57" s="184" t="n"/>
       <c r="AJ57" s="184" t="n"/>
     </row>
-    <row r="58" ht="21.54999999999984" customHeight="1" s="127"/>
-    <row r="59" ht="17.25" customHeight="1" s="127">
+    <row r="58" ht="124.5499999999998" customHeight="1" s="127"/>
+    <row r="59" ht="13.5" customHeight="1" s="127">
       <c r="A59" s="128" t="inlineStr">
         <is>
           <t xml:space="preserve"> </t>
@@ -24018,8 +24018,8 @@
       <c r="AI54" s="184" t="n"/>
       <c r="AJ54" s="184" t="n"/>
     </row>
-    <row r="55" ht="263.85" customHeight="1" s="127"/>
-    <row r="56" ht="17.25" customHeight="1" s="127">
+    <row r="55" ht="366.85" customHeight="1" s="127"/>
+    <row r="56" ht="13.5" customHeight="1" s="127">
       <c r="A56" s="128" t="inlineStr">
         <is>
           <t xml:space="preserve"> </t>
@@ -26602,8 +26602,8 @@
       <c r="AI66" s="126" t="n"/>
       <c r="AJ66" s="126" t="n"/>
     </row>
-    <row r="67" ht="8.599999999999682" customHeight="1" s="127"/>
-    <row r="68" ht="17.25" customHeight="1" s="127">
+    <row r="67" ht="111.5999999999997" customHeight="1" s="127"/>
+    <row r="68" ht="13.5" customHeight="1" s="127">
       <c r="A68" s="128" t="inlineStr">
         <is>
           <t xml:space="preserve"> </t>
@@ -28903,8 +28903,8 @@
       <c r="AI55" s="126" t="n"/>
       <c r="AJ55" s="126" t="n"/>
     </row>
-    <row r="56" ht="351.3" customHeight="1" s="127"/>
-    <row r="57" ht="17.25" customHeight="1" s="127">
+    <row r="56" ht="454.3" customHeight="1" s="127"/>
+    <row r="57" ht="13.5" customHeight="1" s="127">
       <c r="A57" s="128" t="inlineStr">
         <is>
           <t xml:space="preserve"> </t>

</xml_diff>